<commit_message>
Merge xlsx trade book generation into build_trade_book.py
One script, one cron job now writes both trade_book.csv and trade_book.xlsx
from the same in-memory rows (was two separate scripts on two cron jobs).
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,12 +63,8 @@
     <font>
       <color rgb="00006100"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="007F6000"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -108,11 +104,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -270,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -333,12 +324,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="9" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="9" fillId="9" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1025,31 +1010,31 @@
       <c r="B5" s="4" t="n"/>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>26 / 1</t>
+          <t>27 / 0</t>
         </is>
       </c>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="10" t="inlineStr">
         <is>
-          <t>50%  (13W-13L)</t>
+          <t>52%  (14W-13L)</t>
         </is>
       </c>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>₹4,151</t>
+          <t>₹6,961</t>
         </is>
       </c>
       <c r="H5" s="6" t="n"/>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>₹1,375</t>
+          <t>₹1,476</t>
         </is>
       </c>
       <c r="J5" s="8" t="n"/>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>₹2,776</t>
+          <t>₹5,484</t>
         </is>
       </c>
       <c r="L5" s="6" t="n"/>
@@ -1264,16 +1249,16 @@
         <v>1</v>
       </c>
       <c r="C17" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D17" s="13" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="14" t="n">
-        <v>0</v>
+        <v>2810.2</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>0</v>
+        <v>2708.76</v>
       </c>
     </row>
   </sheetData>
@@ -3240,7 +3225,7 @@
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-07-30   ·   1 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-07-30   ·   1 trade(s), 1 closed   ·   Gross PnL: ₹2,810.20   ·   Net PnL: ₹2,708.76</t>
         </is>
       </c>
       <c r="B57" s="17" t="n"/>
@@ -3318,34 +3303,50 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="38" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B59" s="39" t="inlineStr">
+      <c r="A59" s="28" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B59" s="29" t="inlineStr">
         <is>
           <t>63MOONS</t>
         </is>
       </c>
-      <c r="C59" s="39" t="inlineStr">
+      <c r="C59" s="29" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="D59" s="39" t="n"/>
-      <c r="E59" s="40" t="n">
+      <c r="D59" s="29" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="E59" s="30" t="n">
         <v>44</v>
       </c>
-      <c r="F59" s="41" t="n">
+      <c r="F59" s="31" t="n">
         <v>845.4318</v>
       </c>
-      <c r="G59" s="41" t="n"/>
-      <c r="H59" s="41" t="n"/>
-      <c r="I59" s="42" t="n"/>
-      <c r="J59" s="41" t="n"/>
-      <c r="K59" s="41" t="n"/>
-      <c r="L59" s="43" t="n"/>
+      <c r="G59" s="31" t="n">
+        <v>909.3</v>
+      </c>
+      <c r="H59" s="31" t="n">
+        <v>2810.2</v>
+      </c>
+      <c r="I59" s="32" t="n">
+        <v>7.5545</v>
+      </c>
+      <c r="J59" s="31" t="n">
+        <v>101.44</v>
+      </c>
+      <c r="K59" s="31" t="n">
+        <v>2708.76</v>
+      </c>
+      <c r="L59" s="33" t="n">
+        <v>7.2818</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="34" t="inlineStr">
@@ -3360,12 +3361,12 @@
       <c r="F60" s="35" t="n"/>
       <c r="G60" s="35" t="n"/>
       <c r="H60" s="36" t="n">
-        <v>0</v>
+        <v>2810.2</v>
       </c>
       <c r="I60" s="35" t="n"/>
       <c r="J60" s="35" t="n"/>
       <c r="K60" s="36" t="n">
-        <v>0</v>
+        <v>2708.76</v>
       </c>
       <c r="L60" s="37" t="n"/>
     </row>

</xml_diff>

<commit_message>
Drop Dashboard sheet from trade book xlsx, keep Trade Book only
Also removed the now-dead KPI-tile/chart helpers and their unused
openpyxl.chart imports. Gridlines were already off on the Trade Book
sheet (ws.sheet_view.showGridLines = False), confirmed still in effect.
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Trade Book" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Trade Book" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,31 +20,13 @@
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="22"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="20"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -58,13 +39,16 @@
       <sz val="13"/>
     </font>
     <font>
+      <b val="1"/>
+    </font>
+    <font>
       <color rgb="009C0006"/>
     </font>
     <font>
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,22 +57,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00305496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002E7D32"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007F7F7F"/>
       </patternFill>
     </fill>
     <fill>
@@ -107,27 +76,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="12">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="001F3864"/>
-      </left>
-      <right style="medium">
-        <color rgb="001F3864"/>
-      </right>
-      <top style="medium">
-        <color rgb="001F3864"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="001F3864"/>
-      </bottom>
     </border>
     <border>
       <left style="thin">
@@ -261,69 +216,41 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="7" fillId="7" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="8" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="8" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -398,231 +325,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Daily Net PnL</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'📊 Dashboard'!F9</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <dPt>
-            <idx val="0"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="C62828"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="1"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="2"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="C62828"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="3"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="4"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="C62828"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="5"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="6"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="7"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <cat>
-            <numRef>
-              <f>'📊 Dashboard'!$A$10:$A$17</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'📊 Dashboard'!$F$10:$F$17</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Entry Date</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>₹ Net PnL</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>7</col>
-      <colOff>0</colOff>
-      <row>8</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="9360000" cy="3960000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -914,380 +616,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="3" customWidth="1" min="2" max="2"/>
-    <col width="3" customWidth="1" min="3" max="3"/>
-    <col width="3" customWidth="1" min="4" max="4"/>
-    <col width="3" customWidth="1" min="5" max="5"/>
-    <col width="3" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="3" customWidth="1" min="8" max="8"/>
-    <col width="3" customWidth="1" min="9" max="9"/>
-    <col width="3" customWidth="1" min="10" max="10"/>
-    <col width="3" customWidth="1" min="11" max="11"/>
-    <col width="3" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>📊  TRADING DASHBOARD</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL TRADES</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>CLOSED / OPEN</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>WIN RATE 🎯</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>GROSS PnL</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL CHARGES</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="n"/>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>NET PnL 💰</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="9" t="inlineStr">
-        <is>
-          <t>27 / 0</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>52%  (14W-13L)</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>₹6,961</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>₹1,476</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="n"/>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>₹5,484</t>
-        </is>
-      </c>
-      <c r="L5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="8" customHeight="1">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Entry Date</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Trades</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Wins</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Losses</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Gross PnL</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>Net PnL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-21</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>-10.06</v>
-      </c>
-      <c r="F10" s="14" t="n">
-        <v>-99</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="C11" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>159.08</v>
-      </c>
-      <c r="F11" s="14" t="n">
-        <v>118.22</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-23</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>-137.84</v>
-      </c>
-      <c r="F12" s="14" t="n">
-        <v>-191.96</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-24</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="14" t="n">
-        <v>838.3</v>
-      </c>
-      <c r="F13" s="14" t="n">
-        <v>789.6799999999999</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-27</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="C14" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E14" s="14" t="n">
-        <v>-389.53</v>
-      </c>
-      <c r="F14" s="14" t="n">
-        <v>-795.13</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-28</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>2642</v>
-      </c>
-      <c r="F15" s="14" t="n">
-        <v>2342.15</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-29</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>1048.6</v>
-      </c>
-      <c r="F16" s="14" t="n">
-        <v>611.7</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="B17" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>2810.2</v>
-      </c>
-      <c r="F17" s="14" t="n">
-        <v>2708.76</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A1:L2"/>
-    <mergeCell ref="C5:D6"/>
-    <mergeCell ref="A5:B6"/>
-    <mergeCell ref="G5:H6"/>
-    <mergeCell ref="E5:F6"/>
-    <mergeCell ref="K5:L6"/>
-    <mergeCell ref="I5:J6"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="C4:D4"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1306,2069 +634,2069 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>📅  TRADE BOOK — DAY-BY-DAY LOG</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔴  2026-07-21   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹-10.06   ·   Net PnL: ₹-99.00</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n"/>
-      <c r="C3" s="17" t="n"/>
-      <c r="D3" s="17" t="n"/>
-      <c r="E3" s="17" t="n"/>
-      <c r="F3" s="17" t="n"/>
-      <c r="G3" s="17" t="n"/>
-      <c r="H3" s="17" t="n"/>
-      <c r="I3" s="17" t="n"/>
-      <c r="J3" s="17" t="n"/>
-      <c r="K3" s="17" t="n"/>
-      <c r="L3" s="18" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="4" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I4" s="20" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J4" s="20" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K4" s="20" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L4" s="21" t="inlineStr">
+      <c r="L4" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>EPIGRAL</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E5" s="24" t="n">
+      <c r="E5" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="25" t="n">
+      <c r="F5" s="11" t="n">
         <v>1162.9</v>
       </c>
-      <c r="G5" s="25" t="n">
+      <c r="G5" s="11" t="n">
         <v>1157.5</v>
       </c>
-      <c r="H5" s="25" t="n">
+      <c r="H5" s="11" t="n">
         <v>-5.4</v>
       </c>
-      <c r="I5" s="26" t="n">
+      <c r="I5" s="12" t="n">
         <v>-0.4644</v>
       </c>
-      <c r="J5" s="25" t="n">
+      <c r="J5" s="11" t="n">
         <v>17.75</v>
       </c>
-      <c r="K5" s="25" t="n">
+      <c r="K5" s="11" t="n">
         <v>-23.15</v>
       </c>
-      <c r="L5" s="27" t="n">
+      <c r="L5" s="13" t="n">
         <v>-1.9907</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>RAJRATAN</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E6" s="24" t="n">
+      <c r="E6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="11" t="n">
         <v>512.675</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="11" t="n">
         <v>512.45</v>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="H6" s="11" t="n">
         <v>-0.45</v>
       </c>
-      <c r="I6" s="26" t="n">
+      <c r="I6" s="12" t="n">
         <v>-0.0439</v>
       </c>
-      <c r="J6" s="25" t="n">
+      <c r="J6" s="11" t="n">
         <v>17.47</v>
       </c>
-      <c r="K6" s="25" t="n">
+      <c r="K6" s="11" t="n">
         <v>-17.92</v>
       </c>
-      <c r="L6" s="27" t="n">
+      <c r="L6" s="13" t="n">
         <v>-1.7477</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>SHK</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E7" s="24" t="n">
+      <c r="E7" s="10" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="11" t="n">
         <v>143</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="11" t="n">
         <v>142.06</v>
       </c>
-      <c r="H7" s="25" t="n">
+      <c r="H7" s="11" t="n">
         <v>-8.460000000000001</v>
       </c>
-      <c r="I7" s="26" t="n">
+      <c r="I7" s="12" t="n">
         <v>-0.6573</v>
       </c>
-      <c r="J7" s="25" t="n">
+      <c r="J7" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="K7" s="25" t="n">
+      <c r="K7" s="11" t="n">
         <v>-26.46</v>
       </c>
-      <c r="L7" s="27" t="n">
+      <c r="L7" s="13" t="n">
         <v>-2.0559</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>STALLION</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="31" t="n">
+      <c r="F8" s="17" t="n">
         <v>246.12</v>
       </c>
-      <c r="G8" s="31" t="n">
+      <c r="G8" s="17" t="n">
         <v>255.55</v>
       </c>
-      <c r="H8" s="31" t="n">
+      <c r="H8" s="17" t="n">
         <v>47.15</v>
       </c>
-      <c r="I8" s="32" t="n">
+      <c r="I8" s="18" t="n">
         <v>3.8315</v>
       </c>
-      <c r="J8" s="31" t="n">
+      <c r="J8" s="17" t="n">
         <v>17.94</v>
       </c>
-      <c r="K8" s="31" t="n">
+      <c r="K8" s="17" t="n">
         <v>29.21</v>
       </c>
-      <c r="L8" s="33" t="n">
+      <c r="L8" s="19" t="n">
         <v>2.3736</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>VIMTALABS</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>2026-07-21</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E9" s="24" t="n">
+      <c r="E9" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="11" t="n">
         <v>598.3</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="11" t="n">
         <v>576.85</v>
       </c>
-      <c r="H9" s="25" t="n">
+      <c r="H9" s="11" t="n">
         <v>-42.9</v>
       </c>
-      <c r="I9" s="26" t="n">
+      <c r="I9" s="12" t="n">
         <v>-3.5852</v>
       </c>
-      <c r="J9" s="25" t="n">
+      <c r="J9" s="11" t="n">
         <v>17.78</v>
       </c>
-      <c r="K9" s="25" t="n">
+      <c r="K9" s="11" t="n">
         <v>-60.68</v>
       </c>
-      <c r="L9" s="27" t="n">
+      <c r="L9" s="13" t="n">
         <v>-5.071</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="34" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B10" s="35" t="n"/>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="35" t="n"/>
-      <c r="G10" s="35" t="n"/>
-      <c r="H10" s="36" t="n">
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="22" t="n">
         <v>-10.06</v>
       </c>
-      <c r="I10" s="35" t="n"/>
-      <c r="J10" s="35" t="n"/>
-      <c r="K10" s="36" t="n">
+      <c r="I10" s="21" t="n"/>
+      <c r="J10" s="21" t="n"/>
+      <c r="K10" s="22" t="n">
         <v>-99</v>
       </c>
-      <c r="L10" s="37" t="n"/>
+      <c r="L10" s="23" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟢  2026-07-22   ·   2 trade(s), 2 closed   ·   Gross PnL: ₹159.08   ·   Net PnL: ₹118.22</t>
         </is>
       </c>
-      <c r="B12" s="17" t="n"/>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="17" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="17" t="n"/>
-      <c r="I12" s="17" t="n"/>
-      <c r="J12" s="17" t="n"/>
-      <c r="K12" s="17" t="n"/>
-      <c r="L12" s="18" t="n"/>
+      <c r="B12" s="3" t="n"/>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+      <c r="E12" s="3" t="n"/>
+      <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="n"/>
+      <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="4" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C13" s="20" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D13" s="20" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E13" s="20" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F13" s="20" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G13" s="20" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H13" s="20" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I13" s="20" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J13" s="20" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K13" s="20" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L13" s="21" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>HUHTAMAKI</t>
         </is>
       </c>
-      <c r="C14" s="29" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="D14" s="29" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E14" s="30" t="n">
+      <c r="E14" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="F14" s="31" t="n">
+      <c r="F14" s="17" t="n">
         <v>293.57</v>
       </c>
-      <c r="G14" s="31" t="n">
+      <c r="G14" s="17" t="n">
         <v>310.33</v>
       </c>
-      <c r="H14" s="31" t="n">
+      <c r="H14" s="17" t="n">
         <v>134.08</v>
       </c>
-      <c r="I14" s="32" t="n">
+      <c r="I14" s="18" t="n">
         <v>5.709</v>
       </c>
-      <c r="J14" s="31" t="n">
+      <c r="J14" s="17" t="n">
         <v>20.35</v>
       </c>
-      <c r="K14" s="31" t="n">
+      <c r="K14" s="17" t="n">
         <v>113.73</v>
       </c>
-      <c r="L14" s="33" t="n">
+      <c r="L14" s="19" t="n">
         <v>4.8425</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>UFLEX</t>
         </is>
       </c>
-      <c r="C15" s="29" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="D15" s="29" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="E15" s="30" t="n">
+      <c r="E15" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="31" t="n">
+      <c r="F15" s="17" t="n">
         <v>496</v>
       </c>
-      <c r="G15" s="31" t="n">
+      <c r="G15" s="17" t="n">
         <v>501</v>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H15" s="17" t="n">
         <v>25</v>
       </c>
-      <c r="I15" s="32" t="n">
+      <c r="I15" s="18" t="n">
         <v>1.0081</v>
       </c>
-      <c r="J15" s="31" t="n">
+      <c r="J15" s="17" t="n">
         <v>20.51</v>
       </c>
-      <c r="K15" s="31" t="n">
+      <c r="K15" s="17" t="n">
         <v>4.49</v>
       </c>
-      <c r="L15" s="33" t="n">
+      <c r="L15" s="19" t="n">
         <v>0.181</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="34" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="35" t="n"/>
-      <c r="E16" s="35" t="n"/>
-      <c r="F16" s="35" t="n"/>
-      <c r="G16" s="35" t="n"/>
-      <c r="H16" s="36" t="n">
+      <c r="B16" s="21" t="n"/>
+      <c r="C16" s="21" t="n"/>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="21" t="n"/>
+      <c r="G16" s="21" t="n"/>
+      <c r="H16" s="22" t="n">
         <v>159.08</v>
       </c>
-      <c r="I16" s="35" t="n"/>
-      <c r="J16" s="35" t="n"/>
-      <c r="K16" s="36" t="n">
+      <c r="I16" s="21" t="n"/>
+      <c r="J16" s="21" t="n"/>
+      <c r="K16" s="22" t="n">
         <v>118.22</v>
       </c>
-      <c r="L16" s="37" t="n"/>
+      <c r="L16" s="23" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔴  2026-07-23   ·   3 trade(s), 3 closed   ·   Gross PnL: ₹-137.84   ·   Net PnL: ₹-191.96</t>
         </is>
       </c>
-      <c r="B18" s="17" t="n"/>
-      <c r="C18" s="17" t="n"/>
-      <c r="D18" s="17" t="n"/>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="17" t="n"/>
-      <c r="H18" s="17" t="n"/>
-      <c r="I18" s="17" t="n"/>
-      <c r="J18" s="17" t="n"/>
-      <c r="K18" s="17" t="n"/>
-      <c r="L18" s="18" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="n"/>
+      <c r="J18" s="3" t="n"/>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B19" s="20" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C19" s="20" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D19" s="20" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E19" s="20" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F19" s="20" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G19" s="20" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H19" s="20" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I19" s="20" t="inlineStr">
+      <c r="I19" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J19" s="20" t="inlineStr">
+      <c r="J19" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K19" s="20" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L19" s="21" t="inlineStr">
+      <c r="L19" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>CHEMPLASTS</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="E20" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="F20" s="25" t="n">
+      <c r="F20" s="11" t="n">
         <v>210</v>
       </c>
-      <c r="G20" s="25" t="n">
+      <c r="G20" s="11" t="n">
         <v>203.3157</v>
       </c>
-      <c r="H20" s="25" t="n">
+      <c r="H20" s="11" t="n">
         <v>-46.79</v>
       </c>
-      <c r="I20" s="26" t="n">
+      <c r="I20" s="12" t="n">
         <v>-3.183</v>
       </c>
-      <c r="J20" s="25" t="n">
+      <c r="J20" s="11" t="n">
         <v>18.34</v>
       </c>
-      <c r="K20" s="25" t="n">
+      <c r="K20" s="11" t="n">
         <v>-65.13</v>
       </c>
-      <c r="L20" s="27" t="n">
+      <c r="L20" s="13" t="n">
         <v>-4.4306</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>ROUTE</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="E21" s="24" t="n">
+      <c r="E21" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="25" t="n">
+      <c r="F21" s="11" t="n">
         <v>600.95</v>
       </c>
-      <c r="G21" s="25" t="n">
+      <c r="G21" s="11" t="n">
         <v>574.45</v>
       </c>
-      <c r="H21" s="25" t="n">
+      <c r="H21" s="11" t="n">
         <v>-53</v>
       </c>
-      <c r="I21" s="26" t="n">
+      <c r="I21" s="12" t="n">
         <v>-4.4097</v>
       </c>
-      <c r="J21" s="25" t="n">
+      <c r="J21" s="11" t="n">
         <v>17.78</v>
       </c>
-      <c r="K21" s="25" t="n">
+      <c r="K21" s="11" t="n">
         <v>-70.78</v>
       </c>
-      <c r="L21" s="27" t="n">
+      <c r="L21" s="13" t="n">
         <v>-5.889</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>SOTL</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="9" t="inlineStr">
         <is>
           <t>2026-07-23</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="E22" s="24" t="n">
+      <c r="E22" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="25" t="n">
+      <c r="F22" s="11" t="n">
         <v>649.775</v>
       </c>
-      <c r="G22" s="25" t="n">
+      <c r="G22" s="11" t="n">
         <v>630.75</v>
       </c>
-      <c r="H22" s="25" t="n">
+      <c r="H22" s="11" t="n">
         <v>-38.05</v>
       </c>
-      <c r="I22" s="26" t="n">
+      <c r="I22" s="12" t="n">
         <v>-2.9279</v>
       </c>
-      <c r="J22" s="25" t="n">
+      <c r="J22" s="11" t="n">
         <v>18</v>
       </c>
-      <c r="K22" s="25" t="n">
+      <c r="K22" s="11" t="n">
         <v>-56.05</v>
       </c>
-      <c r="L22" s="27" t="n">
+      <c r="L22" s="13" t="n">
         <v>-4.313</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="34" t="inlineStr">
+      <c r="A23" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B23" s="35" t="n"/>
-      <c r="C23" s="35" t="n"/>
-      <c r="D23" s="35" t="n"/>
-      <c r="E23" s="35" t="n"/>
-      <c r="F23" s="35" t="n"/>
-      <c r="G23" s="35" t="n"/>
-      <c r="H23" s="36" t="n">
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="21" t="n"/>
+      <c r="G23" s="21" t="n"/>
+      <c r="H23" s="22" t="n">
         <v>-137.84</v>
       </c>
-      <c r="I23" s="35" t="n"/>
-      <c r="J23" s="35" t="n"/>
-      <c r="K23" s="36" t="n">
+      <c r="I23" s="21" t="n"/>
+      <c r="J23" s="21" t="n"/>
+      <c r="K23" s="22" t="n">
         <v>-191.96</v>
       </c>
-      <c r="L23" s="37" t="n"/>
+      <c r="L23" s="23" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟢  2026-07-24   ·   1 trade(s), 1 closed   ·   Gross PnL: ₹838.30   ·   Net PnL: ₹789.68</t>
         </is>
       </c>
-      <c r="B25" s="17" t="n"/>
-      <c r="C25" s="17" t="n"/>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="17" t="n"/>
-      <c r="F25" s="17" t="n"/>
-      <c r="G25" s="17" t="n"/>
-      <c r="H25" s="17" t="n"/>
-      <c r="I25" s="17" t="n"/>
-      <c r="J25" s="17" t="n"/>
-      <c r="K25" s="17" t="n"/>
-      <c r="L25" s="18" t="n"/>
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+      <c r="I25" s="3" t="n"/>
+      <c r="J25" s="3" t="n"/>
+      <c r="K25" s="3" t="n"/>
+      <c r="L25" s="4" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C26" s="20" t="inlineStr">
+      <c r="C26" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D26" s="20" t="inlineStr">
+      <c r="D26" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F26" s="20" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G26" s="20" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H26" s="20" t="inlineStr">
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I26" s="20" t="inlineStr">
+      <c r="I26" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J26" s="20" t="inlineStr">
+      <c r="J26" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K26" s="20" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L26" s="21" t="inlineStr">
+      <c r="L26" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>TECHNVISN</t>
         </is>
       </c>
-      <c r="C27" s="29" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="D27" s="29" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="E27" s="30" t="n">
+      <c r="E27" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="31" t="n">
+      <c r="F27" s="17" t="n">
         <v>4884.9</v>
       </c>
-      <c r="G27" s="31" t="n">
+      <c r="G27" s="17" t="n">
         <v>5164.3333</v>
       </c>
-      <c r="H27" s="31" t="n">
+      <c r="H27" s="17" t="n">
         <v>838.3</v>
       </c>
-      <c r="I27" s="32" t="n">
+      <c r="I27" s="18" t="n">
         <v>5.7203</v>
       </c>
-      <c r="J27" s="31" t="n">
+      <c r="J27" s="17" t="n">
         <v>48.62</v>
       </c>
-      <c r="K27" s="31" t="n">
+      <c r="K27" s="17" t="n">
         <v>789.6799999999999</v>
       </c>
-      <c r="L27" s="33" t="n">
+      <c r="L27" s="19" t="n">
         <v>5.3886</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="34" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B28" s="35" t="n"/>
-      <c r="C28" s="35" t="n"/>
-      <c r="D28" s="35" t="n"/>
-      <c r="E28" s="35" t="n"/>
-      <c r="F28" s="35" t="n"/>
-      <c r="G28" s="35" t="n"/>
-      <c r="H28" s="36" t="n">
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="21" t="n"/>
+      <c r="G28" s="21" t="n"/>
+      <c r="H28" s="22" t="n">
         <v>838.3</v>
       </c>
-      <c r="I28" s="35" t="n"/>
-      <c r="J28" s="35" t="n"/>
-      <c r="K28" s="36" t="n">
+      <c r="I28" s="21" t="n"/>
+      <c r="J28" s="21" t="n"/>
+      <c r="K28" s="22" t="n">
         <v>789.6799999999999</v>
       </c>
-      <c r="L28" s="37" t="n"/>
+      <c r="L28" s="23" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔴  2026-07-27   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹-389.53   ·   Net PnL: ₹-795.13</t>
         </is>
       </c>
-      <c r="B30" s="17" t="n"/>
-      <c r="C30" s="17" t="n"/>
-      <c r="D30" s="17" t="n"/>
-      <c r="E30" s="17" t="n"/>
-      <c r="F30" s="17" t="n"/>
-      <c r="G30" s="17" t="n"/>
-      <c r="H30" s="17" t="n"/>
-      <c r="I30" s="17" t="n"/>
-      <c r="J30" s="17" t="n"/>
-      <c r="K30" s="17" t="n"/>
-      <c r="L30" s="18" t="n"/>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+      <c r="I30" s="3" t="n"/>
+      <c r="J30" s="3" t="n"/>
+      <c r="K30" s="3" t="n"/>
+      <c r="L30" s="4" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="19" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B31" s="20" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C31" s="20" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D31" s="20" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E31" s="20" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F31" s="20" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G31" s="20" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H31" s="20" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I31" s="20" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J31" s="20" t="inlineStr">
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K31" s="20" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L31" s="21" t="inlineStr">
+      <c r="L31" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="inlineStr">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>CAPILLARY</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D32" s="23" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E32" s="24" t="n">
+      <c r="E32" s="10" t="n">
         <v>56</v>
       </c>
-      <c r="F32" s="25" t="n">
+      <c r="F32" s="11" t="n">
         <v>535.4</v>
       </c>
-      <c r="G32" s="25" t="n">
+      <c r="G32" s="11" t="n">
         <v>515.7</v>
       </c>
-      <c r="H32" s="25" t="n">
+      <c r="H32" s="11" t="n">
         <v>-1103.2</v>
       </c>
-      <c r="I32" s="26" t="n">
+      <c r="I32" s="12" t="n">
         <v>-3.6795</v>
       </c>
-      <c r="J32" s="25" t="n">
+      <c r="J32" s="11" t="n">
         <v>80.40000000000001</v>
       </c>
-      <c r="K32" s="25" t="n">
+      <c r="K32" s="11" t="n">
         <v>-1183.6</v>
       </c>
-      <c r="L32" s="27" t="n">
+      <c r="L32" s="13" t="n">
         <v>-3.9476</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B33" s="29" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>DEEPINDS</t>
         </is>
       </c>
-      <c r="C33" s="29" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D33" s="29" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E33" s="30" t="n">
+      <c r="E33" s="16" t="n">
         <v>57</v>
       </c>
-      <c r="F33" s="31" t="n">
+      <c r="F33" s="17" t="n">
         <v>517.9</v>
       </c>
-      <c r="G33" s="31" t="n">
+      <c r="G33" s="17" t="n">
         <v>535.2746</v>
       </c>
-      <c r="H33" s="31" t="n">
+      <c r="H33" s="17" t="n">
         <v>990.35</v>
       </c>
-      <c r="I33" s="32" t="n">
+      <c r="I33" s="18" t="n">
         <v>3.3548</v>
       </c>
-      <c r="J33" s="31" t="n">
+      <c r="J33" s="17" t="n">
         <v>81.62</v>
       </c>
-      <c r="K33" s="31" t="n">
+      <c r="K33" s="17" t="n">
         <v>908.73</v>
       </c>
-      <c r="L33" s="33" t="n">
+      <c r="L33" s="19" t="n">
         <v>3.0783</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B34" s="29" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>MONARCH</t>
         </is>
       </c>
-      <c r="C34" s="29" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D34" s="29" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E34" s="30" t="n">
+      <c r="E34" s="16" t="n">
         <v>76</v>
       </c>
-      <c r="F34" s="31" t="n">
+      <c r="F34" s="17" t="n">
         <v>391.9</v>
       </c>
-      <c r="G34" s="31" t="n">
+      <c r="G34" s="17" t="n">
         <v>395.5</v>
       </c>
-      <c r="H34" s="31" t="n">
+      <c r="H34" s="17" t="n">
         <v>273.6</v>
       </c>
-      <c r="I34" s="32" t="n">
+      <c r="I34" s="18" t="n">
         <v>0.9186</v>
       </c>
-      <c r="J34" s="31" t="n">
+      <c r="J34" s="17" t="n">
         <v>81.42</v>
       </c>
-      <c r="K34" s="31" t="n">
+      <c r="K34" s="17" t="n">
         <v>192.18</v>
       </c>
-      <c r="L34" s="33" t="n">
+      <c r="L34" s="19" t="n">
         <v>0.6452</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="inlineStr">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B35" s="23" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>SESHAPAPER</t>
         </is>
       </c>
-      <c r="C35" s="23" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D35" s="23" t="inlineStr">
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E35" s="24" t="n">
+      <c r="E35" s="10" t="n">
         <v>125</v>
       </c>
-      <c r="F35" s="25" t="n">
+      <c r="F35" s="11" t="n">
         <v>238.777</v>
       </c>
-      <c r="G35" s="25" t="n">
+      <c r="G35" s="11" t="n">
         <v>235.1329</v>
       </c>
-      <c r="H35" s="25" t="n">
+      <c r="H35" s="11" t="n">
         <v>-455.51</v>
       </c>
-      <c r="I35" s="26" t="n">
+      <c r="I35" s="12" t="n">
         <v>-1.5262</v>
       </c>
-      <c r="J35" s="25" t="n">
+      <c r="J35" s="11" t="n">
         <v>80.79000000000001</v>
       </c>
-      <c r="K35" s="25" t="n">
+      <c r="K35" s="11" t="n">
         <v>-536.3</v>
       </c>
-      <c r="L35" s="27" t="n">
+      <c r="L35" s="13" t="n">
         <v>-1.7968</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="inlineStr">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B36" s="23" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>VRLLOG</t>
         </is>
       </c>
-      <c r="C36" s="23" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="D36" s="23" t="inlineStr">
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="E36" s="24" t="n">
+      <c r="E36" s="10" t="n">
         <v>114</v>
       </c>
-      <c r="F36" s="25" t="n">
+      <c r="F36" s="11" t="n">
         <v>262.6553</v>
       </c>
-      <c r="G36" s="25" t="n">
+      <c r="G36" s="11" t="n">
         <v>261.8239</v>
       </c>
-      <c r="H36" s="25" t="n">
+      <c r="H36" s="11" t="n">
         <v>-94.77</v>
       </c>
-      <c r="I36" s="26" t="n">
+      <c r="I36" s="12" t="n">
         <v>-0.3165</v>
       </c>
-      <c r="J36" s="25" t="n">
+      <c r="J36" s="11" t="n">
         <v>81.37</v>
       </c>
-      <c r="K36" s="25" t="n">
+      <c r="K36" s="11" t="n">
         <v>-176.14</v>
       </c>
-      <c r="L36" s="27" t="n">
+      <c r="L36" s="13" t="n">
         <v>-0.5883</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="34" t="inlineStr">
+      <c r="A37" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B37" s="35" t="n"/>
-      <c r="C37" s="35" t="n"/>
-      <c r="D37" s="35" t="n"/>
-      <c r="E37" s="35" t="n"/>
-      <c r="F37" s="35" t="n"/>
-      <c r="G37" s="35" t="n"/>
-      <c r="H37" s="36" t="n">
+      <c r="B37" s="21" t="n"/>
+      <c r="C37" s="21" t="n"/>
+      <c r="D37" s="21" t="n"/>
+      <c r="E37" s="21" t="n"/>
+      <c r="F37" s="21" t="n"/>
+      <c r="G37" s="21" t="n"/>
+      <c r="H37" s="22" t="n">
         <v>-389.53</v>
       </c>
-      <c r="I37" s="35" t="n"/>
-      <c r="J37" s="35" t="n"/>
-      <c r="K37" s="36" t="n">
+      <c r="I37" s="21" t="n"/>
+      <c r="J37" s="21" t="n"/>
+      <c r="K37" s="22" t="n">
         <v>-795.13</v>
       </c>
-      <c r="L37" s="37" t="n"/>
+      <c r="L37" s="23" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="16" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟢  2026-07-28   ·   3 trade(s), 3 closed   ·   Gross PnL: ₹2,642.00   ·   Net PnL: ₹2,342.15</t>
         </is>
       </c>
-      <c r="B39" s="17" t="n"/>
-      <c r="C39" s="17" t="n"/>
-      <c r="D39" s="17" t="n"/>
-      <c r="E39" s="17" t="n"/>
-      <c r="F39" s="17" t="n"/>
-      <c r="G39" s="17" t="n"/>
-      <c r="H39" s="17" t="n"/>
-      <c r="I39" s="17" t="n"/>
-      <c r="J39" s="17" t="n"/>
-      <c r="K39" s="17" t="n"/>
-      <c r="L39" s="18" t="n"/>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+      <c r="I39" s="3" t="n"/>
+      <c r="J39" s="3" t="n"/>
+      <c r="K39" s="3" t="n"/>
+      <c r="L39" s="4" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="19" t="inlineStr">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B40" s="20" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C40" s="20" t="inlineStr">
+      <c r="C40" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D40" s="20" t="inlineStr">
+      <c r="D40" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E40" s="20" t="inlineStr">
+      <c r="E40" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F40" s="20" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G40" s="20" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H40" s="20" t="inlineStr">
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I40" s="20" t="inlineStr">
+      <c r="I40" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J40" s="20" t="inlineStr">
+      <c r="J40" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K40" s="20" t="inlineStr">
+      <c r="K40" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L40" s="21" t="inlineStr">
+      <c r="L40" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="28" t="inlineStr">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B41" s="29" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>ASHIKAG</t>
         </is>
       </c>
-      <c r="C41" s="29" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="D41" s="29" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="E41" s="30" t="n">
+      <c r="E41" s="16" t="n">
         <v>76</v>
       </c>
-      <c r="F41" s="31" t="n">
+      <c r="F41" s="17" t="n">
         <v>488.1</v>
       </c>
-      <c r="G41" s="31" t="n">
+      <c r="G41" s="17" t="n">
         <v>492.5289</v>
       </c>
-      <c r="H41" s="31" t="n">
+      <c r="H41" s="17" t="n">
         <v>336.6</v>
       </c>
-      <c r="I41" s="32" t="n">
+      <c r="I41" s="18" t="n">
         <v>0.9074</v>
       </c>
-      <c r="J41" s="31" t="n">
+      <c r="J41" s="17" t="n">
         <v>98.66</v>
       </c>
-      <c r="K41" s="31" t="n">
+      <c r="K41" s="17" t="n">
         <v>237.94</v>
       </c>
-      <c r="L41" s="33" t="n">
+      <c r="L41" s="19" t="n">
         <v>0.6414</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="28" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B42" s="29" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>ASIANTILES</t>
         </is>
       </c>
-      <c r="C42" s="29" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="D42" s="29" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="E42" s="30" t="n">
+      <c r="E42" s="16" t="n">
         <v>657</v>
       </c>
-      <c r="F42" s="31" t="n">
+      <c r="F42" s="17" t="n">
         <v>57.3382</v>
       </c>
-      <c r="G42" s="31" t="n">
+      <c r="G42" s="17" t="n">
         <v>60.62</v>
       </c>
-      <c r="H42" s="31" t="n">
+      <c r="H42" s="17" t="n">
         <v>2156.14</v>
       </c>
-      <c r="I42" s="32" t="n">
+      <c r="I42" s="18" t="n">
         <v>5.7236</v>
       </c>
-      <c r="J42" s="31" t="n">
+      <c r="J42" s="17" t="n">
         <v>101.74</v>
       </c>
-      <c r="K42" s="31" t="n">
+      <c r="K42" s="17" t="n">
         <v>2054.4</v>
       </c>
-      <c r="L42" s="33" t="n">
+      <c r="L42" s="19" t="n">
         <v>5.4535</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B43" s="29" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>INFOBEAN</t>
         </is>
       </c>
-      <c r="C43" s="29" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
-      <c r="D43" s="29" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="E43" s="30" t="n">
+      <c r="E43" s="16" t="n">
         <v>223</v>
       </c>
-      <c r="F43" s="31" t="n">
+      <c r="F43" s="17" t="n">
         <v>168.4769</v>
       </c>
-      <c r="G43" s="31" t="n">
+      <c r="G43" s="17" t="n">
         <v>169.1462</v>
       </c>
-      <c r="H43" s="31" t="n">
+      <c r="H43" s="17" t="n">
         <v>149.26</v>
       </c>
-      <c r="I43" s="32" t="n">
+      <c r="I43" s="18" t="n">
         <v>0.3973</v>
       </c>
-      <c r="J43" s="31" t="n">
+      <c r="J43" s="17" t="n">
         <v>99.45</v>
       </c>
-      <c r="K43" s="31" t="n">
+      <c r="K43" s="17" t="n">
         <v>49.81</v>
       </c>
-      <c r="L43" s="33" t="n">
+      <c r="L43" s="19" t="n">
         <v>0.1326</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="34" t="inlineStr">
+      <c r="A44" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B44" s="35" t="n"/>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="n"/>
-      <c r="F44" s="35" t="n"/>
-      <c r="G44" s="35" t="n"/>
-      <c r="H44" s="36" t="n">
+      <c r="B44" s="21" t="n"/>
+      <c r="C44" s="21" t="n"/>
+      <c r="D44" s="21" t="n"/>
+      <c r="E44" s="21" t="n"/>
+      <c r="F44" s="21" t="n"/>
+      <c r="G44" s="21" t="n"/>
+      <c r="H44" s="22" t="n">
         <v>2642</v>
       </c>
-      <c r="I44" s="35" t="n"/>
-      <c r="J44" s="35" t="n"/>
-      <c r="K44" s="36" t="n">
+      <c r="I44" s="21" t="n"/>
+      <c r="J44" s="21" t="n"/>
+      <c r="K44" s="22" t="n">
         <v>2342.15</v>
       </c>
-      <c r="L44" s="37" t="n"/>
+      <c r="L44" s="23" t="n"/>
     </row>
     <row r="46" ht="22" customHeight="1">
-      <c r="A46" s="16" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟢  2026-07-29   ·   7 trade(s), 7 closed   ·   Gross PnL: ₹1,048.60   ·   Net PnL: ₹611.70</t>
         </is>
       </c>
-      <c r="B46" s="17" t="n"/>
-      <c r="C46" s="17" t="n"/>
-      <c r="D46" s="17" t="n"/>
-      <c r="E46" s="17" t="n"/>
-      <c r="F46" s="17" t="n"/>
-      <c r="G46" s="17" t="n"/>
-      <c r="H46" s="17" t="n"/>
-      <c r="I46" s="17" t="n"/>
-      <c r="J46" s="17" t="n"/>
-      <c r="K46" s="17" t="n"/>
-      <c r="L46" s="18" t="n"/>
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+      <c r="I46" s="3" t="n"/>
+      <c r="J46" s="3" t="n"/>
+      <c r="K46" s="3" t="n"/>
+      <c r="L46" s="4" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B47" s="20" t="inlineStr">
+      <c r="B47" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C47" s="20" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D47" s="20" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E47" s="20" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F47" s="20" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G47" s="20" t="inlineStr">
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H47" s="20" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I47" s="20" t="inlineStr">
+      <c r="I47" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J47" s="20" t="inlineStr">
+      <c r="J47" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K47" s="20" t="inlineStr">
+      <c r="K47" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L47" s="21" t="inlineStr">
+      <c r="L47" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="inlineStr">
+      <c r="A48" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B48" s="23" t="inlineStr">
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>APCOTEXIND</t>
         </is>
       </c>
-      <c r="C48" s="23" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D48" s="23" t="inlineStr">
+      <c r="D48" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E48" s="24" t="n">
+      <c r="E48" s="10" t="n">
         <v>31</v>
       </c>
-      <c r="F48" s="25" t="n">
+      <c r="F48" s="11" t="n">
         <v>683.65</v>
       </c>
-      <c r="G48" s="25" t="n">
+      <c r="G48" s="11" t="n">
         <v>668.25</v>
       </c>
-      <c r="H48" s="25" t="n">
+      <c r="H48" s="11" t="n">
         <v>-477.4</v>
       </c>
-      <c r="I48" s="26" t="n">
+      <c r="I48" s="12" t="n">
         <v>-2.2526</v>
       </c>
-      <c r="J48" s="25" t="n">
+      <c r="J48" s="11" t="n">
         <v>61.82</v>
       </c>
-      <c r="K48" s="25" t="n">
+      <c r="K48" s="11" t="n">
         <v>-539.22</v>
       </c>
-      <c r="L48" s="27" t="n">
+      <c r="L48" s="13" t="n">
         <v>-2.5443</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="28" t="inlineStr">
+      <c r="A49" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B49" s="29" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>ARTEMISMED</t>
         </is>
       </c>
-      <c r="C49" s="29" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D49" s="29" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E49" s="30" t="n">
+      <c r="E49" s="16" t="n">
         <v>72</v>
       </c>
-      <c r="F49" s="31" t="n">
+      <c r="F49" s="17" t="n">
         <v>296.9</v>
       </c>
-      <c r="G49" s="31" t="n">
+      <c r="G49" s="17" t="n">
         <v>301.1042</v>
       </c>
-      <c r="H49" s="31" t="n">
+      <c r="H49" s="17" t="n">
         <v>302.7</v>
       </c>
-      <c r="I49" s="32" t="n">
+      <c r="I49" s="18" t="n">
         <v>1.416</v>
       </c>
-      <c r="J49" s="31" t="n">
+      <c r="J49" s="17" t="n">
         <v>63.01</v>
       </c>
-      <c r="K49" s="31" t="n">
+      <c r="K49" s="17" t="n">
         <v>239.69</v>
       </c>
-      <c r="L49" s="33" t="n">
+      <c r="L49" s="19" t="n">
         <v>1.1213</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="inlineStr">
+      <c r="A50" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B50" s="23" t="inlineStr">
+      <c r="B50" s="9" t="inlineStr">
         <is>
           <t>ASIANTILES</t>
         </is>
       </c>
-      <c r="C50" s="23" t="inlineStr">
+      <c r="C50" s="9" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D50" s="23" t="inlineStr">
+      <c r="D50" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E50" s="24" t="n">
+      <c r="E50" s="10" t="n">
         <v>347</v>
       </c>
-      <c r="F50" s="25" t="n">
+      <c r="F50" s="11" t="n">
         <v>61.59</v>
       </c>
-      <c r="G50" s="25" t="n">
+      <c r="G50" s="11" t="n">
         <v>61</v>
       </c>
-      <c r="H50" s="25" t="n">
+      <c r="H50" s="11" t="n">
         <v>-204.73</v>
       </c>
-      <c r="I50" s="26" t="n">
+      <c r="I50" s="12" t="n">
         <v>-0.9579</v>
       </c>
-      <c r="J50" s="25" t="n">
+      <c r="J50" s="11" t="n">
         <v>62.47</v>
       </c>
-      <c r="K50" s="25" t="n">
+      <c r="K50" s="11" t="n">
         <v>-267.2</v>
       </c>
-      <c r="L50" s="27" t="n">
+      <c r="L50" s="13" t="n">
         <v>-1.2502</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="28" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B51" s="29" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>DEEPINDS</t>
         </is>
       </c>
-      <c r="C51" s="29" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D51" s="29" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E51" s="30" t="n">
+      <c r="E51" s="16" t="n">
         <v>39</v>
       </c>
-      <c r="F51" s="31" t="n">
+      <c r="F51" s="17" t="n">
         <v>543.6769</v>
       </c>
-      <c r="G51" s="31" t="n">
+      <c r="G51" s="17" t="n">
         <v>571.4</v>
       </c>
-      <c r="H51" s="31" t="n">
+      <c r="H51" s="17" t="n">
         <v>1081.2</v>
       </c>
-      <c r="I51" s="32" t="n">
+      <c r="I51" s="18" t="n">
         <v>5.0992</v>
       </c>
-      <c r="J51" s="31" t="n">
+      <c r="J51" s="17" t="n">
         <v>63.45</v>
       </c>
-      <c r="K51" s="31" t="n">
+      <c r="K51" s="17" t="n">
         <v>1017.75</v>
       </c>
-      <c r="L51" s="33" t="n">
+      <c r="L51" s="19" t="n">
         <v>4.7999</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="28" t="inlineStr">
+      <c r="A52" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B52" s="29" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>ORISSAMINE</t>
         </is>
       </c>
-      <c r="C52" s="29" t="inlineStr">
+      <c r="C52" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D52" s="29" t="inlineStr">
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E52" s="30" t="n">
+      <c r="E52" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="F52" s="31" t="n">
+      <c r="F52" s="17" t="n">
         <v>4045.4</v>
       </c>
-      <c r="G52" s="31" t="n">
+      <c r="G52" s="17" t="n">
         <v>4050.12</v>
       </c>
-      <c r="H52" s="31" t="n">
+      <c r="H52" s="17" t="n">
         <v>23.6</v>
       </c>
-      <c r="I52" s="32" t="n">
+      <c r="I52" s="18" t="n">
         <v>0.1167</v>
       </c>
-      <c r="J52" s="31" t="n">
+      <c r="J52" s="17" t="n">
         <v>60.33</v>
       </c>
-      <c r="K52" s="31" t="n">
+      <c r="K52" s="17" t="n">
         <v>-36.73</v>
       </c>
-      <c r="L52" s="33" t="n">
+      <c r="L52" s="19" t="n">
         <v>-0.1816</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="28" t="inlineStr">
+      <c r="A53" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B53" s="29" t="inlineStr">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>SHK</t>
         </is>
       </c>
-      <c r="C53" s="29" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D53" s="29" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E53" s="30" t="n">
+      <c r="E53" s="16" t="n">
         <v>131</v>
       </c>
-      <c r="F53" s="31" t="n">
+      <c r="F53" s="17" t="n">
         <v>162.6454</v>
       </c>
-      <c r="G53" s="31" t="n">
+      <c r="G53" s="17" t="n">
         <v>168.1477</v>
       </c>
-      <c r="H53" s="31" t="n">
+      <c r="H53" s="17" t="n">
         <v>720.8</v>
       </c>
-      <c r="I53" s="32" t="n">
+      <c r="I53" s="18" t="n">
         <v>3.383</v>
       </c>
-      <c r="J53" s="31" t="n">
+      <c r="J53" s="17" t="n">
         <v>63.29</v>
       </c>
-      <c r="K53" s="31" t="n">
+      <c r="K53" s="17" t="n">
         <v>657.51</v>
       </c>
-      <c r="L53" s="33" t="n">
+      <c r="L53" s="19" t="n">
         <v>3.086</v>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="22" t="inlineStr">
+      <c r="A54" s="8" t="inlineStr">
         <is>
           <t>🔴 LOSS</t>
         </is>
       </c>
-      <c r="B54" s="23" t="inlineStr">
+      <c r="B54" s="9" t="inlineStr">
         <is>
           <t>TIL</t>
         </is>
       </c>
-      <c r="C54" s="23" t="inlineStr">
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="D54" s="23" t="inlineStr">
+      <c r="D54" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="E54" s="24" t="n">
+      <c r="E54" s="10" t="n">
         <v>83</v>
       </c>
-      <c r="F54" s="25" t="n">
+      <c r="F54" s="11" t="n">
         <v>259</v>
       </c>
-      <c r="G54" s="25" t="n">
+      <c r="G54" s="11" t="n">
         <v>254.21</v>
       </c>
-      <c r="H54" s="25" t="n">
+      <c r="H54" s="11" t="n">
         <v>-397.57</v>
       </c>
-      <c r="I54" s="26" t="n">
+      <c r="I54" s="12" t="n">
         <v>-1.8494</v>
       </c>
-      <c r="J54" s="25" t="n">
+      <c r="J54" s="11" t="n">
         <v>62.53</v>
       </c>
-      <c r="K54" s="25" t="n">
+      <c r="K54" s="11" t="n">
         <v>-460.1</v>
       </c>
-      <c r="L54" s="27" t="n">
+      <c r="L54" s="13" t="n">
         <v>-2.1403</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="34" t="inlineStr">
+      <c r="A55" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B55" s="35" t="n"/>
-      <c r="C55" s="35" t="n"/>
-      <c r="D55" s="35" t="n"/>
-      <c r="E55" s="35" t="n"/>
-      <c r="F55" s="35" t="n"/>
-      <c r="G55" s="35" t="n"/>
-      <c r="H55" s="36" t="n">
+      <c r="B55" s="21" t="n"/>
+      <c r="C55" s="21" t="n"/>
+      <c r="D55" s="21" t="n"/>
+      <c r="E55" s="21" t="n"/>
+      <c r="F55" s="21" t="n"/>
+      <c r="G55" s="21" t="n"/>
+      <c r="H55" s="22" t="n">
         <v>1048.6</v>
       </c>
-      <c r="I55" s="35" t="n"/>
-      <c r="J55" s="35" t="n"/>
-      <c r="K55" s="36" t="n">
+      <c r="I55" s="21" t="n"/>
+      <c r="J55" s="21" t="n"/>
+      <c r="K55" s="22" t="n">
         <v>611.7</v>
       </c>
-      <c r="L55" s="37" t="n"/>
+      <c r="L55" s="23" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1">
-      <c r="A57" s="16" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  🟢  2026-07-30   ·   1 trade(s), 1 closed   ·   Gross PnL: ₹2,810.20   ·   Net PnL: ₹2,708.76</t>
         </is>
       </c>
-      <c r="B57" s="17" t="n"/>
-      <c r="C57" s="17" t="n"/>
-      <c r="D57" s="17" t="n"/>
-      <c r="E57" s="17" t="n"/>
-      <c r="F57" s="17" t="n"/>
-      <c r="G57" s="17" t="n"/>
-      <c r="H57" s="17" t="n"/>
-      <c r="I57" s="17" t="n"/>
-      <c r="J57" s="17" t="n"/>
-      <c r="K57" s="17" t="n"/>
-      <c r="L57" s="18" t="n"/>
+      <c r="B57" s="3" t="n"/>
+      <c r="C57" s="3" t="n"/>
+      <c r="D57" s="3" t="n"/>
+      <c r="E57" s="3" t="n"/>
+      <c r="F57" s="3" t="n"/>
+      <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="n"/>
+      <c r="I57" s="3" t="n"/>
+      <c r="J57" s="3" t="n"/>
+      <c r="K57" s="3" t="n"/>
+      <c r="L57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="19" t="inlineStr">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="B58" s="20" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>Stock Name</t>
         </is>
       </c>
-      <c r="C58" s="20" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>Position entry date</t>
         </is>
       </c>
-      <c r="D58" s="20" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>Position Exit date</t>
         </is>
       </c>
-      <c r="E58" s="20" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>No of shares</t>
         </is>
       </c>
-      <c r="F58" s="20" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>Entry Price</t>
         </is>
       </c>
-      <c r="G58" s="20" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H58" s="20" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I58" s="20" t="inlineStr">
+      <c r="I58" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J58" s="20" t="inlineStr">
+      <c r="J58" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K58" s="20" t="inlineStr">
+      <c r="K58" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L58" s="21" t="inlineStr">
+      <c r="L58" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="inlineStr">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>🟢 WIN</t>
         </is>
       </c>
-      <c r="B59" s="29" t="inlineStr">
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t>63MOONS</t>
         </is>
       </c>
-      <c r="C59" s="29" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="D59" s="29" t="inlineStr">
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="E59" s="30" t="n">
+      <c r="E59" s="16" t="n">
         <v>44</v>
       </c>
-      <c r="F59" s="31" t="n">
+      <c r="F59" s="17" t="n">
         <v>845.4318</v>
       </c>
-      <c r="G59" s="31" t="n">
+      <c r="G59" s="17" t="n">
         <v>909.3</v>
       </c>
-      <c r="H59" s="31" t="n">
+      <c r="H59" s="17" t="n">
         <v>2810.2</v>
       </c>
-      <c r="I59" s="32" t="n">
+      <c r="I59" s="18" t="n">
         <v>7.5545</v>
       </c>
-      <c r="J59" s="31" t="n">
+      <c r="J59" s="17" t="n">
         <v>101.44</v>
       </c>
-      <c r="K59" s="31" t="n">
+      <c r="K59" s="17" t="n">
         <v>2708.76</v>
       </c>
-      <c r="L59" s="33" t="n">
+      <c r="L59" s="19" t="n">
         <v>7.2818</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="34" t="inlineStr">
+      <c r="A60" s="20" t="inlineStr">
         <is>
           <t>Σ Day total</t>
         </is>
       </c>
-      <c r="B60" s="35" t="n"/>
-      <c r="C60" s="35" t="n"/>
-      <c r="D60" s="35" t="n"/>
-      <c r="E60" s="35" t="n"/>
-      <c r="F60" s="35" t="n"/>
-      <c r="G60" s="35" t="n"/>
-      <c r="H60" s="36" t="n">
+      <c r="B60" s="21" t="n"/>
+      <c r="C60" s="21" t="n"/>
+      <c r="D60" s="21" t="n"/>
+      <c r="E60" s="21" t="n"/>
+      <c r="F60" s="21" t="n"/>
+      <c r="G60" s="21" t="n"/>
+      <c r="H60" s="22" t="n">
         <v>2810.2</v>
       </c>
-      <c r="I60" s="35" t="n"/>
-      <c r="J60" s="35" t="n"/>
-      <c r="K60" s="36" t="n">
+      <c r="I60" s="21" t="n"/>
+      <c r="J60" s="21" t="n"/>
+      <c r="K60" s="22" t="n">
         <v>2708.76</v>
       </c>
-      <c r="L60" s="37" t="n"/>
+      <c r="L60" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">

</xml_diff>

<commit_message>
Data update — 2026-07-31 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,8 +47,12 @@
     <font>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -216,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -251,6 +260,12 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -616,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2698,8 +2713,230 @@
       </c>
       <c r="L60" s="23" t="n"/>
     </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-07-31   ·   4 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="n"/>
+      <c r="C62" s="3" t="n"/>
+      <c r="D62" s="3" t="n"/>
+      <c r="E62" s="3" t="n"/>
+      <c r="F62" s="3" t="n"/>
+      <c r="G62" s="3" t="n"/>
+      <c r="H62" s="3" t="n"/>
+      <c r="I62" s="3" t="n"/>
+      <c r="J62" s="3" t="n"/>
+      <c r="K62" s="3" t="n"/>
+      <c r="L62" s="4" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="I63" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="J63" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="K63" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B64" s="25" t="inlineStr">
+        <is>
+          <t>63MOONS</t>
+        </is>
+      </c>
+      <c r="C64" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D64" s="25" t="n"/>
+      <c r="E64" s="26" t="n">
+        <v>27</v>
+      </c>
+      <c r="F64" s="27" t="n">
+        <v>920.9981</v>
+      </c>
+      <c r="G64" s="27" t="n"/>
+      <c r="H64" s="27" t="n"/>
+      <c r="I64" s="28" t="n"/>
+      <c r="J64" s="27" t="n"/>
+      <c r="K64" s="27" t="n"/>
+      <c r="L64" s="29" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B65" s="25" t="inlineStr">
+        <is>
+          <t>ESAFSFB</t>
+        </is>
+      </c>
+      <c r="C65" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D65" s="25" t="n"/>
+      <c r="E65" s="26" t="n">
+        <v>594</v>
+      </c>
+      <c r="F65" s="27" t="n">
+        <v>41.95</v>
+      </c>
+      <c r="G65" s="27" t="n"/>
+      <c r="H65" s="27" t="n"/>
+      <c r="I65" s="28" t="n"/>
+      <c r="J65" s="27" t="n"/>
+      <c r="K65" s="27" t="n"/>
+      <c r="L65" s="29" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B66" s="25" t="inlineStr">
+        <is>
+          <t>THEJO</t>
+        </is>
+      </c>
+      <c r="C66" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D66" s="25" t="n"/>
+      <c r="E66" s="26" t="n">
+        <v>11</v>
+      </c>
+      <c r="F66" s="27" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G66" s="27" t="n"/>
+      <c r="H66" s="27" t="n"/>
+      <c r="I66" s="28" t="n"/>
+      <c r="J66" s="27" t="n"/>
+      <c r="K66" s="27" t="n"/>
+      <c r="L66" s="29" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B67" s="25" t="inlineStr">
+        <is>
+          <t>VERANDA</t>
+        </is>
+      </c>
+      <c r="C67" s="25" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="D67" s="25" t="n"/>
+      <c r="E67" s="26" t="n">
+        <v>96</v>
+      </c>
+      <c r="F67" s="27" t="n">
+        <v>259.22</v>
+      </c>
+      <c r="G67" s="27" t="n"/>
+      <c r="H67" s="27" t="n"/>
+      <c r="I67" s="28" t="n"/>
+      <c r="J67" s="27" t="n"/>
+      <c r="K67" s="27" t="n"/>
+      <c r="L67" s="29" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B68" s="21" t="n"/>
+      <c r="C68" s="21" t="n"/>
+      <c r="D68" s="21" t="n"/>
+      <c r="E68" s="21" t="n"/>
+      <c r="F68" s="21" t="n"/>
+      <c r="G68" s="21" t="n"/>
+      <c r="H68" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="21" t="n"/>
+      <c r="J68" s="21" t="n"/>
+      <c r="K68" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" s="23" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A57:L57"/>
     <mergeCell ref="A30:L30"/>
     <mergeCell ref="A25:L25"/>
@@ -2709,6 +2946,7 @@
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A39:L39"/>
     <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A62:L62"/>
   </mergeCells>
   <conditionalFormatting sqref="H5:H9">
     <cfRule type="dataBar" priority="1">
@@ -2854,6 +3092,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H64:H67">
+    <cfRule type="dataBar" priority="17">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K64:K67">
+    <cfRule type="dataBar" priority="18">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-03 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2716,7 +2716,7 @@
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-07-31   ·   4 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-07-31   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹206.88   ·   Net PnL: ₹-72.55</t>
         </is>
       </c>
       <c r="B62" s="3" t="n"/>
@@ -2794,124 +2794,188 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B64" s="25" t="inlineStr">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t>63MOONS</t>
         </is>
       </c>
-      <c r="C64" s="25" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D64" s="25" t="n"/>
-      <c r="E64" s="26" t="n">
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="F64" s="27" t="n">
+      <c r="F64" s="17" t="n">
         <v>920.9981</v>
       </c>
-      <c r="G64" s="27" t="n"/>
-      <c r="H64" s="27" t="n"/>
-      <c r="I64" s="28" t="n"/>
-      <c r="J64" s="27" t="n"/>
-      <c r="K64" s="27" t="n"/>
-      <c r="L64" s="29" t="n"/>
+      <c r="G64" s="17" t="n">
+        <v>941.8</v>
+      </c>
+      <c r="H64" s="17" t="n">
+        <v>561.65</v>
+      </c>
+      <c r="I64" s="18" t="n">
+        <v>2.2586</v>
+      </c>
+      <c r="J64" s="17" t="n">
+        <v>71.52</v>
+      </c>
+      <c r="K64" s="17" t="n">
+        <v>490.13</v>
+      </c>
+      <c r="L64" s="19" t="n">
+        <v>1.971</v>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B65" s="25" t="inlineStr">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B65" s="9" t="inlineStr">
         <is>
           <t>ESAFSFB</t>
         </is>
       </c>
-      <c r="C65" s="25" t="inlineStr">
+      <c r="C65" s="9" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D65" s="25" t="n"/>
-      <c r="E65" s="26" t="n">
+      <c r="D65" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E65" s="10" t="n">
         <v>594</v>
       </c>
-      <c r="F65" s="27" t="n">
+      <c r="F65" s="11" t="n">
         <v>41.95</v>
       </c>
-      <c r="G65" s="27" t="n"/>
-      <c r="H65" s="27" t="n"/>
-      <c r="I65" s="28" t="n"/>
-      <c r="J65" s="27" t="n"/>
-      <c r="K65" s="27" t="n"/>
-      <c r="L65" s="29" t="n"/>
+      <c r="G65" s="11" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="H65" s="11" t="n">
+        <v>-29.7</v>
+      </c>
+      <c r="I65" s="12" t="n">
+        <v>-0.1192</v>
+      </c>
+      <c r="J65" s="11" t="n">
+        <v>71.01000000000001</v>
+      </c>
+      <c r="K65" s="11" t="n">
+        <v>-100.71</v>
+      </c>
+      <c r="L65" s="13" t="n">
+        <v>-0.4042</v>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B66" s="25" t="inlineStr">
+      <c r="A66" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
         <is>
           <t>THEJO</t>
         </is>
       </c>
-      <c r="C66" s="25" t="inlineStr">
+      <c r="C66" s="15" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D66" s="25" t="n"/>
-      <c r="E66" s="26" t="n">
+      <c r="D66" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="F66" s="27" t="n">
+      <c r="F66" s="17" t="n">
         <v>2100</v>
       </c>
-      <c r="G66" s="27" t="n"/>
-      <c r="H66" s="27" t="n"/>
-      <c r="I66" s="28" t="n"/>
-      <c r="J66" s="27" t="n"/>
-      <c r="K66" s="27" t="n"/>
-      <c r="L66" s="29" t="n"/>
+      <c r="G66" s="17" t="n">
+        <v>2110.0455</v>
+      </c>
+      <c r="H66" s="17" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="I66" s="18" t="n">
+        <v>0.4784</v>
+      </c>
+      <c r="J66" s="17" t="n">
+        <v>66.38</v>
+      </c>
+      <c r="K66" s="17" t="n">
+        <v>44.12</v>
+      </c>
+      <c r="L66" s="19" t="n">
+        <v>0.191</v>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B67" s="25" t="inlineStr">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B67" s="9" t="inlineStr">
         <is>
           <t>VERANDA</t>
         </is>
       </c>
-      <c r="C67" s="25" t="inlineStr">
+      <c r="C67" s="9" t="inlineStr">
         <is>
           <t>2026-07-31</t>
         </is>
       </c>
-      <c r="D67" s="25" t="n"/>
-      <c r="E67" s="26" t="n">
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="n">
         <v>96</v>
       </c>
-      <c r="F67" s="27" t="n">
+      <c r="F67" s="11" t="n">
         <v>259.22</v>
       </c>
-      <c r="G67" s="27" t="n"/>
-      <c r="H67" s="27" t="n"/>
-      <c r="I67" s="28" t="n"/>
-      <c r="J67" s="27" t="n"/>
-      <c r="K67" s="27" t="n"/>
-      <c r="L67" s="29" t="n"/>
+      <c r="G67" s="11" t="n">
+        <v>254.6828</v>
+      </c>
+      <c r="H67" s="11" t="n">
+        <v>-435.57</v>
+      </c>
+      <c r="I67" s="12" t="n">
+        <v>-1.7503</v>
+      </c>
+      <c r="J67" s="11" t="n">
+        <v>70.52</v>
+      </c>
+      <c r="K67" s="11" t="n">
+        <v>-506.09</v>
+      </c>
+      <c r="L67" s="13" t="n">
+        <v>-2.0337</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="20" t="inlineStr">
@@ -2926,23 +2990,276 @@
       <c r="F68" s="21" t="n"/>
       <c r="G68" s="21" t="n"/>
       <c r="H68" s="22" t="n">
-        <v>0</v>
+        <v>206.88</v>
       </c>
       <c r="I68" s="21" t="n"/>
       <c r="J68" s="21" t="n"/>
       <c r="K68" s="22" t="n">
+        <v>-72.55</v>
+      </c>
+      <c r="L68" s="23" t="n"/>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-03   ·   5 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="n"/>
+      <c r="C70" s="3" t="n"/>
+      <c r="D70" s="3" t="n"/>
+      <c r="E70" s="3" t="n"/>
+      <c r="F70" s="3" t="n"/>
+      <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
+      <c r="I70" s="3" t="n"/>
+      <c r="J70" s="3" t="n"/>
+      <c r="K70" s="3" t="n"/>
+      <c r="L70" s="4" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F71" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="K71" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="L71" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B72" s="25" t="inlineStr">
+        <is>
+          <t>DALMIASUG</t>
+        </is>
+      </c>
+      <c r="C72" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D72" s="25" t="n"/>
+      <c r="E72" s="26" t="n">
+        <v>52</v>
+      </c>
+      <c r="F72" s="27" t="n">
+        <v>407.5</v>
+      </c>
+      <c r="G72" s="27" t="n"/>
+      <c r="H72" s="27" t="n"/>
+      <c r="I72" s="28" t="n"/>
+      <c r="J72" s="27" t="n"/>
+      <c r="K72" s="27" t="n"/>
+      <c r="L72" s="29" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B73" s="25" t="inlineStr">
+        <is>
+          <t>DEEPINDS</t>
+        </is>
+      </c>
+      <c r="C73" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D73" s="25" t="n"/>
+      <c r="E73" s="26" t="n">
+        <v>33</v>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>646.15</v>
+      </c>
+      <c r="G73" s="27" t="n"/>
+      <c r="H73" s="27" t="n"/>
+      <c r="I73" s="28" t="n"/>
+      <c r="J73" s="27" t="n"/>
+      <c r="K73" s="27" t="n"/>
+      <c r="L73" s="29" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B74" s="25" t="inlineStr">
+        <is>
+          <t>JINDWORLD</t>
+        </is>
+      </c>
+      <c r="C74" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D74" s="25" t="n"/>
+      <c r="E74" s="26" t="n">
+        <v>528</v>
+      </c>
+      <c r="F74" s="27" t="n">
+        <v>40.52</v>
+      </c>
+      <c r="G74" s="27" t="n"/>
+      <c r="H74" s="27" t="n"/>
+      <c r="I74" s="28" t="n"/>
+      <c r="J74" s="27" t="n"/>
+      <c r="K74" s="27" t="n"/>
+      <c r="L74" s="29" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B75" s="25" t="inlineStr">
+        <is>
+          <t>LUMAXIND</t>
+        </is>
+      </c>
+      <c r="C75" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D75" s="25" t="n"/>
+      <c r="E75" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" s="27" t="n">
+        <v>5745.3333</v>
+      </c>
+      <c r="G75" s="27" t="n"/>
+      <c r="H75" s="27" t="n"/>
+      <c r="I75" s="28" t="n"/>
+      <c r="J75" s="27" t="n"/>
+      <c r="K75" s="27" t="n"/>
+      <c r="L75" s="29" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B76" s="25" t="inlineStr">
+        <is>
+          <t>SPORTKING</t>
+        </is>
+      </c>
+      <c r="C76" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="D76" s="25" t="n"/>
+      <c r="E76" s="26" t="n">
+        <v>94</v>
+      </c>
+      <c r="F76" s="27" t="n">
+        <v>228.19</v>
+      </c>
+      <c r="G76" s="27" t="n"/>
+      <c r="H76" s="27" t="n"/>
+      <c r="I76" s="28" t="n"/>
+      <c r="J76" s="27" t="n"/>
+      <c r="K76" s="27" t="n"/>
+      <c r="L76" s="29" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B77" s="21" t="n"/>
+      <c r="C77" s="21" t="n"/>
+      <c r="D77" s="21" t="n"/>
+      <c r="E77" s="21" t="n"/>
+      <c r="F77" s="21" t="n"/>
+      <c r="G77" s="21" t="n"/>
+      <c r="H77" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L68" s="23" t="n"/>
+      <c r="I77" s="21" t="n"/>
+      <c r="J77" s="21" t="n"/>
+      <c r="K77" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A57:L57"/>
     <mergeCell ref="A30:L30"/>
     <mergeCell ref="A25:L25"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A46:L46"/>
     <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A70:L70"/>
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A39:L39"/>
     <mergeCell ref="A12:L12"/>
@@ -3110,6 +3427,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H72:H76">
+    <cfRule type="dataBar" priority="19">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K72:K76">
+    <cfRule type="dataBar" priority="20">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-04 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2088,7 +2088,7 @@
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-03   ·   5 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-08-03   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹55.96   ·   Net PnL: ₹-248.65</t>
         </is>
       </c>
       <c r="B43" s="3" t="n"/>
@@ -2166,154 +2166,234 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B45" s="25" t="inlineStr">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>DALMIASUG</t>
         </is>
       </c>
-      <c r="C45" s="25" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D45" s="25" t="n"/>
-      <c r="E45" s="26" t="n">
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="n">
         <v>52</v>
       </c>
-      <c r="F45" s="27" t="n">
+      <c r="F45" s="17" t="n">
         <v>407.5</v>
       </c>
-      <c r="G45" s="27" t="n"/>
-      <c r="H45" s="27" t="n"/>
-      <c r="I45" s="28" t="n"/>
-      <c r="J45" s="27" t="n"/>
-      <c r="K45" s="27" t="n"/>
-      <c r="L45" s="29" t="n"/>
+      <c r="G45" s="17" t="n">
+        <v>422.2</v>
+      </c>
+      <c r="H45" s="17" t="n">
+        <v>764.4</v>
+      </c>
+      <c r="I45" s="18" t="n">
+        <v>3.6074</v>
+      </c>
+      <c r="J45" s="17" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="K45" s="17" t="n">
+        <v>701.3</v>
+      </c>
+      <c r="L45" s="19" t="n">
+        <v>3.3096</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B46" s="25" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>DEEPINDS</t>
         </is>
       </c>
-      <c r="C46" s="25" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D46" s="25" t="n"/>
-      <c r="E46" s="26" t="n">
+      <c r="D46" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="F46" s="27" t="n">
+      <c r="F46" s="17" t="n">
         <v>646.15</v>
       </c>
-      <c r="G46" s="27" t="n"/>
-      <c r="H46" s="27" t="n"/>
-      <c r="I46" s="28" t="n"/>
-      <c r="J46" s="27" t="n"/>
-      <c r="K46" s="27" t="n"/>
-      <c r="L46" s="29" t="n"/>
+      <c r="G46" s="17" t="n">
+        <v>649.1378999999999</v>
+      </c>
+      <c r="H46" s="17" t="n">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="I46" s="18" t="n">
+        <v>0.4624</v>
+      </c>
+      <c r="J46" s="17" t="n">
+        <v>62.68</v>
+      </c>
+      <c r="K46" s="17" t="n">
+        <v>35.92</v>
+      </c>
+      <c r="L46" s="19" t="n">
+        <v>0.1685</v>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B47" s="25" t="inlineStr">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="inlineStr">
         <is>
           <t>JINDWORLD</t>
         </is>
       </c>
-      <c r="C47" s="25" t="inlineStr">
+      <c r="C47" s="9" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D47" s="25" t="n"/>
-      <c r="E47" s="26" t="n">
+      <c r="D47" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="n">
         <v>528</v>
       </c>
-      <c r="F47" s="27" t="n">
+      <c r="F47" s="11" t="n">
         <v>40.52</v>
       </c>
-      <c r="G47" s="27" t="n"/>
-      <c r="H47" s="27" t="n"/>
-      <c r="I47" s="28" t="n"/>
-      <c r="J47" s="27" t="n"/>
-      <c r="K47" s="27" t="n"/>
-      <c r="L47" s="29" t="n"/>
+      <c r="G47" s="11" t="n">
+        <v>39.12</v>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>-739.2</v>
+      </c>
+      <c r="I47" s="12" t="n">
+        <v>-3.4551</v>
+      </c>
+      <c r="J47" s="11" t="n">
+        <v>61.96</v>
+      </c>
+      <c r="K47" s="11" t="n">
+        <v>-801.16</v>
+      </c>
+      <c r="L47" s="13" t="n">
+        <v>-3.7447</v>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B48" s="25" t="inlineStr">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
         <is>
           <t>LUMAXIND</t>
         </is>
       </c>
-      <c r="C48" s="25" t="inlineStr">
+      <c r="C48" s="9" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D48" s="25" t="n"/>
-      <c r="E48" s="26" t="n">
+      <c r="D48" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E48" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="F48" s="27" t="n">
+      <c r="F48" s="11" t="n">
         <v>5745.3333</v>
       </c>
-      <c r="G48" s="27" t="n"/>
-      <c r="H48" s="27" t="n"/>
-      <c r="I48" s="28" t="n"/>
-      <c r="J48" s="27" t="n"/>
-      <c r="K48" s="27" t="n"/>
-      <c r="L48" s="29" t="n"/>
+      <c r="G48" s="11" t="n">
+        <v>5710.5</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>-104.5</v>
+      </c>
+      <c r="I48" s="12" t="n">
+        <v>-0.6063</v>
+      </c>
+      <c r="J48" s="11" t="n">
+        <v>53.99</v>
+      </c>
+      <c r="K48" s="11" t="n">
+        <v>-158.49</v>
+      </c>
+      <c r="L48" s="13" t="n">
+        <v>-0.9195</v>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B49" s="25" t="inlineStr">
+      <c r="A49" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>SPORTKING</t>
         </is>
       </c>
-      <c r="C49" s="25" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="D49" s="25" t="n"/>
-      <c r="E49" s="26" t="n">
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="n">
         <v>94</v>
       </c>
-      <c r="F49" s="27" t="n">
+      <c r="F49" s="17" t="n">
         <v>228.19</v>
       </c>
-      <c r="G49" s="27" t="n"/>
-      <c r="H49" s="27" t="n"/>
-      <c r="I49" s="28" t="n"/>
-      <c r="J49" s="27" t="n"/>
-      <c r="K49" s="27" t="n"/>
-      <c r="L49" s="29" t="n"/>
+      <c r="G49" s="17" t="n">
+        <v>228.58</v>
+      </c>
+      <c r="H49" s="17" t="n">
+        <v>36.66</v>
+      </c>
+      <c r="I49" s="18" t="n">
+        <v>0.1709</v>
+      </c>
+      <c r="J49" s="17" t="n">
+        <v>62.88</v>
+      </c>
+      <c r="K49" s="17" t="n">
+        <v>-26.22</v>
+      </c>
+      <c r="L49" s="19" t="n">
+        <v>-0.1222</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="20" t="inlineStr">
@@ -2328,18 +2408,271 @@
       <c r="F50" s="21" t="n"/>
       <c r="G50" s="21" t="n"/>
       <c r="H50" s="22" t="n">
-        <v>0</v>
+        <v>55.96</v>
       </c>
       <c r="I50" s="21" t="n"/>
       <c r="J50" s="21" t="n"/>
       <c r="K50" s="22" t="n">
+        <v>-248.65</v>
+      </c>
+      <c r="L50" s="23" t="n"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-04   ·   5 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="n"/>
+      <c r="C52" s="3" t="n"/>
+      <c r="D52" s="3" t="n"/>
+      <c r="E52" s="3" t="n"/>
+      <c r="F52" s="3" t="n"/>
+      <c r="G52" s="3" t="n"/>
+      <c r="H52" s="3" t="n"/>
+      <c r="I52" s="3" t="n"/>
+      <c r="J52" s="3" t="n"/>
+      <c r="K52" s="3" t="n"/>
+      <c r="L52" s="4" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="J53" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="K53" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="L53" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B54" s="25" t="inlineStr">
+        <is>
+          <t>CAPILLARY</t>
+        </is>
+      </c>
+      <c r="C54" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D54" s="25" t="n"/>
+      <c r="E54" s="26" t="n">
+        <v>93</v>
+      </c>
+      <c r="F54" s="27" t="n">
+        <v>537.7328</v>
+      </c>
+      <c r="G54" s="27" t="n"/>
+      <c r="H54" s="27" t="n"/>
+      <c r="I54" s="28" t="n"/>
+      <c r="J54" s="27" t="n"/>
+      <c r="K54" s="27" t="n"/>
+      <c r="L54" s="29" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B55" s="25" t="inlineStr">
+        <is>
+          <t>EPACKPEB</t>
+        </is>
+      </c>
+      <c r="C55" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D55" s="25" t="n"/>
+      <c r="E55" s="26" t="n">
+        <v>193</v>
+      </c>
+      <c r="F55" s="27" t="n">
+        <v>258.6</v>
+      </c>
+      <c r="G55" s="27" t="n"/>
+      <c r="H55" s="27" t="n"/>
+      <c r="I55" s="28" t="n"/>
+      <c r="J55" s="27" t="n"/>
+      <c r="K55" s="27" t="n"/>
+      <c r="L55" s="29" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B56" s="25" t="inlineStr">
+        <is>
+          <t>KKCL</t>
+        </is>
+      </c>
+      <c r="C56" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D56" s="25" t="n"/>
+      <c r="E56" s="26" t="n">
+        <v>93</v>
+      </c>
+      <c r="F56" s="27" t="n">
+        <v>534.4527</v>
+      </c>
+      <c r="G56" s="27" t="n"/>
+      <c r="H56" s="27" t="n"/>
+      <c r="I56" s="28" t="n"/>
+      <c r="J56" s="27" t="n"/>
+      <c r="K56" s="27" t="n"/>
+      <c r="L56" s="29" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B57" s="25" t="inlineStr">
+        <is>
+          <t>MAHASTEEL</t>
+        </is>
+      </c>
+      <c r="C57" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D57" s="25" t="n"/>
+      <c r="E57" s="26" t="n">
+        <v>23</v>
+      </c>
+      <c r="F57" s="27" t="n">
+        <v>1084</v>
+      </c>
+      <c r="G57" s="27" t="n"/>
+      <c r="H57" s="27" t="n"/>
+      <c r="I57" s="28" t="n"/>
+      <c r="J57" s="27" t="n"/>
+      <c r="K57" s="27" t="n"/>
+      <c r="L57" s="29" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B58" s="25" t="inlineStr">
+        <is>
+          <t>PAUSHAKLTD</t>
+        </is>
+      </c>
+      <c r="C58" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="D58" s="25" t="n"/>
+      <c r="E58" s="26" t="n">
+        <v>67</v>
+      </c>
+      <c r="F58" s="27" t="n">
+        <v>735.75</v>
+      </c>
+      <c r="G58" s="27" t="n"/>
+      <c r="H58" s="27" t="n"/>
+      <c r="I58" s="28" t="n"/>
+      <c r="J58" s="27" t="n"/>
+      <c r="K58" s="27" t="n"/>
+      <c r="L58" s="29" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B59" s="21" t="n"/>
+      <c r="C59" s="21" t="n"/>
+      <c r="D59" s="21" t="n"/>
+      <c r="E59" s="21" t="n"/>
+      <c r="F59" s="21" t="n"/>
+      <c r="G59" s="21" t="n"/>
+      <c r="H59" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L50" s="23" t="n"/>
+      <c r="I59" s="21" t="n"/>
+      <c r="J59" s="21" t="n"/>
+      <c r="K59" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A30:L30"/>
+    <mergeCell ref="A52:L52"/>
     <mergeCell ref="A43:L43"/>
     <mergeCell ref="A19:L19"/>
     <mergeCell ref="A1:L1"/>
@@ -2455,6 +2788,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H54:H58">
+    <cfRule type="dataBar" priority="13">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K54:K58">
+    <cfRule type="dataBar" priority="14">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-05 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2420,7 +2420,7 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-04   ·   5 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,440.35</t>
         </is>
       </c>
       <c r="B52" s="3" t="n"/>
@@ -2498,154 +2498,234 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B54" s="25" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t>CAPILLARY</t>
         </is>
       </c>
-      <c r="C54" s="25" t="inlineStr">
+      <c r="C54" s="15" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D54" s="25" t="n"/>
-      <c r="E54" s="26" t="n">
+      <c r="D54" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="n">
         <v>93</v>
       </c>
-      <c r="F54" s="27" t="n">
+      <c r="F54" s="17" t="n">
         <v>537.7328</v>
       </c>
-      <c r="G54" s="27" t="n"/>
-      <c r="H54" s="27" t="n"/>
-      <c r="I54" s="28" t="n"/>
-      <c r="J54" s="27" t="n"/>
-      <c r="K54" s="27" t="n"/>
-      <c r="L54" s="29" t="n"/>
+      <c r="G54" s="17" t="n">
+        <v>557.0672</v>
+      </c>
+      <c r="H54" s="17" t="n">
+        <v>1798.1</v>
+      </c>
+      <c r="I54" s="18" t="n">
+        <v>3.5955</v>
+      </c>
+      <c r="J54" s="17" t="n">
+        <v>176.16</v>
+      </c>
+      <c r="K54" s="17" t="n">
+        <v>1621.94</v>
+      </c>
+      <c r="L54" s="19" t="n">
+        <v>3.2433</v>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B55" s="25" t="inlineStr">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
         <is>
           <t>EPACKPEB</t>
         </is>
       </c>
-      <c r="C55" s="25" t="inlineStr">
+      <c r="C55" s="15" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D55" s="25" t="n"/>
-      <c r="E55" s="26" t="n">
+      <c r="D55" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="n">
         <v>193</v>
       </c>
-      <c r="F55" s="27" t="n">
+      <c r="F55" s="17" t="n">
         <v>258.6</v>
       </c>
-      <c r="G55" s="27" t="n"/>
-      <c r="H55" s="27" t="n"/>
-      <c r="I55" s="28" t="n"/>
-      <c r="J55" s="27" t="n"/>
-      <c r="K55" s="27" t="n"/>
-      <c r="L55" s="29" t="n"/>
+      <c r="G55" s="17" t="n">
+        <v>264.4503</v>
+      </c>
+      <c r="H55" s="17" t="n">
+        <v>1129.1</v>
+      </c>
+      <c r="I55" s="18" t="n">
+        <v>2.2623</v>
+      </c>
+      <c r="J55" s="17" t="n">
+        <v>174.26</v>
+      </c>
+      <c r="K55" s="17" t="n">
+        <v>954.84</v>
+      </c>
+      <c r="L55" s="19" t="n">
+        <v>1.9131</v>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B56" s="25" t="inlineStr">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B56" s="15" t="inlineStr">
         <is>
           <t>KKCL</t>
         </is>
       </c>
-      <c r="C56" s="25" t="inlineStr">
+      <c r="C56" s="15" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D56" s="25" t="n"/>
-      <c r="E56" s="26" t="n">
+      <c r="D56" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E56" s="16" t="n">
         <v>93</v>
       </c>
-      <c r="F56" s="27" t="n">
+      <c r="F56" s="17" t="n">
         <v>534.4527</v>
       </c>
-      <c r="G56" s="27" t="n"/>
-      <c r="H56" s="27" t="n"/>
-      <c r="I56" s="28" t="n"/>
-      <c r="J56" s="27" t="n"/>
-      <c r="K56" s="27" t="n"/>
-      <c r="L56" s="29" t="n"/>
+      <c r="G56" s="17" t="n">
+        <v>554.5048</v>
+      </c>
+      <c r="H56" s="17" t="n">
+        <v>1864.85</v>
+      </c>
+      <c r="I56" s="18" t="n">
+        <v>3.7519</v>
+      </c>
+      <c r="J56" s="17" t="n">
+        <v>174.6</v>
+      </c>
+      <c r="K56" s="17" t="n">
+        <v>1690.25</v>
+      </c>
+      <c r="L56" s="19" t="n">
+        <v>3.4006</v>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B57" s="25" t="inlineStr">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>MAHASTEEL</t>
         </is>
       </c>
-      <c r="C57" s="25" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D57" s="25" t="n"/>
-      <c r="E57" s="26" t="n">
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E57" s="16" t="n">
         <v>23</v>
       </c>
-      <c r="F57" s="27" t="n">
+      <c r="F57" s="17" t="n">
         <v>1084</v>
       </c>
-      <c r="G57" s="27" t="n"/>
-      <c r="H57" s="27" t="n"/>
-      <c r="I57" s="28" t="n"/>
-      <c r="J57" s="27" t="n"/>
-      <c r="K57" s="27" t="n"/>
-      <c r="L57" s="29" t="n"/>
+      <c r="G57" s="17" t="n">
+        <v>1085.4217</v>
+      </c>
+      <c r="H57" s="17" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="I57" s="18" t="n">
+        <v>0.1312</v>
+      </c>
+      <c r="J57" s="17" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="K57" s="17" t="n">
+        <v>-38.4</v>
+      </c>
+      <c r="L57" s="19" t="n">
+        <v>-0.154</v>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B58" s="25" t="inlineStr">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B58" s="9" t="inlineStr">
         <is>
           <t>PAUSHAKLTD</t>
         </is>
       </c>
-      <c r="C58" s="25" t="inlineStr">
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>2026-08-04</t>
         </is>
       </c>
-      <c r="D58" s="25" t="n"/>
-      <c r="E58" s="26" t="n">
+      <c r="D58" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E58" s="10" t="n">
         <v>67</v>
       </c>
-      <c r="F58" s="27" t="n">
+      <c r="F58" s="11" t="n">
         <v>735.75</v>
       </c>
-      <c r="G58" s="27" t="n"/>
-      <c r="H58" s="27" t="n"/>
-      <c r="I58" s="28" t="n"/>
-      <c r="J58" s="27" t="n"/>
-      <c r="K58" s="27" t="n"/>
-      <c r="L58" s="29" t="n"/>
+      <c r="G58" s="11" t="n">
+        <v>726.5396</v>
+      </c>
+      <c r="H58" s="11" t="n">
+        <v>-617.1</v>
+      </c>
+      <c r="I58" s="12" t="n">
+        <v>-1.2518</v>
+      </c>
+      <c r="J58" s="11" t="n">
+        <v>171.18</v>
+      </c>
+      <c r="K58" s="11" t="n">
+        <v>-788.28</v>
+      </c>
+      <c r="L58" s="13" t="n">
+        <v>-1.5991</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="20" t="inlineStr">
@@ -2660,23 +2740,186 @@
       <c r="F59" s="21" t="n"/>
       <c r="G59" s="21" t="n"/>
       <c r="H59" s="22" t="n">
-        <v>0</v>
+        <v>4207.65</v>
       </c>
       <c r="I59" s="21" t="n"/>
       <c r="J59" s="21" t="n"/>
       <c r="K59" s="22" t="n">
+        <v>3440.35</v>
+      </c>
+      <c r="L59" s="23" t="n"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-05   ·   2 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="n"/>
+      <c r="C61" s="3" t="n"/>
+      <c r="D61" s="3" t="n"/>
+      <c r="E61" s="3" t="n"/>
+      <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
+      <c r="I61" s="3" t="n"/>
+      <c r="J61" s="3" t="n"/>
+      <c r="K61" s="3" t="n"/>
+      <c r="L61" s="4" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F62" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="K62" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B63" s="25" t="inlineStr">
+        <is>
+          <t>JGCHEM</t>
+        </is>
+      </c>
+      <c r="C63" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D63" s="25" t="n"/>
+      <c r="E63" s="26" t="n">
+        <v>137</v>
+      </c>
+      <c r="F63" s="27" t="n">
+        <v>546.2409</v>
+      </c>
+      <c r="G63" s="27" t="n"/>
+      <c r="H63" s="27" t="n"/>
+      <c r="I63" s="28" t="n"/>
+      <c r="J63" s="27" t="n"/>
+      <c r="K63" s="27" t="n"/>
+      <c r="L63" s="29" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B64" s="25" t="inlineStr">
+        <is>
+          <t>UNIPARTS</t>
+        </is>
+      </c>
+      <c r="C64" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="D64" s="25" t="n"/>
+      <c r="E64" s="26" t="n">
+        <v>93</v>
+      </c>
+      <c r="F64" s="27" t="n">
+        <v>805.4892</v>
+      </c>
+      <c r="G64" s="27" t="n"/>
+      <c r="H64" s="27" t="n"/>
+      <c r="I64" s="28" t="n"/>
+      <c r="J64" s="27" t="n"/>
+      <c r="K64" s="27" t="n"/>
+      <c r="L64" s="29" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B65" s="21" t="n"/>
+      <c r="C65" s="21" t="n"/>
+      <c r="D65" s="21" t="n"/>
+      <c r="E65" s="21" t="n"/>
+      <c r="F65" s="21" t="n"/>
+      <c r="G65" s="21" t="n"/>
+      <c r="H65" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L59" s="23" t="n"/>
+      <c r="I65" s="21" t="n"/>
+      <c r="J65" s="21" t="n"/>
+      <c r="K65" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A30:L30"/>
     <mergeCell ref="A52:L52"/>
     <mergeCell ref="A43:L43"/>
     <mergeCell ref="A19:L19"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A35:L35"/>
+    <mergeCell ref="A61:L61"/>
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A12:L12"/>
   </mergeCells>
@@ -2806,6 +3049,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H63:H64">
+    <cfRule type="dataBar" priority="15">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K63:K64">
+    <cfRule type="dataBar" priority="16">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add MTF pledge/unpledge charge to trade book cost analysis
MTF trades incur a flat ₹35.40 pledge+unpledge charge not exposed by any
Kite API (same category as the existing DP_CHARGE). Applied only when
product=="MTF" -- CNC and legacy untagged trades are unaffected.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -2420,7 +2420,7 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,440.35</t>
+          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,298.75</t>
         </is>
       </c>
       <c r="B52" s="3" t="n"/>
@@ -2534,13 +2534,13 @@
         <v>3.5955</v>
       </c>
       <c r="J54" s="17" t="n">
-        <v>176.16</v>
+        <v>211.56</v>
       </c>
       <c r="K54" s="17" t="n">
-        <v>1621.94</v>
+        <v>1586.54</v>
       </c>
       <c r="L54" s="19" t="n">
-        <v>3.2433</v>
+        <v>3.1725</v>
       </c>
     </row>
     <row r="55">
@@ -2580,13 +2580,13 @@
         <v>2.2623</v>
       </c>
       <c r="J55" s="17" t="n">
-        <v>174.26</v>
+        <v>209.66</v>
       </c>
       <c r="K55" s="17" t="n">
-        <v>954.84</v>
+        <v>919.4400000000001</v>
       </c>
       <c r="L55" s="19" t="n">
-        <v>1.9131</v>
+        <v>1.8422</v>
       </c>
     </row>
     <row r="56">
@@ -2626,13 +2626,13 @@
         <v>3.7519</v>
       </c>
       <c r="J56" s="17" t="n">
-        <v>174.6</v>
+        <v>210</v>
       </c>
       <c r="K56" s="17" t="n">
-        <v>1690.25</v>
+        <v>1654.85</v>
       </c>
       <c r="L56" s="19" t="n">
-        <v>3.4006</v>
+        <v>3.3294</v>
       </c>
     </row>
     <row r="57">
@@ -2718,13 +2718,13 @@
         <v>-1.2518</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>171.18</v>
+        <v>206.58</v>
       </c>
       <c r="K58" s="11" t="n">
-        <v>-788.28</v>
+        <v>-823.6799999999999</v>
       </c>
       <c r="L58" s="13" t="n">
-        <v>-1.5991</v>
+        <v>-1.6709</v>
       </c>
     </row>
     <row r="59">
@@ -2745,7 +2745,7 @@
       <c r="I59" s="21" t="n"/>
       <c r="J59" s="21" t="n"/>
       <c r="K59" s="22" t="n">
-        <v>3440.35</v>
+        <v>3298.75</v>
       </c>
       <c r="L59" s="23" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add capital deployed/margin used columns, gross return %, and capital-pool note
- build_trade_book.py: new "Capital Deployed" (shares x entry price, same
  calc for every trade) and "Margin Used" columns (actual cash/margin
  locked up -- for MTF trades this is less than Capital Deployed due to
  leverage, read from mtf_entries_<date>.csv's margin_required by
  entry_order_id; CNC/legacy trades have no leverage so both columns match).
- dashboard/build_dashboard.py + template.html: surface both new columns
  in the Ledger table (after Shares), plus a Gross Return % column (the
  existing Realised PnL Pct field, not previously shown) after Realised.
- template.html: description now leads with the actual capital pools
  (₹1,50,000 CNC / ₹3,00,000 MTF) instead of just the CNC figure, and
  fixes the stale "3:15pm" entry-time mention to 3:21pm.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -640,12 +640,14 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -671,7 +673,9 @@
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="4" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -706,30 +710,40 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
+      <c r="N4" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -763,21 +777,27 @@
         <v>535.4</v>
       </c>
       <c r="G5" s="11" t="n">
+        <v>29982.4</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>29982.4</v>
+      </c>
+      <c r="I5" s="11" t="n">
         <v>515.7</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="J5" s="11" t="n">
         <v>-1103.2</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="K5" s="12" t="n">
         <v>-3.6795</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="L5" s="11" t="n">
         <v>80.40000000000001</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="M5" s="11" t="n">
         <v>-1183.6</v>
       </c>
-      <c r="L5" s="13" t="n">
+      <c r="N5" s="13" t="n">
         <v>-3.9476</v>
       </c>
     </row>
@@ -809,21 +829,27 @@
         <v>517.9</v>
       </c>
       <c r="G6" s="17" t="n">
+        <v>29520.3</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>29520.3</v>
+      </c>
+      <c r="I6" s="17" t="n">
         <v>535.2746</v>
       </c>
-      <c r="H6" s="17" t="n">
+      <c r="J6" s="17" t="n">
         <v>990.35</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="K6" s="18" t="n">
         <v>3.3548</v>
       </c>
-      <c r="J6" s="17" t="n">
+      <c r="L6" s="17" t="n">
         <v>81.62</v>
       </c>
-      <c r="K6" s="17" t="n">
+      <c r="M6" s="17" t="n">
         <v>908.73</v>
       </c>
-      <c r="L6" s="19" t="n">
+      <c r="N6" s="19" t="n">
         <v>3.0783</v>
       </c>
     </row>
@@ -855,21 +881,27 @@
         <v>391.9</v>
       </c>
       <c r="G7" s="17" t="n">
+        <v>29784.4</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>29784.4</v>
+      </c>
+      <c r="I7" s="17" t="n">
         <v>395.5</v>
       </c>
-      <c r="H7" s="17" t="n">
+      <c r="J7" s="17" t="n">
         <v>273.6</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="K7" s="18" t="n">
         <v>0.9186</v>
       </c>
-      <c r="J7" s="17" t="n">
+      <c r="L7" s="17" t="n">
         <v>81.42</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="M7" s="17" t="n">
         <v>192.18</v>
       </c>
-      <c r="L7" s="19" t="n">
+      <c r="N7" s="19" t="n">
         <v>0.6452</v>
       </c>
     </row>
@@ -901,21 +933,27 @@
         <v>238.777</v>
       </c>
       <c r="G8" s="11" t="n">
+        <v>29847.12</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>29847.12</v>
+      </c>
+      <c r="I8" s="11" t="n">
         <v>235.1329</v>
       </c>
-      <c r="H8" s="11" t="n">
+      <c r="J8" s="11" t="n">
         <v>-455.51</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="K8" s="12" t="n">
         <v>-1.5262</v>
       </c>
-      <c r="J8" s="11" t="n">
+      <c r="L8" s="11" t="n">
         <v>80.79000000000001</v>
       </c>
-      <c r="K8" s="11" t="n">
+      <c r="M8" s="11" t="n">
         <v>-536.3</v>
       </c>
-      <c r="L8" s="13" t="n">
+      <c r="N8" s="13" t="n">
         <v>-1.7968</v>
       </c>
     </row>
@@ -947,21 +985,27 @@
         <v>262.6553</v>
       </c>
       <c r="G9" s="11" t="n">
+        <v>29942.7</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>29942.7</v>
+      </c>
+      <c r="I9" s="11" t="n">
         <v>261.8239</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="J9" s="11" t="n">
         <v>-94.77</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="K9" s="12" t="n">
         <v>-0.3165</v>
       </c>
-      <c r="J9" s="11" t="n">
+      <c r="L9" s="11" t="n">
         <v>81.37</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="M9" s="11" t="n">
         <v>-176.14</v>
       </c>
-      <c r="L9" s="13" t="n">
+      <c r="N9" s="13" t="n">
         <v>-0.5883</v>
       </c>
     </row>
@@ -977,15 +1021,17 @@
       <c r="E10" s="21" t="n"/>
       <c r="F10" s="21" t="n"/>
       <c r="G10" s="21" t="n"/>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="21" t="n"/>
+      <c r="I10" s="21" t="n"/>
+      <c r="J10" s="22" t="n">
         <v>-389.53</v>
       </c>
-      <c r="I10" s="21" t="n"/>
-      <c r="J10" s="21" t="n"/>
-      <c r="K10" s="22" t="n">
+      <c r="K10" s="21" t="n"/>
+      <c r="L10" s="21" t="n"/>
+      <c r="M10" s="22" t="n">
         <v>-795.13</v>
       </c>
-      <c r="L10" s="23" t="n"/>
+      <c r="N10" s="23" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -1003,7 +1049,9 @@
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
-      <c r="L12" s="4" t="n"/>
+      <c r="L12" s="3" t="n"/>
+      <c r="M12" s="3" t="n"/>
+      <c r="N12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1038,30 +1086,40 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr">
+      <c r="N13" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -1095,21 +1153,27 @@
         <v>488.1</v>
       </c>
       <c r="G14" s="17" t="n">
+        <v>37095.6</v>
+      </c>
+      <c r="H14" s="17" t="n">
+        <v>37095.6</v>
+      </c>
+      <c r="I14" s="17" t="n">
         <v>492.5289</v>
       </c>
-      <c r="H14" s="17" t="n">
+      <c r="J14" s="17" t="n">
         <v>336.6</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="K14" s="18" t="n">
         <v>0.9074</v>
       </c>
-      <c r="J14" s="17" t="n">
+      <c r="L14" s="17" t="n">
         <v>98.66</v>
       </c>
-      <c r="K14" s="17" t="n">
+      <c r="M14" s="17" t="n">
         <v>237.94</v>
       </c>
-      <c r="L14" s="19" t="n">
+      <c r="N14" s="19" t="n">
         <v>0.6414</v>
       </c>
     </row>
@@ -1141,21 +1205,27 @@
         <v>57.3382</v>
       </c>
       <c r="G15" s="17" t="n">
+        <v>37671.2</v>
+      </c>
+      <c r="H15" s="17" t="n">
+        <v>37671.2</v>
+      </c>
+      <c r="I15" s="17" t="n">
         <v>60.62</v>
       </c>
-      <c r="H15" s="17" t="n">
+      <c r="J15" s="17" t="n">
         <v>2156.14</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="K15" s="18" t="n">
         <v>5.7236</v>
       </c>
-      <c r="J15" s="17" t="n">
+      <c r="L15" s="17" t="n">
         <v>101.74</v>
       </c>
-      <c r="K15" s="17" t="n">
+      <c r="M15" s="17" t="n">
         <v>2054.4</v>
       </c>
-      <c r="L15" s="19" t="n">
+      <c r="N15" s="19" t="n">
         <v>5.4535</v>
       </c>
     </row>
@@ -1187,21 +1257,27 @@
         <v>168.4769</v>
       </c>
       <c r="G16" s="17" t="n">
+        <v>37570.35</v>
+      </c>
+      <c r="H16" s="17" t="n">
+        <v>37570.35</v>
+      </c>
+      <c r="I16" s="17" t="n">
         <v>169.1462</v>
       </c>
-      <c r="H16" s="17" t="n">
+      <c r="J16" s="17" t="n">
         <v>149.26</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="K16" s="18" t="n">
         <v>0.3973</v>
       </c>
-      <c r="J16" s="17" t="n">
+      <c r="L16" s="17" t="n">
         <v>99.45</v>
       </c>
-      <c r="K16" s="17" t="n">
+      <c r="M16" s="17" t="n">
         <v>49.81</v>
       </c>
-      <c r="L16" s="19" t="n">
+      <c r="N16" s="19" t="n">
         <v>0.1326</v>
       </c>
     </row>
@@ -1217,15 +1293,17 @@
       <c r="E17" s="21" t="n"/>
       <c r="F17" s="21" t="n"/>
       <c r="G17" s="21" t="n"/>
-      <c r="H17" s="22" t="n">
+      <c r="H17" s="21" t="n"/>
+      <c r="I17" s="21" t="n"/>
+      <c r="J17" s="22" t="n">
         <v>2642</v>
       </c>
-      <c r="I17" s="21" t="n"/>
-      <c r="J17" s="21" t="n"/>
-      <c r="K17" s="22" t="n">
+      <c r="K17" s="21" t="n"/>
+      <c r="L17" s="21" t="n"/>
+      <c r="M17" s="22" t="n">
         <v>2342.15</v>
       </c>
-      <c r="L17" s="23" t="n"/>
+      <c r="N17" s="23" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
@@ -1243,7 +1321,9 @@
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="3" t="n"/>
-      <c r="L19" s="4" t="n"/>
+      <c r="L19" s="3" t="n"/>
+      <c r="M19" s="3" t="n"/>
+      <c r="N19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1278,30 +1358,40 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="L20" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="M20" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr">
+      <c r="N20" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -1335,21 +1425,27 @@
         <v>683.65</v>
       </c>
       <c r="G21" s="11" t="n">
+        <v>21193.15</v>
+      </c>
+      <c r="H21" s="11" t="n">
+        <v>21193.15</v>
+      </c>
+      <c r="I21" s="11" t="n">
         <v>668.25</v>
       </c>
-      <c r="H21" s="11" t="n">
+      <c r="J21" s="11" t="n">
         <v>-477.4</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="K21" s="12" t="n">
         <v>-2.2526</v>
       </c>
-      <c r="J21" s="11" t="n">
+      <c r="L21" s="11" t="n">
         <v>61.82</v>
       </c>
-      <c r="K21" s="11" t="n">
+      <c r="M21" s="11" t="n">
         <v>-539.22</v>
       </c>
-      <c r="L21" s="13" t="n">
+      <c r="N21" s="13" t="n">
         <v>-2.5443</v>
       </c>
     </row>
@@ -1381,21 +1477,27 @@
         <v>296.9</v>
       </c>
       <c r="G22" s="17" t="n">
+        <v>21376.8</v>
+      </c>
+      <c r="H22" s="17" t="n">
+        <v>21376.8</v>
+      </c>
+      <c r="I22" s="17" t="n">
         <v>301.1042</v>
       </c>
-      <c r="H22" s="17" t="n">
+      <c r="J22" s="17" t="n">
         <v>302.7</v>
       </c>
-      <c r="I22" s="18" t="n">
+      <c r="K22" s="18" t="n">
         <v>1.416</v>
       </c>
-      <c r="J22" s="17" t="n">
+      <c r="L22" s="17" t="n">
         <v>63.01</v>
       </c>
-      <c r="K22" s="17" t="n">
+      <c r="M22" s="17" t="n">
         <v>239.69</v>
       </c>
-      <c r="L22" s="19" t="n">
+      <c r="N22" s="19" t="n">
         <v>1.1213</v>
       </c>
     </row>
@@ -1427,21 +1529,27 @@
         <v>61.59</v>
       </c>
       <c r="G23" s="11" t="n">
+        <v>21371.73</v>
+      </c>
+      <c r="H23" s="11" t="n">
+        <v>21371.73</v>
+      </c>
+      <c r="I23" s="11" t="n">
         <v>61</v>
       </c>
-      <c r="H23" s="11" t="n">
+      <c r="J23" s="11" t="n">
         <v>-204.73</v>
       </c>
-      <c r="I23" s="12" t="n">
+      <c r="K23" s="12" t="n">
         <v>-0.9579</v>
       </c>
-      <c r="J23" s="11" t="n">
+      <c r="L23" s="11" t="n">
         <v>62.47</v>
       </c>
-      <c r="K23" s="11" t="n">
+      <c r="M23" s="11" t="n">
         <v>-267.2</v>
       </c>
-      <c r="L23" s="13" t="n">
+      <c r="N23" s="13" t="n">
         <v>-1.2502</v>
       </c>
     </row>
@@ -1473,21 +1581,27 @@
         <v>543.6769</v>
       </c>
       <c r="G24" s="17" t="n">
+        <v>21203.4</v>
+      </c>
+      <c r="H24" s="17" t="n">
+        <v>21203.4</v>
+      </c>
+      <c r="I24" s="17" t="n">
         <v>571.4</v>
       </c>
-      <c r="H24" s="17" t="n">
+      <c r="J24" s="17" t="n">
         <v>1081.2</v>
       </c>
-      <c r="I24" s="18" t="n">
+      <c r="K24" s="18" t="n">
         <v>5.0992</v>
       </c>
-      <c r="J24" s="17" t="n">
+      <c r="L24" s="17" t="n">
         <v>63.45</v>
       </c>
-      <c r="K24" s="17" t="n">
+      <c r="M24" s="17" t="n">
         <v>1017.75</v>
       </c>
-      <c r="L24" s="19" t="n">
+      <c r="N24" s="19" t="n">
         <v>4.7999</v>
       </c>
     </row>
@@ -1519,21 +1633,27 @@
         <v>4045.4</v>
       </c>
       <c r="G25" s="17" t="n">
+        <v>20227</v>
+      </c>
+      <c r="H25" s="17" t="n">
+        <v>20227</v>
+      </c>
+      <c r="I25" s="17" t="n">
         <v>4050.12</v>
       </c>
-      <c r="H25" s="17" t="n">
+      <c r="J25" s="17" t="n">
         <v>23.6</v>
       </c>
-      <c r="I25" s="18" t="n">
+      <c r="K25" s="18" t="n">
         <v>0.1167</v>
       </c>
-      <c r="J25" s="17" t="n">
+      <c r="L25" s="17" t="n">
         <v>60.33</v>
       </c>
-      <c r="K25" s="17" t="n">
+      <c r="M25" s="17" t="n">
         <v>-36.73</v>
       </c>
-      <c r="L25" s="19" t="n">
+      <c r="N25" s="19" t="n">
         <v>-0.1816</v>
       </c>
     </row>
@@ -1565,21 +1685,27 @@
         <v>162.6454</v>
       </c>
       <c r="G26" s="17" t="n">
+        <v>21306.55</v>
+      </c>
+      <c r="H26" s="17" t="n">
+        <v>21306.55</v>
+      </c>
+      <c r="I26" s="17" t="n">
         <v>168.1477</v>
       </c>
-      <c r="H26" s="17" t="n">
+      <c r="J26" s="17" t="n">
         <v>720.8</v>
       </c>
-      <c r="I26" s="18" t="n">
+      <c r="K26" s="18" t="n">
         <v>3.383</v>
       </c>
-      <c r="J26" s="17" t="n">
+      <c r="L26" s="17" t="n">
         <v>63.29</v>
       </c>
-      <c r="K26" s="17" t="n">
+      <c r="M26" s="17" t="n">
         <v>657.51</v>
       </c>
-      <c r="L26" s="19" t="n">
+      <c r="N26" s="19" t="n">
         <v>3.086</v>
       </c>
     </row>
@@ -1611,21 +1737,27 @@
         <v>259</v>
       </c>
       <c r="G27" s="11" t="n">
+        <v>21497</v>
+      </c>
+      <c r="H27" s="11" t="n">
+        <v>21497</v>
+      </c>
+      <c r="I27" s="11" t="n">
         <v>254.21</v>
       </c>
-      <c r="H27" s="11" t="n">
+      <c r="J27" s="11" t="n">
         <v>-397.57</v>
       </c>
-      <c r="I27" s="12" t="n">
+      <c r="K27" s="12" t="n">
         <v>-1.8494</v>
       </c>
-      <c r="J27" s="11" t="n">
+      <c r="L27" s="11" t="n">
         <v>62.53</v>
       </c>
-      <c r="K27" s="11" t="n">
+      <c r="M27" s="11" t="n">
         <v>-460.1</v>
       </c>
-      <c r="L27" s="13" t="n">
+      <c r="N27" s="13" t="n">
         <v>-2.1403</v>
       </c>
     </row>
@@ -1641,15 +1773,17 @@
       <c r="E28" s="21" t="n"/>
       <c r="F28" s="21" t="n"/>
       <c r="G28" s="21" t="n"/>
-      <c r="H28" s="22" t="n">
+      <c r="H28" s="21" t="n"/>
+      <c r="I28" s="21" t="n"/>
+      <c r="J28" s="22" t="n">
         <v>1048.6</v>
       </c>
-      <c r="I28" s="21" t="n"/>
-      <c r="J28" s="21" t="n"/>
-      <c r="K28" s="22" t="n">
+      <c r="K28" s="21" t="n"/>
+      <c r="L28" s="21" t="n"/>
+      <c r="M28" s="22" t="n">
         <v>611.7</v>
       </c>
-      <c r="L28" s="23" t="n"/>
+      <c r="N28" s="23" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
@@ -1667,7 +1801,9 @@
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="3" t="n"/>
-      <c r="L30" s="4" t="n"/>
+      <c r="L30" s="3" t="n"/>
+      <c r="M30" s="3" t="n"/>
+      <c r="N30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -1702,30 +1838,40 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="J31" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="L31" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K31" s="6" t="inlineStr">
+      <c r="M31" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L31" s="7" t="inlineStr">
+      <c r="N31" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -1759,21 +1905,27 @@
         <v>845.4318</v>
       </c>
       <c r="G32" s="17" t="n">
+        <v>37199</v>
+      </c>
+      <c r="H32" s="17" t="n">
+        <v>37199</v>
+      </c>
+      <c r="I32" s="17" t="n">
         <v>909.3</v>
       </c>
-      <c r="H32" s="17" t="n">
+      <c r="J32" s="17" t="n">
         <v>2810.2</v>
       </c>
-      <c r="I32" s="18" t="n">
+      <c r="K32" s="18" t="n">
         <v>7.5545</v>
       </c>
-      <c r="J32" s="17" t="n">
+      <c r="L32" s="17" t="n">
         <v>101.44</v>
       </c>
-      <c r="K32" s="17" t="n">
+      <c r="M32" s="17" t="n">
         <v>2708.76</v>
       </c>
-      <c r="L32" s="19" t="n">
+      <c r="N32" s="19" t="n">
         <v>7.2818</v>
       </c>
     </row>
@@ -1789,15 +1941,17 @@
       <c r="E33" s="21" t="n"/>
       <c r="F33" s="21" t="n"/>
       <c r="G33" s="21" t="n"/>
-      <c r="H33" s="22" t="n">
+      <c r="H33" s="21" t="n"/>
+      <c r="I33" s="21" t="n"/>
+      <c r="J33" s="22" t="n">
         <v>2810.2</v>
       </c>
-      <c r="I33" s="21" t="n"/>
-      <c r="J33" s="21" t="n"/>
-      <c r="K33" s="22" t="n">
+      <c r="K33" s="21" t="n"/>
+      <c r="L33" s="21" t="n"/>
+      <c r="M33" s="22" t="n">
         <v>2708.76</v>
       </c>
-      <c r="L33" s="23" t="n"/>
+      <c r="N33" s="23" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
@@ -1815,7 +1969,9 @@
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="3" t="n"/>
-      <c r="L35" s="4" t="n"/>
+      <c r="L35" s="3" t="n"/>
+      <c r="M35" s="3" t="n"/>
+      <c r="N35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1850,30 +2006,40 @@
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H36" s="6" t="inlineStr">
+      <c r="J36" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr">
+      <c r="K36" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J36" s="6" t="inlineStr">
+      <c r="L36" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr">
+      <c r="M36" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L36" s="7" t="inlineStr">
+      <c r="N36" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -1907,21 +2073,27 @@
         <v>920.9981</v>
       </c>
       <c r="G37" s="17" t="n">
+        <v>24866.95</v>
+      </c>
+      <c r="H37" s="17" t="n">
+        <v>24866.95</v>
+      </c>
+      <c r="I37" s="17" t="n">
         <v>941.8</v>
       </c>
-      <c r="H37" s="17" t="n">
+      <c r="J37" s="17" t="n">
         <v>561.65</v>
       </c>
-      <c r="I37" s="18" t="n">
+      <c r="K37" s="18" t="n">
         <v>2.2586</v>
       </c>
-      <c r="J37" s="17" t="n">
+      <c r="L37" s="17" t="n">
         <v>71.52</v>
       </c>
-      <c r="K37" s="17" t="n">
+      <c r="M37" s="17" t="n">
         <v>490.13</v>
       </c>
-      <c r="L37" s="19" t="n">
+      <c r="N37" s="19" t="n">
         <v>1.971</v>
       </c>
     </row>
@@ -1953,21 +2125,27 @@
         <v>41.95</v>
       </c>
       <c r="G38" s="11" t="n">
+        <v>24918.3</v>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>24918.3</v>
+      </c>
+      <c r="I38" s="11" t="n">
         <v>41.9</v>
       </c>
-      <c r="H38" s="11" t="n">
+      <c r="J38" s="11" t="n">
         <v>-29.7</v>
       </c>
-      <c r="I38" s="12" t="n">
+      <c r="K38" s="12" t="n">
         <v>-0.1192</v>
       </c>
-      <c r="J38" s="11" t="n">
+      <c r="L38" s="11" t="n">
         <v>71.01000000000001</v>
       </c>
-      <c r="K38" s="11" t="n">
+      <c r="M38" s="11" t="n">
         <v>-100.71</v>
       </c>
-      <c r="L38" s="13" t="n">
+      <c r="N38" s="13" t="n">
         <v>-0.4042</v>
       </c>
     </row>
@@ -1999,21 +2177,27 @@
         <v>2100</v>
       </c>
       <c r="G39" s="17" t="n">
+        <v>23100</v>
+      </c>
+      <c r="H39" s="17" t="n">
+        <v>23100</v>
+      </c>
+      <c r="I39" s="17" t="n">
         <v>2110.0455</v>
       </c>
-      <c r="H39" s="17" t="n">
+      <c r="J39" s="17" t="n">
         <v>110.5</v>
       </c>
-      <c r="I39" s="18" t="n">
+      <c r="K39" s="18" t="n">
         <v>0.4784</v>
       </c>
-      <c r="J39" s="17" t="n">
+      <c r="L39" s="17" t="n">
         <v>66.38</v>
       </c>
-      <c r="K39" s="17" t="n">
+      <c r="M39" s="17" t="n">
         <v>44.12</v>
       </c>
-      <c r="L39" s="19" t="n">
+      <c r="N39" s="19" t="n">
         <v>0.191</v>
       </c>
     </row>
@@ -2045,21 +2229,27 @@
         <v>259.22</v>
       </c>
       <c r="G40" s="11" t="n">
+        <v>24885.12</v>
+      </c>
+      <c r="H40" s="11" t="n">
+        <v>24885.12</v>
+      </c>
+      <c r="I40" s="11" t="n">
         <v>254.6828</v>
       </c>
-      <c r="H40" s="11" t="n">
+      <c r="J40" s="11" t="n">
         <v>-435.57</v>
       </c>
-      <c r="I40" s="12" t="n">
+      <c r="K40" s="12" t="n">
         <v>-1.7503</v>
       </c>
-      <c r="J40" s="11" t="n">
+      <c r="L40" s="11" t="n">
         <v>70.52</v>
       </c>
-      <c r="K40" s="11" t="n">
+      <c r="M40" s="11" t="n">
         <v>-506.09</v>
       </c>
-      <c r="L40" s="13" t="n">
+      <c r="N40" s="13" t="n">
         <v>-2.0337</v>
       </c>
     </row>
@@ -2075,15 +2265,17 @@
       <c r="E41" s="21" t="n"/>
       <c r="F41" s="21" t="n"/>
       <c r="G41" s="21" t="n"/>
-      <c r="H41" s="22" t="n">
+      <c r="H41" s="21" t="n"/>
+      <c r="I41" s="21" t="n"/>
+      <c r="J41" s="22" t="n">
         <v>206.88</v>
       </c>
-      <c r="I41" s="21" t="n"/>
-      <c r="J41" s="21" t="n"/>
-      <c r="K41" s="22" t="n">
+      <c r="K41" s="21" t="n"/>
+      <c r="L41" s="21" t="n"/>
+      <c r="M41" s="22" t="n">
         <v>-72.55</v>
       </c>
-      <c r="L41" s="23" t="n"/>
+      <c r="N41" s="23" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
@@ -2101,7 +2293,9 @@
       <c r="I43" s="3" t="n"/>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="3" t="n"/>
-      <c r="L43" s="4" t="n"/>
+      <c r="L43" s="3" t="n"/>
+      <c r="M43" s="3" t="n"/>
+      <c r="N43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2136,30 +2330,40 @@
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H44" s="6" t="inlineStr">
+      <c r="J44" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
+      <c r="K44" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J44" s="6" t="inlineStr">
+      <c r="L44" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K44" s="6" t="inlineStr">
+      <c r="M44" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L44" s="7" t="inlineStr">
+      <c r="N44" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -2193,21 +2397,27 @@
         <v>407.5</v>
       </c>
       <c r="G45" s="17" t="n">
+        <v>21190</v>
+      </c>
+      <c r="H45" s="17" t="n">
+        <v>21190</v>
+      </c>
+      <c r="I45" s="17" t="n">
         <v>422.2</v>
       </c>
-      <c r="H45" s="17" t="n">
+      <c r="J45" s="17" t="n">
         <v>764.4</v>
       </c>
-      <c r="I45" s="18" t="n">
+      <c r="K45" s="18" t="n">
         <v>3.6074</v>
       </c>
-      <c r="J45" s="17" t="n">
+      <c r="L45" s="17" t="n">
         <v>63.1</v>
       </c>
-      <c r="K45" s="17" t="n">
+      <c r="M45" s="17" t="n">
         <v>701.3</v>
       </c>
-      <c r="L45" s="19" t="n">
+      <c r="N45" s="19" t="n">
         <v>3.3096</v>
       </c>
     </row>
@@ -2239,21 +2449,27 @@
         <v>646.15</v>
       </c>
       <c r="G46" s="17" t="n">
+        <v>21322.95</v>
+      </c>
+      <c r="H46" s="17" t="n">
+        <v>21322.95</v>
+      </c>
+      <c r="I46" s="17" t="n">
         <v>649.1378999999999</v>
       </c>
-      <c r="H46" s="17" t="n">
+      <c r="J46" s="17" t="n">
         <v>98.59999999999999</v>
       </c>
-      <c r="I46" s="18" t="n">
+      <c r="K46" s="18" t="n">
         <v>0.4624</v>
       </c>
-      <c r="J46" s="17" t="n">
+      <c r="L46" s="17" t="n">
         <v>62.68</v>
       </c>
-      <c r="K46" s="17" t="n">
+      <c r="M46" s="17" t="n">
         <v>35.92</v>
       </c>
-      <c r="L46" s="19" t="n">
+      <c r="N46" s="19" t="n">
         <v>0.1685</v>
       </c>
     </row>
@@ -2285,21 +2501,27 @@
         <v>40.52</v>
       </c>
       <c r="G47" s="11" t="n">
+        <v>21394.56</v>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>21394.56</v>
+      </c>
+      <c r="I47" s="11" t="n">
         <v>39.12</v>
       </c>
-      <c r="H47" s="11" t="n">
+      <c r="J47" s="11" t="n">
         <v>-739.2</v>
       </c>
-      <c r="I47" s="12" t="n">
+      <c r="K47" s="12" t="n">
         <v>-3.4551</v>
       </c>
-      <c r="J47" s="11" t="n">
+      <c r="L47" s="11" t="n">
         <v>61.96</v>
       </c>
-      <c r="K47" s="11" t="n">
+      <c r="M47" s="11" t="n">
         <v>-801.16</v>
       </c>
-      <c r="L47" s="13" t="n">
+      <c r="N47" s="13" t="n">
         <v>-3.7447</v>
       </c>
     </row>
@@ -2331,21 +2553,27 @@
         <v>5745.3333</v>
       </c>
       <c r="G48" s="11" t="n">
+        <v>17236</v>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>17236</v>
+      </c>
+      <c r="I48" s="11" t="n">
         <v>5710.5</v>
       </c>
-      <c r="H48" s="11" t="n">
+      <c r="J48" s="11" t="n">
         <v>-104.5</v>
       </c>
-      <c r="I48" s="12" t="n">
+      <c r="K48" s="12" t="n">
         <v>-0.6063</v>
       </c>
-      <c r="J48" s="11" t="n">
+      <c r="L48" s="11" t="n">
         <v>53.99</v>
       </c>
-      <c r="K48" s="11" t="n">
+      <c r="M48" s="11" t="n">
         <v>-158.49</v>
       </c>
-      <c r="L48" s="13" t="n">
+      <c r="N48" s="13" t="n">
         <v>-0.9195</v>
       </c>
     </row>
@@ -2377,21 +2605,27 @@
         <v>228.19</v>
       </c>
       <c r="G49" s="17" t="n">
+        <v>21449.86</v>
+      </c>
+      <c r="H49" s="17" t="n">
+        <v>21449.86</v>
+      </c>
+      <c r="I49" s="17" t="n">
         <v>228.58</v>
       </c>
-      <c r="H49" s="17" t="n">
+      <c r="J49" s="17" t="n">
         <v>36.66</v>
       </c>
-      <c r="I49" s="18" t="n">
+      <c r="K49" s="18" t="n">
         <v>0.1709</v>
       </c>
-      <c r="J49" s="17" t="n">
+      <c r="L49" s="17" t="n">
         <v>62.88</v>
       </c>
-      <c r="K49" s="17" t="n">
+      <c r="M49" s="17" t="n">
         <v>-26.22</v>
       </c>
-      <c r="L49" s="19" t="n">
+      <c r="N49" s="19" t="n">
         <v>-0.1222</v>
       </c>
     </row>
@@ -2407,15 +2641,17 @@
       <c r="E50" s="21" t="n"/>
       <c r="F50" s="21" t="n"/>
       <c r="G50" s="21" t="n"/>
-      <c r="H50" s="22" t="n">
+      <c r="H50" s="21" t="n"/>
+      <c r="I50" s="21" t="n"/>
+      <c r="J50" s="22" t="n">
         <v>55.96</v>
       </c>
-      <c r="I50" s="21" t="n"/>
-      <c r="J50" s="21" t="n"/>
-      <c r="K50" s="22" t="n">
+      <c r="K50" s="21" t="n"/>
+      <c r="L50" s="21" t="n"/>
+      <c r="M50" s="22" t="n">
         <v>-248.65</v>
       </c>
-      <c r="L50" s="23" t="n"/>
+      <c r="N50" s="23" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
@@ -2433,7 +2669,9 @@
       <c r="I52" s="3" t="n"/>
       <c r="J52" s="3" t="n"/>
       <c r="K52" s="3" t="n"/>
-      <c r="L52" s="4" t="n"/>
+      <c r="L52" s="3" t="n"/>
+      <c r="M52" s="3" t="n"/>
+      <c r="N52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -2468,30 +2706,40 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="J53" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
+      <c r="K53" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J53" s="6" t="inlineStr">
+      <c r="L53" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K53" s="6" t="inlineStr">
+      <c r="M53" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L53" s="7" t="inlineStr">
+      <c r="N53" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -2525,21 +2773,27 @@
         <v>537.7328</v>
       </c>
       <c r="G54" s="17" t="n">
+        <v>50009.15</v>
+      </c>
+      <c r="H54" s="17" t="n">
+        <v>15368.3</v>
+      </c>
+      <c r="I54" s="17" t="n">
         <v>557.0672</v>
       </c>
-      <c r="H54" s="17" t="n">
+      <c r="J54" s="17" t="n">
         <v>1798.1</v>
       </c>
-      <c r="I54" s="18" t="n">
+      <c r="K54" s="18" t="n">
         <v>3.5955</v>
       </c>
-      <c r="J54" s="17" t="n">
+      <c r="L54" s="17" t="n">
         <v>211.56</v>
       </c>
-      <c r="K54" s="17" t="n">
+      <c r="M54" s="17" t="n">
         <v>1586.54</v>
       </c>
-      <c r="L54" s="19" t="n">
+      <c r="N54" s="19" t="n">
         <v>3.1725</v>
       </c>
     </row>
@@ -2571,21 +2825,27 @@
         <v>258.6</v>
       </c>
       <c r="G55" s="17" t="n">
+        <v>49909.8</v>
+      </c>
+      <c r="H55" s="17" t="n">
+        <v>24945.25</v>
+      </c>
+      <c r="I55" s="17" t="n">
         <v>264.4503</v>
       </c>
-      <c r="H55" s="17" t="n">
+      <c r="J55" s="17" t="n">
         <v>1129.1</v>
       </c>
-      <c r="I55" s="18" t="n">
+      <c r="K55" s="18" t="n">
         <v>2.2623</v>
       </c>
-      <c r="J55" s="17" t="n">
+      <c r="L55" s="17" t="n">
         <v>209.66</v>
       </c>
-      <c r="K55" s="17" t="n">
+      <c r="M55" s="17" t="n">
         <v>919.4400000000001</v>
       </c>
-      <c r="L55" s="19" t="n">
+      <c r="N55" s="19" t="n">
         <v>1.8422</v>
       </c>
     </row>
@@ -2617,21 +2877,27 @@
         <v>534.4527</v>
       </c>
       <c r="G56" s="17" t="n">
+        <v>49704.1</v>
+      </c>
+      <c r="H56" s="17" t="n">
+        <v>24868.2</v>
+      </c>
+      <c r="I56" s="17" t="n">
         <v>554.5048</v>
       </c>
-      <c r="H56" s="17" t="n">
+      <c r="J56" s="17" t="n">
         <v>1864.85</v>
       </c>
-      <c r="I56" s="18" t="n">
+      <c r="K56" s="18" t="n">
         <v>3.7519</v>
       </c>
-      <c r="J56" s="17" t="n">
+      <c r="L56" s="17" t="n">
         <v>210</v>
       </c>
-      <c r="K56" s="17" t="n">
+      <c r="M56" s="17" t="n">
         <v>1654.85</v>
       </c>
-      <c r="L56" s="19" t="n">
+      <c r="N56" s="19" t="n">
         <v>3.3294</v>
       </c>
     </row>
@@ -2663,21 +2929,27 @@
         <v>1084</v>
       </c>
       <c r="G57" s="17" t="n">
+        <v>24932</v>
+      </c>
+      <c r="H57" s="17" t="n">
+        <v>24932</v>
+      </c>
+      <c r="I57" s="17" t="n">
         <v>1085.4217</v>
       </c>
-      <c r="H57" s="17" t="n">
+      <c r="J57" s="17" t="n">
         <v>32.7</v>
       </c>
-      <c r="I57" s="18" t="n">
+      <c r="K57" s="18" t="n">
         <v>0.1312</v>
       </c>
-      <c r="J57" s="17" t="n">
+      <c r="L57" s="17" t="n">
         <v>71.09999999999999</v>
       </c>
-      <c r="K57" s="17" t="n">
+      <c r="M57" s="17" t="n">
         <v>-38.4</v>
       </c>
-      <c r="L57" s="19" t="n">
+      <c r="N57" s="19" t="n">
         <v>-0.154</v>
       </c>
     </row>
@@ -2709,21 +2981,27 @@
         <v>735.75</v>
       </c>
       <c r="G58" s="11" t="n">
+        <v>49295.25</v>
+      </c>
+      <c r="H58" s="11" t="n">
+        <v>24647.62</v>
+      </c>
+      <c r="I58" s="11" t="n">
         <v>726.5396</v>
       </c>
-      <c r="H58" s="11" t="n">
+      <c r="J58" s="11" t="n">
         <v>-617.1</v>
       </c>
-      <c r="I58" s="12" t="n">
+      <c r="K58" s="12" t="n">
         <v>-1.2518</v>
       </c>
-      <c r="J58" s="11" t="n">
+      <c r="L58" s="11" t="n">
         <v>206.58</v>
       </c>
-      <c r="K58" s="11" t="n">
+      <c r="M58" s="11" t="n">
         <v>-823.6799999999999</v>
       </c>
-      <c r="L58" s="13" t="n">
+      <c r="N58" s="13" t="n">
         <v>-1.6709</v>
       </c>
     </row>
@@ -2739,15 +3017,17 @@
       <c r="E59" s="21" t="n"/>
       <c r="F59" s="21" t="n"/>
       <c r="G59" s="21" t="n"/>
-      <c r="H59" s="22" t="n">
+      <c r="H59" s="21" t="n"/>
+      <c r="I59" s="21" t="n"/>
+      <c r="J59" s="22" t="n">
         <v>4207.65</v>
       </c>
-      <c r="I59" s="21" t="n"/>
-      <c r="J59" s="21" t="n"/>
-      <c r="K59" s="22" t="n">
+      <c r="K59" s="21" t="n"/>
+      <c r="L59" s="21" t="n"/>
+      <c r="M59" s="22" t="n">
         <v>3298.75</v>
       </c>
-      <c r="L59" s="23" t="n"/>
+      <c r="N59" s="23" t="n"/>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
@@ -2765,7 +3045,9 @@
       <c r="I61" s="3" t="n"/>
       <c r="J61" s="3" t="n"/>
       <c r="K61" s="3" t="n"/>
-      <c r="L61" s="4" t="n"/>
+      <c r="L61" s="3" t="n"/>
+      <c r="M61" s="3" t="n"/>
+      <c r="N61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -2800,30 +3082,40 @@
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
           <t>Exit Price</t>
         </is>
       </c>
-      <c r="H62" s="6" t="inlineStr">
+      <c r="J62" s="6" t="inlineStr">
         <is>
           <t>Realised PnL</t>
         </is>
       </c>
-      <c r="I62" s="6" t="inlineStr">
+      <c r="K62" s="6" t="inlineStr">
         <is>
           <t>Realised PnL Pct</t>
         </is>
       </c>
-      <c r="J62" s="6" t="inlineStr">
+      <c r="L62" s="6" t="inlineStr">
         <is>
           <t>Total Charges</t>
         </is>
       </c>
-      <c r="K62" s="6" t="inlineStr">
+      <c r="M62" s="6" t="inlineStr">
         <is>
           <t>Net PnL</t>
         </is>
       </c>
-      <c r="L62" s="7" t="inlineStr">
+      <c r="N62" s="7" t="inlineStr">
         <is>
           <t>Net PnL Pct</t>
         </is>
@@ -2852,12 +3144,18 @@
       <c r="F63" s="27" t="n">
         <v>546.2409</v>
       </c>
-      <c r="G63" s="27" t="n"/>
-      <c r="H63" s="27" t="n"/>
-      <c r="I63" s="28" t="n"/>
+      <c r="G63" s="27" t="n">
+        <v>74835</v>
+      </c>
+      <c r="H63" s="27" t="n">
+        <v>26916.04</v>
+      </c>
+      <c r="I63" s="27" t="n"/>
       <c r="J63" s="27" t="n"/>
-      <c r="K63" s="27" t="n"/>
-      <c r="L63" s="29" t="n"/>
+      <c r="K63" s="28" t="n"/>
+      <c r="L63" s="27" t="n"/>
+      <c r="M63" s="27" t="n"/>
+      <c r="N63" s="29" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="24" t="inlineStr">
@@ -2882,12 +3180,18 @@
       <c r="F64" s="27" t="n">
         <v>805.4892</v>
       </c>
-      <c r="G64" s="27" t="n"/>
-      <c r="H64" s="27" t="n"/>
-      <c r="I64" s="28" t="n"/>
+      <c r="G64" s="27" t="n">
+        <v>74910.5</v>
+      </c>
+      <c r="H64" s="27" t="n">
+        <v>24438.87</v>
+      </c>
+      <c r="I64" s="27" t="n"/>
       <c r="J64" s="27" t="n"/>
-      <c r="K64" s="27" t="n"/>
-      <c r="L64" s="29" t="n"/>
+      <c r="K64" s="28" t="n"/>
+      <c r="L64" s="27" t="n"/>
+      <c r="M64" s="27" t="n"/>
+      <c r="N64" s="29" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="20" t="inlineStr">
@@ -2901,29 +3205,31 @@
       <c r="E65" s="21" t="n"/>
       <c r="F65" s="21" t="n"/>
       <c r="G65" s="21" t="n"/>
-      <c r="H65" s="22" t="n">
+      <c r="H65" s="21" t="n"/>
+      <c r="I65" s="21" t="n"/>
+      <c r="J65" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="I65" s="21" t="n"/>
-      <c r="J65" s="21" t="n"/>
-      <c r="K65" s="22" t="n">
+      <c r="K65" s="21" t="n"/>
+      <c r="L65" s="21" t="n"/>
+      <c r="M65" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L65" s="23" t="n"/>
+      <c r="N65" s="23" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A30:L30"/>
-    <mergeCell ref="A52:L52"/>
-    <mergeCell ref="A43:L43"/>
-    <mergeCell ref="A19:L19"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A35:L35"/>
-    <mergeCell ref="A61:L61"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A12:L12"/>
+    <mergeCell ref="A3:N3"/>
+    <mergeCell ref="A61:N61"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A35:N35"/>
+    <mergeCell ref="A30:N30"/>
+    <mergeCell ref="A52:N52"/>
+    <mergeCell ref="A43:N43"/>
+    <mergeCell ref="A19:N19"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H9">
+  <conditionalFormatting sqref="J5:J9">
     <cfRule type="dataBar" priority="1">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2932,7 +3238,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K9">
+  <conditionalFormatting sqref="M5:M9">
     <cfRule type="dataBar" priority="2">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2941,7 +3247,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H14:H16">
+  <conditionalFormatting sqref="J14:J16">
     <cfRule type="dataBar" priority="3">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2950,7 +3256,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K14:K16">
+  <conditionalFormatting sqref="M14:M16">
     <cfRule type="dataBar" priority="4">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2959,7 +3265,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H21:H27">
+  <conditionalFormatting sqref="J21:J27">
     <cfRule type="dataBar" priority="5">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2968,7 +3274,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K21:K27">
+  <conditionalFormatting sqref="M21:M27">
     <cfRule type="dataBar" priority="6">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2977,7 +3283,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H32">
+  <conditionalFormatting sqref="J32">
     <cfRule type="dataBar" priority="7">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2986,7 +3292,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K32">
+  <conditionalFormatting sqref="M32">
     <cfRule type="dataBar" priority="8">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -2995,7 +3301,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H37:H40">
+  <conditionalFormatting sqref="J37:J40">
     <cfRule type="dataBar" priority="9">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3004,7 +3310,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K37:K40">
+  <conditionalFormatting sqref="M37:M40">
     <cfRule type="dataBar" priority="10">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3013,7 +3319,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H45:H49">
+  <conditionalFormatting sqref="J45:J49">
     <cfRule type="dataBar" priority="11">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3022,7 +3328,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K45:K49">
+  <conditionalFormatting sqref="M45:M49">
     <cfRule type="dataBar" priority="12">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3031,7 +3337,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H54:H58">
+  <conditionalFormatting sqref="J54:J58">
     <cfRule type="dataBar" priority="13">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3040,7 +3346,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K54:K58">
+  <conditionalFormatting sqref="M54:M58">
     <cfRule type="dataBar" priority="14">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3049,7 +3355,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H63:H64">
+  <conditionalFormatting sqref="J63:J64">
     <cfRule type="dataBar" priority="15">
       <dataBar showValue="1">
         <cfvo type="min"/>
@@ -3058,7 +3364,7 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K63:K64">
+  <conditionalFormatting sqref="M63:M64">
     <cfRule type="dataBar" priority="16">
       <dataBar showValue="1">
         <cfvo type="min"/>

</xml_diff>

<commit_message>
Data update — 2026-08-06 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3032,7 +3032,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-05   ·   2 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-08-05   ·   2 trade(s), 2 closed   ·   Gross PnL: ₹322.90   ·   Net PnL: ₹-206.00</t>
         </is>
       </c>
       <c r="B61" s="3" t="n"/>
@@ -3122,76 +3122,108 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B63" s="25" t="inlineStr">
+      <c r="A63" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
         <is>
           <t>JGCHEM</t>
         </is>
       </c>
-      <c r="C63" s="25" t="inlineStr">
+      <c r="C63" s="15" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="D63" s="25" t="n"/>
-      <c r="E63" s="26" t="n">
+      <c r="D63" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="n">
         <v>137</v>
       </c>
-      <c r="F63" s="27" t="n">
+      <c r="F63" s="17" t="n">
         <v>546.2409</v>
       </c>
-      <c r="G63" s="27" t="n">
+      <c r="G63" s="17" t="n">
         <v>74835</v>
       </c>
-      <c r="H63" s="27" t="n">
+      <c r="H63" s="17" t="n">
         <v>26916.04</v>
       </c>
-      <c r="I63" s="27" t="n"/>
-      <c r="J63" s="27" t="n"/>
-      <c r="K63" s="28" t="n"/>
-      <c r="L63" s="27" t="n"/>
-      <c r="M63" s="27" t="n"/>
-      <c r="N63" s="29" t="n"/>
+      <c r="I63" s="17" t="n">
+        <v>548.3938000000001</v>
+      </c>
+      <c r="J63" s="17" t="n">
+        <v>294.95</v>
+      </c>
+      <c r="K63" s="18" t="n">
+        <v>0.3941</v>
+      </c>
+      <c r="L63" s="17" t="n">
+        <v>264.51</v>
+      </c>
+      <c r="M63" s="17" t="n">
+        <v>30.44</v>
+      </c>
+      <c r="N63" s="19" t="n">
+        <v>0.0407</v>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B64" s="25" t="inlineStr">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t>UNIPARTS</t>
         </is>
       </c>
-      <c r="C64" s="25" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="D64" s="25" t="n"/>
-      <c r="E64" s="26" t="n">
+      <c r="D64" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="n">
         <v>93</v>
       </c>
-      <c r="F64" s="27" t="n">
+      <c r="F64" s="17" t="n">
         <v>805.4892</v>
       </c>
-      <c r="G64" s="27" t="n">
+      <c r="G64" s="17" t="n">
         <v>74910.5</v>
       </c>
-      <c r="H64" s="27" t="n">
+      <c r="H64" s="17" t="n">
         <v>24438.87</v>
       </c>
-      <c r="I64" s="27" t="n"/>
-      <c r="J64" s="27" t="n"/>
-      <c r="K64" s="28" t="n"/>
-      <c r="L64" s="27" t="n"/>
-      <c r="M64" s="27" t="n"/>
-      <c r="N64" s="29" t="n"/>
+      <c r="I64" s="17" t="n">
+        <v>805.7898</v>
+      </c>
+      <c r="J64" s="17" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="K64" s="18" t="n">
+        <v>0.0373</v>
+      </c>
+      <c r="L64" s="17" t="n">
+        <v>264.39</v>
+      </c>
+      <c r="M64" s="17" t="n">
+        <v>-236.44</v>
+      </c>
+      <c r="N64" s="19" t="n">
+        <v>-0.3156</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="20" t="inlineStr">
@@ -3208,17 +3240,386 @@
       <c r="H65" s="21" t="n"/>
       <c r="I65" s="21" t="n"/>
       <c r="J65" s="22" t="n">
-        <v>0</v>
+        <v>322.9</v>
       </c>
       <c r="K65" s="21" t="n"/>
       <c r="L65" s="21" t="n"/>
       <c r="M65" s="22" t="n">
+        <v>-206</v>
+      </c>
+      <c r="N65" s="23" t="n"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-06   ·   7 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="n"/>
+      <c r="C67" s="3" t="n"/>
+      <c r="D67" s="3" t="n"/>
+      <c r="E67" s="3" t="n"/>
+      <c r="F67" s="3" t="n"/>
+      <c r="G67" s="3" t="n"/>
+      <c r="H67" s="3" t="n"/>
+      <c r="I67" s="3" t="n"/>
+      <c r="J67" s="3" t="n"/>
+      <c r="K67" s="3" t="n"/>
+      <c r="L67" s="3" t="n"/>
+      <c r="M67" s="3" t="n"/>
+      <c r="N67" s="4" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F68" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="K68" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="L68" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="M68" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="N68" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B69" s="25" t="inlineStr">
+        <is>
+          <t>BAJAJELEC</t>
+        </is>
+      </c>
+      <c r="C69" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D69" s="25" t="n"/>
+      <c r="E69" s="26" t="n">
+        <v>111</v>
+      </c>
+      <c r="F69" s="27" t="n">
+        <v>385.55</v>
+      </c>
+      <c r="G69" s="27" t="n">
+        <v>42796.05</v>
+      </c>
+      <c r="H69" s="27" t="n">
+        <v>12820.99</v>
+      </c>
+      <c r="I69" s="27" t="n"/>
+      <c r="J69" s="27" t="n"/>
+      <c r="K69" s="28" t="n"/>
+      <c r="L69" s="27" t="n"/>
+      <c r="M69" s="27" t="n"/>
+      <c r="N69" s="29" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B70" s="25" t="inlineStr">
+        <is>
+          <t>DECNGOLD</t>
+        </is>
+      </c>
+      <c r="C70" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D70" s="25" t="n"/>
+      <c r="E70" s="26" t="n">
+        <v>190</v>
+      </c>
+      <c r="F70" s="27" t="n">
+        <v>225.1953</v>
+      </c>
+      <c r="G70" s="27" t="n">
+        <v>42787.11</v>
+      </c>
+      <c r="H70" s="27" t="n">
+        <v>19254.6</v>
+      </c>
+      <c r="I70" s="27" t="n"/>
+      <c r="J70" s="27" t="n"/>
+      <c r="K70" s="28" t="n"/>
+      <c r="L70" s="27" t="n"/>
+      <c r="M70" s="27" t="n"/>
+      <c r="N70" s="29" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B71" s="25" t="inlineStr">
+        <is>
+          <t>GMMPFAUDLR</t>
+        </is>
+      </c>
+      <c r="C71" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D71" s="25" t="n"/>
+      <c r="E71" s="26" t="n">
+        <v>43</v>
+      </c>
+      <c r="F71" s="27" t="n">
+        <v>978.7314</v>
+      </c>
+      <c r="G71" s="27" t="n">
+        <v>42085.45</v>
+      </c>
+      <c r="H71" s="27" t="n">
+        <v>12359.47</v>
+      </c>
+      <c r="I71" s="27" t="n"/>
+      <c r="J71" s="27" t="n"/>
+      <c r="K71" s="28" t="n"/>
+      <c r="L71" s="27" t="n"/>
+      <c r="M71" s="27" t="n"/>
+      <c r="N71" s="29" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B72" s="25" t="inlineStr">
+        <is>
+          <t>KOLTEPATIL</t>
+        </is>
+      </c>
+      <c r="C72" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D72" s="25" t="n"/>
+      <c r="E72" s="26" t="n">
+        <v>99</v>
+      </c>
+      <c r="F72" s="27" t="n">
+        <v>429.4303</v>
+      </c>
+      <c r="G72" s="27" t="n">
+        <v>42513.6</v>
+      </c>
+      <c r="H72" s="27" t="n">
+        <v>13178.29</v>
+      </c>
+      <c r="I72" s="27" t="n"/>
+      <c r="J72" s="27" t="n"/>
+      <c r="K72" s="28" t="n"/>
+      <c r="L72" s="27" t="n"/>
+      <c r="M72" s="27" t="n"/>
+      <c r="N72" s="29" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B73" s="25" t="inlineStr">
+        <is>
+          <t>ROLEXRINGS</t>
+        </is>
+      </c>
+      <c r="C73" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D73" s="25" t="n"/>
+      <c r="E73" s="26" t="n">
+        <v>279</v>
+      </c>
+      <c r="F73" s="27" t="n">
+        <v>153.48</v>
+      </c>
+      <c r="G73" s="27" t="n">
+        <v>42820.92</v>
+      </c>
+      <c r="H73" s="27" t="n">
+        <v>14390.24</v>
+      </c>
+      <c r="I73" s="27" t="n"/>
+      <c r="J73" s="27" t="n"/>
+      <c r="K73" s="28" t="n"/>
+      <c r="L73" s="27" t="n"/>
+      <c r="M73" s="27" t="n"/>
+      <c r="N73" s="29" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B74" s="25" t="inlineStr">
+        <is>
+          <t>SOTL</t>
+        </is>
+      </c>
+      <c r="C74" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D74" s="25" t="n"/>
+      <c r="E74" s="26" t="n">
+        <v>55</v>
+      </c>
+      <c r="F74" s="27" t="n">
+        <v>776.25</v>
+      </c>
+      <c r="G74" s="27" t="n">
+        <v>42693.75</v>
+      </c>
+      <c r="H74" s="27" t="n">
+        <v>15466.24</v>
+      </c>
+      <c r="I74" s="27" t="n"/>
+      <c r="J74" s="27" t="n"/>
+      <c r="K74" s="28" t="n"/>
+      <c r="L74" s="27" t="n"/>
+      <c r="M74" s="27" t="n"/>
+      <c r="N74" s="29" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B75" s="25" t="inlineStr">
+        <is>
+          <t>STOVEKRAFT</t>
+        </is>
+      </c>
+      <c r="C75" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="D75" s="25" t="n"/>
+      <c r="E75" s="26" t="n">
+        <v>53</v>
+      </c>
+      <c r="F75" s="27" t="n">
+        <v>798.9</v>
+      </c>
+      <c r="G75" s="27" t="n">
+        <v>42341.7</v>
+      </c>
+      <c r="H75" s="27" t="n">
+        <v>14986.57</v>
+      </c>
+      <c r="I75" s="27" t="n"/>
+      <c r="J75" s="27" t="n"/>
+      <c r="K75" s="28" t="n"/>
+      <c r="L75" s="27" t="n"/>
+      <c r="M75" s="27" t="n"/>
+      <c r="N75" s="29" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B76" s="21" t="n"/>
+      <c r="C76" s="21" t="n"/>
+      <c r="D76" s="21" t="n"/>
+      <c r="E76" s="21" t="n"/>
+      <c r="F76" s="21" t="n"/>
+      <c r="G76" s="21" t="n"/>
+      <c r="H76" s="21" t="n"/>
+      <c r="I76" s="21" t="n"/>
+      <c r="J76" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="N65" s="23" t="n"/>
+      <c r="K76" s="21" t="n"/>
+      <c r="L76" s="21" t="n"/>
+      <c r="M76" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="A67:N67"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A61:N61"/>
     <mergeCell ref="A12:N12"/>
@@ -3373,6 +3774,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J69:J75">
+    <cfRule type="dataBar" priority="17">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M69:M75">
+    <cfRule type="dataBar" priority="18">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-07 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3252,7 +3252,7 @@
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-06   ·   7 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-08-06   ·   7 trade(s), 7 closed   ·   Gross PnL: ₹2,202.67   ·   Net PnL: ₹854.42</t>
         </is>
       </c>
       <c r="B67" s="3" t="n"/>
@@ -3342,256 +3342,368 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B69" s="25" t="inlineStr">
+      <c r="A69" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
         <is>
           <t>BAJAJELEC</t>
         </is>
       </c>
-      <c r="C69" s="25" t="inlineStr">
+      <c r="C69" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D69" s="25" t="n"/>
-      <c r="E69" s="26" t="n">
+      <c r="D69" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E69" s="16" t="n">
         <v>111</v>
       </c>
-      <c r="F69" s="27" t="n">
+      <c r="F69" s="17" t="n">
         <v>385.55</v>
       </c>
-      <c r="G69" s="27" t="n">
+      <c r="G69" s="17" t="n">
         <v>42796.05</v>
       </c>
-      <c r="H69" s="27" t="n">
+      <c r="H69" s="17" t="n">
         <v>12820.99</v>
       </c>
-      <c r="I69" s="27" t="n"/>
-      <c r="J69" s="27" t="n"/>
-      <c r="K69" s="28" t="n"/>
-      <c r="L69" s="27" t="n"/>
-      <c r="M69" s="27" t="n"/>
-      <c r="N69" s="29" t="n"/>
+      <c r="I69" s="17" t="n">
+        <v>388.1</v>
+      </c>
+      <c r="J69" s="17" t="n">
+        <v>283.05</v>
+      </c>
+      <c r="K69" s="18" t="n">
+        <v>0.6614</v>
+      </c>
+      <c r="L69" s="17" t="n">
+        <v>193.03</v>
+      </c>
+      <c r="M69" s="17" t="n">
+        <v>90.02</v>
+      </c>
+      <c r="N69" s="19" t="n">
+        <v>0.2103</v>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B70" s="25" t="inlineStr">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="inlineStr">
         <is>
           <t>DECNGOLD</t>
         </is>
       </c>
-      <c r="C70" s="25" t="inlineStr">
+      <c r="C70" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D70" s="25" t="n"/>
-      <c r="E70" s="26" t="n">
+      <c r="D70" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E70" s="16" t="n">
         <v>190</v>
       </c>
-      <c r="F70" s="27" t="n">
+      <c r="F70" s="17" t="n">
         <v>225.1953</v>
       </c>
-      <c r="G70" s="27" t="n">
+      <c r="G70" s="17" t="n">
         <v>42787.11</v>
       </c>
-      <c r="H70" s="27" t="n">
+      <c r="H70" s="17" t="n">
         <v>19254.6</v>
       </c>
-      <c r="I70" s="27" t="n"/>
-      <c r="J70" s="27" t="n"/>
-      <c r="K70" s="28" t="n"/>
-      <c r="L70" s="27" t="n"/>
-      <c r="M70" s="27" t="n"/>
-      <c r="N70" s="29" t="n"/>
+      <c r="I70" s="17" t="n">
+        <v>228.9489</v>
+      </c>
+      <c r="J70" s="17" t="n">
+        <v>713.1900000000001</v>
+      </c>
+      <c r="K70" s="18" t="n">
+        <v>1.6668</v>
+      </c>
+      <c r="L70" s="17" t="n">
+        <v>193.46</v>
+      </c>
+      <c r="M70" s="17" t="n">
+        <v>519.73</v>
+      </c>
+      <c r="N70" s="19" t="n">
+        <v>1.2147</v>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B71" s="25" t="inlineStr">
+      <c r="A71" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>GMMPFAUDLR</t>
         </is>
       </c>
-      <c r="C71" s="25" t="inlineStr">
+      <c r="C71" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D71" s="25" t="n"/>
-      <c r="E71" s="26" t="n">
+      <c r="D71" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E71" s="16" t="n">
         <v>43</v>
       </c>
-      <c r="F71" s="27" t="n">
+      <c r="F71" s="17" t="n">
         <v>978.7314</v>
       </c>
-      <c r="G71" s="27" t="n">
+      <c r="G71" s="17" t="n">
         <v>42085.45</v>
       </c>
-      <c r="H71" s="27" t="n">
+      <c r="H71" s="17" t="n">
         <v>12359.47</v>
       </c>
-      <c r="I71" s="27" t="n"/>
-      <c r="J71" s="27" t="n"/>
-      <c r="K71" s="28" t="n"/>
-      <c r="L71" s="27" t="n"/>
-      <c r="M71" s="27" t="n"/>
-      <c r="N71" s="29" t="n"/>
+      <c r="I71" s="17" t="n">
+        <v>980.5</v>
+      </c>
+      <c r="J71" s="17" t="n">
+        <v>76.05</v>
+      </c>
+      <c r="K71" s="18" t="n">
+        <v>0.1807</v>
+      </c>
+      <c r="L71" s="17" t="n">
+        <v>191.34</v>
+      </c>
+      <c r="M71" s="17" t="n">
+        <v>-115.29</v>
+      </c>
+      <c r="N71" s="19" t="n">
+        <v>-0.2739</v>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B72" s="25" t="inlineStr">
+      <c r="A72" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B72" s="15" t="inlineStr">
         <is>
           <t>KOLTEPATIL</t>
         </is>
       </c>
-      <c r="C72" s="25" t="inlineStr">
+      <c r="C72" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D72" s="25" t="n"/>
-      <c r="E72" s="26" t="n">
+      <c r="D72" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E72" s="16" t="n">
         <v>99</v>
       </c>
-      <c r="F72" s="27" t="n">
+      <c r="F72" s="17" t="n">
         <v>429.4303</v>
       </c>
-      <c r="G72" s="27" t="n">
+      <c r="G72" s="17" t="n">
         <v>42513.6</v>
       </c>
-      <c r="H72" s="27" t="n">
+      <c r="H72" s="17" t="n">
         <v>13178.29</v>
       </c>
-      <c r="I72" s="27" t="n"/>
-      <c r="J72" s="27" t="n"/>
-      <c r="K72" s="28" t="n"/>
-      <c r="L72" s="27" t="n"/>
-      <c r="M72" s="27" t="n"/>
-      <c r="N72" s="29" t="n"/>
+      <c r="I72" s="17" t="n">
+        <v>431.7773</v>
+      </c>
+      <c r="J72" s="17" t="n">
+        <v>232.35</v>
+      </c>
+      <c r="K72" s="18" t="n">
+        <v>0.5465</v>
+      </c>
+      <c r="L72" s="17" t="n">
+        <v>192.39</v>
+      </c>
+      <c r="M72" s="17" t="n">
+        <v>39.96</v>
+      </c>
+      <c r="N72" s="19" t="n">
+        <v>0.094</v>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B73" s="25" t="inlineStr">
+      <c r="A73" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>ROLEXRINGS</t>
         </is>
       </c>
-      <c r="C73" s="25" t="inlineStr">
+      <c r="C73" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D73" s="25" t="n"/>
-      <c r="E73" s="26" t="n">
+      <c r="D73" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E73" s="16" t="n">
         <v>279</v>
       </c>
-      <c r="F73" s="27" t="n">
+      <c r="F73" s="17" t="n">
         <v>153.48</v>
       </c>
-      <c r="G73" s="27" t="n">
+      <c r="G73" s="17" t="n">
         <v>42820.92</v>
       </c>
-      <c r="H73" s="27" t="n">
+      <c r="H73" s="17" t="n">
         <v>14390.24</v>
       </c>
-      <c r="I73" s="27" t="n"/>
-      <c r="J73" s="27" t="n"/>
-      <c r="K73" s="28" t="n"/>
-      <c r="L73" s="27" t="n"/>
-      <c r="M73" s="27" t="n"/>
-      <c r="N73" s="29" t="n"/>
+      <c r="I73" s="17" t="n">
+        <v>153.9539</v>
+      </c>
+      <c r="J73" s="17" t="n">
+        <v>132.23</v>
+      </c>
+      <c r="K73" s="18" t="n">
+        <v>0.3088</v>
+      </c>
+      <c r="L73" s="17" t="n">
+        <v>192.92</v>
+      </c>
+      <c r="M73" s="17" t="n">
+        <v>-60.69</v>
+      </c>
+      <c r="N73" s="19" t="n">
+        <v>-0.1417</v>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B74" s="25" t="inlineStr">
+      <c r="A74" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>SOTL</t>
         </is>
       </c>
-      <c r="C74" s="25" t="inlineStr">
+      <c r="C74" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D74" s="25" t="n"/>
-      <c r="E74" s="26" t="n">
+      <c r="D74" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E74" s="16" t="n">
         <v>55</v>
       </c>
-      <c r="F74" s="27" t="n">
+      <c r="F74" s="17" t="n">
         <v>776.25</v>
       </c>
-      <c r="G74" s="27" t="n">
+      <c r="G74" s="17" t="n">
         <v>42693.75</v>
       </c>
-      <c r="H74" s="27" t="n">
+      <c r="H74" s="17" t="n">
         <v>15466.24</v>
       </c>
-      <c r="I74" s="27" t="n"/>
-      <c r="J74" s="27" t="n"/>
-      <c r="K74" s="28" t="n"/>
-      <c r="L74" s="27" t="n"/>
-      <c r="M74" s="27" t="n"/>
-      <c r="N74" s="29" t="n"/>
+      <c r="I74" s="17" t="n">
+        <v>783.7027</v>
+      </c>
+      <c r="J74" s="17" t="n">
+        <v>409.9</v>
+      </c>
+      <c r="K74" s="18" t="n">
+        <v>0.9601</v>
+      </c>
+      <c r="L74" s="17" t="n">
+        <v>192.95</v>
+      </c>
+      <c r="M74" s="17" t="n">
+        <v>216.95</v>
+      </c>
+      <c r="N74" s="19" t="n">
+        <v>0.5082</v>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B75" s="25" t="inlineStr">
+      <c r="A75" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B75" s="15" t="inlineStr">
         <is>
           <t>STOVEKRAFT</t>
         </is>
       </c>
-      <c r="C75" s="25" t="inlineStr">
+      <c r="C75" s="15" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="D75" s="25" t="n"/>
-      <c r="E75" s="26" t="n">
+      <c r="D75" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="n">
         <v>53</v>
       </c>
-      <c r="F75" s="27" t="n">
+      <c r="F75" s="17" t="n">
         <v>798.9</v>
       </c>
-      <c r="G75" s="27" t="n">
+      <c r="G75" s="17" t="n">
         <v>42341.7</v>
       </c>
-      <c r="H75" s="27" t="n">
+      <c r="H75" s="17" t="n">
         <v>14986.57</v>
       </c>
-      <c r="I75" s="27" t="n"/>
-      <c r="J75" s="27" t="n"/>
-      <c r="K75" s="28" t="n"/>
-      <c r="L75" s="27" t="n"/>
-      <c r="M75" s="27" t="n"/>
-      <c r="N75" s="29" t="n"/>
+      <c r="I75" s="17" t="n">
+        <v>805.6151</v>
+      </c>
+      <c r="J75" s="17" t="n">
+        <v>355.9</v>
+      </c>
+      <c r="K75" s="18" t="n">
+        <v>0.8405</v>
+      </c>
+      <c r="L75" s="17" t="n">
+        <v>192.16</v>
+      </c>
+      <c r="M75" s="17" t="n">
+        <v>163.74</v>
+      </c>
+      <c r="N75" s="19" t="n">
+        <v>0.3867</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="20" t="inlineStr">
@@ -3608,22 +3720,283 @@
       <c r="H76" s="21" t="n"/>
       <c r="I76" s="21" t="n"/>
       <c r="J76" s="22" t="n">
-        <v>0</v>
+        <v>2202.67</v>
       </c>
       <c r="K76" s="21" t="n"/>
       <c r="L76" s="21" t="n"/>
       <c r="M76" s="22" t="n">
+        <v>854.42</v>
+      </c>
+      <c r="N76" s="23" t="n"/>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-07   ·   4 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="n"/>
+      <c r="C78" s="3" t="n"/>
+      <c r="D78" s="3" t="n"/>
+      <c r="E78" s="3" t="n"/>
+      <c r="F78" s="3" t="n"/>
+      <c r="G78" s="3" t="n"/>
+      <c r="H78" s="3" t="n"/>
+      <c r="I78" s="3" t="n"/>
+      <c r="J78" s="3" t="n"/>
+      <c r="K78" s="3" t="n"/>
+      <c r="L78" s="3" t="n"/>
+      <c r="M78" s="3" t="n"/>
+      <c r="N78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="K79" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="L79" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="M79" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="N79" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B80" s="25" t="inlineStr">
+        <is>
+          <t>ARVSMART</t>
+        </is>
+      </c>
+      <c r="C80" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D80" s="25" t="n"/>
+      <c r="E80" s="26" t="n">
+        <v>92</v>
+      </c>
+      <c r="F80" s="27" t="n">
+        <v>651.1261</v>
+      </c>
+      <c r="G80" s="27" t="n">
+        <v>59903.6</v>
+      </c>
+      <c r="H80" s="27" t="n">
+        <v>19104.42</v>
+      </c>
+      <c r="I80" s="27" t="n"/>
+      <c r="J80" s="27" t="n"/>
+      <c r="K80" s="28" t="n"/>
+      <c r="L80" s="27" t="n"/>
+      <c r="M80" s="27" t="n"/>
+      <c r="N80" s="29" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B81" s="25" t="inlineStr">
+        <is>
+          <t>ELLEN</t>
+        </is>
+      </c>
+      <c r="C81" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D81" s="25" t="n"/>
+      <c r="E81" s="26" t="n">
+        <v>204</v>
+      </c>
+      <c r="F81" s="27" t="n">
+        <v>293.2</v>
+      </c>
+      <c r="G81" s="27" t="n">
+        <v>59812.8</v>
+      </c>
+      <c r="H81" s="27" t="n">
+        <v>21137.84</v>
+      </c>
+      <c r="I81" s="27" t="n"/>
+      <c r="J81" s="27" t="n"/>
+      <c r="K81" s="28" t="n"/>
+      <c r="L81" s="27" t="n"/>
+      <c r="M81" s="27" t="n"/>
+      <c r="N81" s="29" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B82" s="25" t="inlineStr">
+        <is>
+          <t>GOCLCORP</t>
+        </is>
+      </c>
+      <c r="C82" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D82" s="25" t="n"/>
+      <c r="E82" s="26" t="n">
+        <v>136</v>
+      </c>
+      <c r="F82" s="27" t="n">
+        <v>439.7</v>
+      </c>
+      <c r="G82" s="27" t="n">
+        <v>59799.2</v>
+      </c>
+      <c r="H82" s="27" t="n">
+        <v>21634.64</v>
+      </c>
+      <c r="I82" s="27" t="n"/>
+      <c r="J82" s="27" t="n"/>
+      <c r="K82" s="28" t="n"/>
+      <c r="L82" s="27" t="n"/>
+      <c r="M82" s="27" t="n"/>
+      <c r="N82" s="29" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B83" s="25" t="inlineStr">
+        <is>
+          <t>WINDMACHIN</t>
+        </is>
+      </c>
+      <c r="C83" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="D83" s="25" t="n"/>
+      <c r="E83" s="26" t="n">
+        <v>196</v>
+      </c>
+      <c r="F83" s="27" t="n">
+        <v>304.813</v>
+      </c>
+      <c r="G83" s="27" t="n">
+        <v>59743.35</v>
+      </c>
+      <c r="H83" s="27" t="n">
+        <v>29870.4</v>
+      </c>
+      <c r="I83" s="27" t="n"/>
+      <c r="J83" s="27" t="n"/>
+      <c r="K83" s="28" t="n"/>
+      <c r="L83" s="27" t="n"/>
+      <c r="M83" s="27" t="n"/>
+      <c r="N83" s="29" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B84" s="21" t="n"/>
+      <c r="C84" s="21" t="n"/>
+      <c r="D84" s="21" t="n"/>
+      <c r="E84" s="21" t="n"/>
+      <c r="F84" s="21" t="n"/>
+      <c r="G84" s="21" t="n"/>
+      <c r="H84" s="21" t="n"/>
+      <c r="I84" s="21" t="n"/>
+      <c r="J84" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="N76" s="23" t="n"/>
+      <c r="K84" s="21" t="n"/>
+      <c r="L84" s="21" t="n"/>
+      <c r="M84" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N84" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A67:N67"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A61:N61"/>
     <mergeCell ref="A12:N12"/>
     <mergeCell ref="A35:N35"/>
+    <mergeCell ref="A78:N78"/>
     <mergeCell ref="A30:N30"/>
     <mergeCell ref="A52:N52"/>
     <mergeCell ref="A43:N43"/>
@@ -3792,6 +4165,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J80:J83">
+    <cfRule type="dataBar" priority="19">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M80:M83">
+    <cfRule type="dataBar" priority="20">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-10 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N84"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3732,7 +3732,7 @@
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-07   ·   4 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-08-07   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹437.85   ·   Net PnL: ₹-486.78</t>
         </is>
       </c>
       <c r="B78" s="3" t="n"/>
@@ -3822,148 +3822,212 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B80" s="25" t="inlineStr">
+      <c r="A80" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>ARVSMART</t>
         </is>
       </c>
-      <c r="C80" s="25" t="inlineStr">
+      <c r="C80" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="D80" s="25" t="n"/>
-      <c r="E80" s="26" t="n">
+      <c r="D80" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="n">
         <v>92</v>
       </c>
-      <c r="F80" s="27" t="n">
+      <c r="F80" s="17" t="n">
         <v>651.1261</v>
       </c>
-      <c r="G80" s="27" t="n">
+      <c r="G80" s="17" t="n">
         <v>59903.6</v>
       </c>
-      <c r="H80" s="27" t="n">
+      <c r="H80" s="17" t="n">
         <v>19104.42</v>
       </c>
-      <c r="I80" s="27" t="n"/>
-      <c r="J80" s="27" t="n"/>
-      <c r="K80" s="28" t="n"/>
-      <c r="L80" s="27" t="n"/>
-      <c r="M80" s="27" t="n"/>
-      <c r="N80" s="29" t="n"/>
+      <c r="I80" s="17" t="n">
+        <v>679.619</v>
+      </c>
+      <c r="J80" s="17" t="n">
+        <v>2621.35</v>
+      </c>
+      <c r="K80" s="18" t="n">
+        <v>4.3759</v>
+      </c>
+      <c r="L80" s="17" t="n">
+        <v>233.95</v>
+      </c>
+      <c r="M80" s="17" t="n">
+        <v>2387.4</v>
+      </c>
+      <c r="N80" s="19" t="n">
+        <v>3.9854</v>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B81" s="25" t="inlineStr">
+      <c r="A81" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
         <is>
           <t>ELLEN</t>
         </is>
       </c>
-      <c r="C81" s="25" t="inlineStr">
+      <c r="C81" s="15" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="D81" s="25" t="n"/>
-      <c r="E81" s="26" t="n">
+      <c r="D81" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="n">
         <v>204</v>
       </c>
-      <c r="F81" s="27" t="n">
+      <c r="F81" s="17" t="n">
         <v>293.2</v>
       </c>
-      <c r="G81" s="27" t="n">
+      <c r="G81" s="17" t="n">
         <v>59812.8</v>
       </c>
-      <c r="H81" s="27" t="n">
+      <c r="H81" s="17" t="n">
         <v>21137.84</v>
       </c>
-      <c r="I81" s="27" t="n"/>
-      <c r="J81" s="27" t="n"/>
-      <c r="K81" s="28" t="n"/>
-      <c r="L81" s="27" t="n"/>
-      <c r="M81" s="27" t="n"/>
-      <c r="N81" s="29" t="n"/>
+      <c r="I81" s="17" t="n">
+        <v>302.1953</v>
+      </c>
+      <c r="J81" s="17" t="n">
+        <v>1835.05</v>
+      </c>
+      <c r="K81" s="18" t="n">
+        <v>3.068</v>
+      </c>
+      <c r="L81" s="17" t="n">
+        <v>232.94</v>
+      </c>
+      <c r="M81" s="17" t="n">
+        <v>1602.11</v>
+      </c>
+      <c r="N81" s="19" t="n">
+        <v>2.6785</v>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B82" s="25" t="inlineStr">
+      <c r="A82" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
         <is>
           <t>GOCLCORP</t>
         </is>
       </c>
-      <c r="C82" s="25" t="inlineStr">
+      <c r="C82" s="9" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="D82" s="25" t="n"/>
-      <c r="E82" s="26" t="n">
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E82" s="10" t="n">
         <v>136</v>
       </c>
-      <c r="F82" s="27" t="n">
+      <c r="F82" s="11" t="n">
         <v>439.7</v>
       </c>
-      <c r="G82" s="27" t="n">
+      <c r="G82" s="11" t="n">
         <v>59799.2</v>
       </c>
-      <c r="H82" s="27" t="n">
+      <c r="H82" s="11" t="n">
         <v>21634.64</v>
       </c>
-      <c r="I82" s="27" t="n"/>
-      <c r="J82" s="27" t="n"/>
-      <c r="K82" s="28" t="n"/>
-      <c r="L82" s="27" t="n"/>
-      <c r="M82" s="27" t="n"/>
-      <c r="N82" s="29" t="n"/>
+      <c r="I82" s="11" t="n">
+        <v>426.0838</v>
+      </c>
+      <c r="J82" s="11" t="n">
+        <v>-1851.8</v>
+      </c>
+      <c r="K82" s="12" t="n">
+        <v>-3.0967</v>
+      </c>
+      <c r="L82" s="11" t="n">
+        <v>229.09</v>
+      </c>
+      <c r="M82" s="11" t="n">
+        <v>-2080.89</v>
+      </c>
+      <c r="N82" s="13" t="n">
+        <v>-3.4798</v>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B83" s="25" t="inlineStr">
+      <c r="A83" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
         <is>
           <t>WINDMACHIN</t>
         </is>
       </c>
-      <c r="C83" s="25" t="inlineStr">
+      <c r="C83" s="9" t="inlineStr">
         <is>
           <t>2026-08-07</t>
         </is>
       </c>
-      <c r="D83" s="25" t="n"/>
-      <c r="E83" s="26" t="n">
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="E83" s="10" t="n">
         <v>196</v>
       </c>
-      <c r="F83" s="27" t="n">
+      <c r="F83" s="11" t="n">
         <v>304.813</v>
       </c>
-      <c r="G83" s="27" t="n">
+      <c r="G83" s="11" t="n">
         <v>59743.35</v>
       </c>
-      <c r="H83" s="27" t="n">
+      <c r="H83" s="11" t="n">
         <v>29870.4</v>
       </c>
-      <c r="I83" s="27" t="n"/>
-      <c r="J83" s="27" t="n"/>
-      <c r="K83" s="28" t="n"/>
-      <c r="L83" s="27" t="n"/>
-      <c r="M83" s="27" t="n"/>
-      <c r="N83" s="29" t="n"/>
+      <c r="I83" s="11" t="n">
+        <v>293.7582</v>
+      </c>
+      <c r="J83" s="11" t="n">
+        <v>-2166.75</v>
+      </c>
+      <c r="K83" s="12" t="n">
+        <v>-3.6268</v>
+      </c>
+      <c r="L83" s="11" t="n">
+        <v>228.65</v>
+      </c>
+      <c r="M83" s="11" t="n">
+        <v>-2395.4</v>
+      </c>
+      <c r="N83" s="13" t="n">
+        <v>-4.0095</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="20" t="inlineStr">
@@ -3980,17 +4044,277 @@
       <c r="H84" s="21" t="n"/>
       <c r="I84" s="21" t="n"/>
       <c r="J84" s="22" t="n">
-        <v>0</v>
+        <v>437.85</v>
       </c>
       <c r="K84" s="21" t="n"/>
       <c r="L84" s="21" t="n"/>
       <c r="M84" s="22" t="n">
+        <v>-486.78</v>
+      </c>
+      <c r="N84" s="23" t="n"/>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-10   ·   4 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="n"/>
+      <c r="C86" s="3" t="n"/>
+      <c r="D86" s="3" t="n"/>
+      <c r="E86" s="3" t="n"/>
+      <c r="F86" s="3" t="n"/>
+      <c r="G86" s="3" t="n"/>
+      <c r="H86" s="3" t="n"/>
+      <c r="I86" s="3" t="n"/>
+      <c r="J86" s="3" t="n"/>
+      <c r="K86" s="3" t="n"/>
+      <c r="L86" s="3" t="n"/>
+      <c r="M86" s="3" t="n"/>
+      <c r="N86" s="4" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C87" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="K87" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="L87" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="M87" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="N87" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B88" s="25" t="inlineStr">
+        <is>
+          <t>GARUDA</t>
+        </is>
+      </c>
+      <c r="C88" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="D88" s="25" t="n"/>
+      <c r="E88" s="26" t="n">
+        <v>128</v>
+      </c>
+      <c r="F88" s="27" t="n">
+        <v>194</v>
+      </c>
+      <c r="G88" s="27" t="n">
+        <v>24832</v>
+      </c>
+      <c r="H88" s="27" t="n">
+        <v>24832</v>
+      </c>
+      <c r="I88" s="27" t="n"/>
+      <c r="J88" s="27" t="n"/>
+      <c r="K88" s="28" t="n"/>
+      <c r="L88" s="27" t="n"/>
+      <c r="M88" s="27" t="n"/>
+      <c r="N88" s="29" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B89" s="25" t="inlineStr">
+        <is>
+          <t>JGCHEM</t>
+        </is>
+      </c>
+      <c r="C89" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="D89" s="25" t="n"/>
+      <c r="E89" s="26" t="n">
+        <v>80</v>
+      </c>
+      <c r="F89" s="27" t="n">
+        <v>619.3</v>
+      </c>
+      <c r="G89" s="27" t="n">
+        <v>49544</v>
+      </c>
+      <c r="H89" s="27" t="n">
+        <v>17957.4</v>
+      </c>
+      <c r="I89" s="27" t="n"/>
+      <c r="J89" s="27" t="n"/>
+      <c r="K89" s="28" t="n"/>
+      <c r="L89" s="27" t="n"/>
+      <c r="M89" s="27" t="n"/>
+      <c r="N89" s="29" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B90" s="25" t="inlineStr">
+        <is>
+          <t>PIXTRANS</t>
+        </is>
+      </c>
+      <c r="C90" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="D90" s="25" t="n"/>
+      <c r="E90" s="26" t="n">
+        <v>25</v>
+      </c>
+      <c r="F90" s="27" t="n">
+        <v>1972</v>
+      </c>
+      <c r="G90" s="27" t="n">
+        <v>49300</v>
+      </c>
+      <c r="H90" s="27" t="n">
+        <v>16130.96</v>
+      </c>
+      <c r="I90" s="27" t="n"/>
+      <c r="J90" s="27" t="n"/>
+      <c r="K90" s="28" t="n"/>
+      <c r="L90" s="27" t="n"/>
+      <c r="M90" s="27" t="n"/>
+      <c r="N90" s="29" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B91" s="25" t="inlineStr">
+        <is>
+          <t>RAMCOIND</t>
+        </is>
+      </c>
+      <c r="C91" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="D91" s="25" t="n"/>
+      <c r="E91" s="26" t="n">
+        <v>134</v>
+      </c>
+      <c r="F91" s="27" t="n">
+        <v>373.5836</v>
+      </c>
+      <c r="G91" s="27" t="n">
+        <v>50060.2</v>
+      </c>
+      <c r="H91" s="27" t="n">
+        <v>16871.52</v>
+      </c>
+      <c r="I91" s="27" t="n"/>
+      <c r="J91" s="27" t="n"/>
+      <c r="K91" s="28" t="n"/>
+      <c r="L91" s="27" t="n"/>
+      <c r="M91" s="27" t="n"/>
+      <c r="N91" s="29" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B92" s="21" t="n"/>
+      <c r="C92" s="21" t="n"/>
+      <c r="D92" s="21" t="n"/>
+      <c r="E92" s="21" t="n"/>
+      <c r="F92" s="21" t="n"/>
+      <c r="G92" s="21" t="n"/>
+      <c r="H92" s="21" t="n"/>
+      <c r="I92" s="21" t="n"/>
+      <c r="J92" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="N84" s="23" t="n"/>
+      <c r="K92" s="21" t="n"/>
+      <c r="L92" s="21" t="n"/>
+      <c r="M92" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A67:N67"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A61:N61"/>
@@ -3998,6 +4322,7 @@
     <mergeCell ref="A35:N35"/>
     <mergeCell ref="A78:N78"/>
     <mergeCell ref="A30:N30"/>
+    <mergeCell ref="A86:N86"/>
     <mergeCell ref="A52:N52"/>
     <mergeCell ref="A43:N43"/>
     <mergeCell ref="A19:N19"/>
@@ -4183,6 +4508,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J88:J91">
+    <cfRule type="dataBar" priority="21">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M88:M91">
+    <cfRule type="dataBar" priority="22">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Account for MTF interest charges in trade book
Kite Connect's /charges/orders API has no interest field -- MTF interest
on the funded (borrowed) portion was silently missing from Total Charges,
overstating Net P&L on every MTF trade. Added at the confirmed 0.04%/day
rate, applied per calendar day held.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -2656,7 +2656,7 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,298.75</t>
+          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,255.11</t>
         </is>
       </c>
       <c r="B52" s="3" t="n"/>
@@ -2788,13 +2788,13 @@
         <v>3.5955</v>
       </c>
       <c r="L54" s="17" t="n">
-        <v>211.56</v>
+        <v>225.42</v>
       </c>
       <c r="M54" s="17" t="n">
-        <v>1586.54</v>
+        <v>1572.68</v>
       </c>
       <c r="N54" s="19" t="n">
-        <v>3.1725</v>
+        <v>3.1448</v>
       </c>
     </row>
     <row r="55">
@@ -2840,13 +2840,13 @@
         <v>2.2623</v>
       </c>
       <c r="L55" s="17" t="n">
-        <v>209.66</v>
+        <v>219.65</v>
       </c>
       <c r="M55" s="17" t="n">
-        <v>919.4400000000001</v>
+        <v>909.45</v>
       </c>
       <c r="N55" s="19" t="n">
-        <v>1.8422</v>
+        <v>1.8222</v>
       </c>
     </row>
     <row r="56">
@@ -2892,13 +2892,13 @@
         <v>3.7519</v>
       </c>
       <c r="L56" s="17" t="n">
-        <v>210</v>
+        <v>219.93</v>
       </c>
       <c r="M56" s="17" t="n">
-        <v>1654.85</v>
+        <v>1644.92</v>
       </c>
       <c r="N56" s="19" t="n">
-        <v>3.3294</v>
+        <v>3.3094</v>
       </c>
     </row>
     <row r="57">
@@ -2996,13 +2996,13 @@
         <v>-1.2518</v>
       </c>
       <c r="L58" s="11" t="n">
-        <v>206.58</v>
+        <v>216.44</v>
       </c>
       <c r="M58" s="11" t="n">
-        <v>-823.6799999999999</v>
+        <v>-833.54</v>
       </c>
       <c r="N58" s="13" t="n">
-        <v>-1.6709</v>
+        <v>-1.6909</v>
       </c>
     </row>
     <row r="59">
@@ -3025,14 +3025,14 @@
       <c r="K59" s="21" t="n"/>
       <c r="L59" s="21" t="n"/>
       <c r="M59" s="22" t="n">
-        <v>3298.75</v>
+        <v>3255.11</v>
       </c>
       <c r="N59" s="23" t="n"/>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-08-05   ·   2 trade(s), 2 closed   ·   Gross PnL: ₹322.90   ·   Net PnL: ₹-206.00</t>
+          <t xml:space="preserve">  🟢  2026-08-05   ·   2 trade(s), 2 closed   ·   Gross PnL: ₹322.90   ·   Net PnL: ₹-245.36</t>
         </is>
       </c>
       <c r="B61" s="3" t="n"/>
@@ -3164,13 +3164,13 @@
         <v>0.3941</v>
       </c>
       <c r="L63" s="17" t="n">
-        <v>264.51</v>
+        <v>283.68</v>
       </c>
       <c r="M63" s="17" t="n">
-        <v>30.44</v>
+        <v>11.27</v>
       </c>
       <c r="N63" s="19" t="n">
-        <v>0.0407</v>
+        <v>0.0151</v>
       </c>
     </row>
     <row r="64">
@@ -3216,13 +3216,13 @@
         <v>0.0373</v>
       </c>
       <c r="L64" s="17" t="n">
-        <v>264.39</v>
+        <v>284.58</v>
       </c>
       <c r="M64" s="17" t="n">
-        <v>-236.44</v>
+        <v>-256.63</v>
       </c>
       <c r="N64" s="19" t="n">
-        <v>-0.3156</v>
+        <v>-0.3426</v>
       </c>
     </row>
     <row r="65">
@@ -3245,14 +3245,14 @@
       <c r="K65" s="21" t="n"/>
       <c r="L65" s="21" t="n"/>
       <c r="M65" s="22" t="n">
-        <v>-206</v>
+        <v>-245.36</v>
       </c>
       <c r="N65" s="23" t="n"/>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-08-06   ·   7 trade(s), 7 closed   ·   Gross PnL: ₹2,202.67   ·   Net PnL: ₹854.42</t>
+          <t xml:space="preserve">  🟢  2026-08-06   ·   7 trade(s), 7 closed   ·   Gross PnL: ₹2,202.67   ·   Net PnL: ₹776.20</t>
         </is>
       </c>
       <c r="B67" s="3" t="n"/>
@@ -3384,13 +3384,13 @@
         <v>0.6614</v>
       </c>
       <c r="L69" s="17" t="n">
-        <v>193.03</v>
+        <v>205.02</v>
       </c>
       <c r="M69" s="17" t="n">
-        <v>90.02</v>
+        <v>78.03</v>
       </c>
       <c r="N69" s="19" t="n">
-        <v>0.2103</v>
+        <v>0.1823</v>
       </c>
     </row>
     <row r="70">
@@ -3436,13 +3436,13 @@
         <v>1.6668</v>
       </c>
       <c r="L70" s="17" t="n">
-        <v>193.46</v>
+        <v>202.87</v>
       </c>
       <c r="M70" s="17" t="n">
-        <v>519.73</v>
+        <v>510.32</v>
       </c>
       <c r="N70" s="19" t="n">
-        <v>1.2147</v>
+        <v>1.1927</v>
       </c>
     </row>
     <row r="71">
@@ -3488,13 +3488,13 @@
         <v>0.1807</v>
       </c>
       <c r="L71" s="17" t="n">
-        <v>191.34</v>
+        <v>203.23</v>
       </c>
       <c r="M71" s="17" t="n">
-        <v>-115.29</v>
+        <v>-127.18</v>
       </c>
       <c r="N71" s="19" t="n">
-        <v>-0.2739</v>
+        <v>-0.3022</v>
       </c>
     </row>
     <row r="72">
@@ -3540,13 +3540,13 @@
         <v>0.5465</v>
       </c>
       <c r="L72" s="17" t="n">
-        <v>192.39</v>
+        <v>204.12</v>
       </c>
       <c r="M72" s="17" t="n">
-        <v>39.96</v>
+        <v>28.23</v>
       </c>
       <c r="N72" s="19" t="n">
-        <v>0.094</v>
+        <v>0.0664</v>
       </c>
     </row>
     <row r="73">
@@ -3592,13 +3592,13 @@
         <v>0.3088</v>
       </c>
       <c r="L73" s="17" t="n">
-        <v>192.92</v>
+        <v>204.29</v>
       </c>
       <c r="M73" s="17" t="n">
-        <v>-60.69</v>
+        <v>-72.06</v>
       </c>
       <c r="N73" s="19" t="n">
-        <v>-0.1417</v>
+        <v>-0.1683</v>
       </c>
     </row>
     <row r="74">
@@ -3644,13 +3644,13 @@
         <v>0.9601</v>
       </c>
       <c r="L74" s="17" t="n">
-        <v>192.95</v>
+        <v>203.84</v>
       </c>
       <c r="M74" s="17" t="n">
-        <v>216.95</v>
+        <v>206.06</v>
       </c>
       <c r="N74" s="19" t="n">
-        <v>0.5082</v>
+        <v>0.4826</v>
       </c>
     </row>
     <row r="75">
@@ -3696,13 +3696,13 @@
         <v>0.8405</v>
       </c>
       <c r="L75" s="17" t="n">
-        <v>192.16</v>
+        <v>203.1</v>
       </c>
       <c r="M75" s="17" t="n">
-        <v>163.74</v>
+        <v>152.8</v>
       </c>
       <c r="N75" s="19" t="n">
-        <v>0.3867</v>
+        <v>0.3609</v>
       </c>
     </row>
     <row r="76">
@@ -3725,14 +3725,14 @@
       <c r="K76" s="21" t="n"/>
       <c r="L76" s="21" t="n"/>
       <c r="M76" s="22" t="n">
-        <v>854.42</v>
+        <v>776.2</v>
       </c>
       <c r="N76" s="23" t="n"/>
     </row>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-08-07   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹437.85   ·   Net PnL: ₹-486.78</t>
+          <t xml:space="preserve">  🟢  2026-08-07   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹437.85   ·   Net PnL: ₹-663.80</t>
         </is>
       </c>
       <c r="B78" s="3" t="n"/>
@@ -3864,13 +3864,13 @@
         <v>4.3759</v>
       </c>
       <c r="L80" s="17" t="n">
-        <v>233.95</v>
+        <v>282.91</v>
       </c>
       <c r="M80" s="17" t="n">
-        <v>2387.4</v>
+        <v>2338.44</v>
       </c>
       <c r="N80" s="19" t="n">
-        <v>3.9854</v>
+        <v>3.9037</v>
       </c>
     </row>
     <row r="81">
@@ -3916,13 +3916,13 @@
         <v>3.068</v>
       </c>
       <c r="L81" s="17" t="n">
-        <v>232.94</v>
+        <v>279.35</v>
       </c>
       <c r="M81" s="17" t="n">
-        <v>1602.11</v>
+        <v>1555.7</v>
       </c>
       <c r="N81" s="19" t="n">
-        <v>2.6785</v>
+        <v>2.6009</v>
       </c>
     </row>
     <row r="82">
@@ -3968,13 +3968,13 @@
         <v>-3.0967</v>
       </c>
       <c r="L82" s="11" t="n">
-        <v>229.09</v>
+        <v>274.89</v>
       </c>
       <c r="M82" s="11" t="n">
-        <v>-2080.89</v>
+        <v>-2126.69</v>
       </c>
       <c r="N82" s="13" t="n">
-        <v>-3.4798</v>
+        <v>-3.5564</v>
       </c>
     </row>
     <row r="83">
@@ -4020,13 +4020,13 @@
         <v>-3.6268</v>
       </c>
       <c r="L83" s="11" t="n">
-        <v>228.65</v>
+        <v>264.5</v>
       </c>
       <c r="M83" s="11" t="n">
-        <v>-2395.4</v>
+        <v>-2431.25</v>
       </c>
       <c r="N83" s="13" t="n">
-        <v>-4.0095</v>
+        <v>-4.0695</v>
       </c>
     </row>
     <row r="84">
@@ -4049,7 +4049,7 @@
       <c r="K84" s="21" t="n"/>
       <c r="L84" s="21" t="n"/>
       <c r="M84" s="22" t="n">
-        <v>-486.78</v>
+        <v>-663.8</v>
       </c>
       <c r="N84" s="23" t="n"/>
     </row>

</xml_diff>

<commit_message>
Data update — 2026-08-11 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1036,7 +1036,7 @@
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-07-28   ·   3 trade(s), 3 closed   ·   Gross PnL: ₹2,642.00   ·   Net PnL: ₹2,342.15</t>
+          <t xml:space="preserve">  🟢  2026-07-28   ·   3 trade(s), 3 closed   ·   Gross PnL: ₹2,642.00   ·   Net PnL: ₹2,104.21</t>
         </is>
       </c>
       <c r="B12" s="3" t="n"/>
@@ -1167,15 +1167,9 @@
       <c r="K14" s="18" t="n">
         <v>0.9074</v>
       </c>
-      <c r="L14" s="17" t="n">
-        <v>98.66</v>
-      </c>
-      <c r="M14" s="17" t="n">
-        <v>237.94</v>
-      </c>
-      <c r="N14" s="19" t="n">
-        <v>0.6414</v>
-      </c>
+      <c r="L14" s="17" t="n"/>
+      <c r="M14" s="17" t="n"/>
+      <c r="N14" s="19" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="14" t="inlineStr">
@@ -1301,14 +1295,14 @@
       <c r="K17" s="21" t="n"/>
       <c r="L17" s="21" t="n"/>
       <c r="M17" s="22" t="n">
-        <v>2342.15</v>
+        <v>2104.21</v>
       </c>
       <c r="N17" s="23" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-07-29   ·   7 trade(s), 7 closed   ·   Gross PnL: ₹1,048.60   ·   Net PnL: ₹611.70</t>
+          <t xml:space="preserve">  🟢  2026-07-29   ·   7 trade(s), 7 closed   ·   Gross PnL: ₹1,048.60   ·   Net PnL: ₹1,071.80</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
@@ -1751,15 +1745,9 @@
       <c r="K27" s="12" t="n">
         <v>-1.8494</v>
       </c>
-      <c r="L27" s="11" t="n">
-        <v>62.53</v>
-      </c>
-      <c r="M27" s="11" t="n">
-        <v>-460.1</v>
-      </c>
-      <c r="N27" s="13" t="n">
-        <v>-2.1403</v>
-      </c>
+      <c r="L27" s="11" t="n"/>
+      <c r="M27" s="11" t="n"/>
+      <c r="N27" s="13" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="20" t="inlineStr">
@@ -1781,7 +1769,7 @@
       <c r="K28" s="21" t="n"/>
       <c r="L28" s="21" t="n"/>
       <c r="M28" s="22" t="n">
-        <v>611.7</v>
+        <v>1071.8</v>
       </c>
       <c r="N28" s="23" t="n"/>
     </row>
@@ -1956,7 +1944,7 @@
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-07-31   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹206.88   ·   Net PnL: ₹-72.55</t>
+          <t xml:space="preserve">  🟢  2026-07-31   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹206.88   ·   Net PnL: ₹28.16</t>
         </is>
       </c>
       <c r="B35" s="3" t="n"/>
@@ -2139,15 +2127,9 @@
       <c r="K38" s="12" t="n">
         <v>-0.1192</v>
       </c>
-      <c r="L38" s="11" t="n">
-        <v>71.01000000000001</v>
-      </c>
-      <c r="M38" s="11" t="n">
-        <v>-100.71</v>
-      </c>
-      <c r="N38" s="13" t="n">
-        <v>-0.4042</v>
-      </c>
+      <c r="L38" s="11" t="n"/>
+      <c r="M38" s="11" t="n"/>
+      <c r="N38" s="13" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="14" t="inlineStr">
@@ -2273,7 +2255,7 @@
       <c r="K41" s="21" t="n"/>
       <c r="L41" s="21" t="n"/>
       <c r="M41" s="22" t="n">
-        <v>-72.55</v>
+        <v>28.16</v>
       </c>
       <c r="N41" s="23" t="n"/>
     </row>
@@ -2656,7 +2638,7 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,255.11</t>
+          <t xml:space="preserve">  🟢  2026-08-04   ·   5 trade(s), 5 closed   ·   Gross PnL: ₹4,207.65   ·   Net PnL: ₹3,293.51</t>
         </is>
       </c>
       <c r="B52" s="3" t="n"/>
@@ -2943,15 +2925,9 @@
       <c r="K57" s="18" t="n">
         <v>0.1312</v>
       </c>
-      <c r="L57" s="17" t="n">
-        <v>71.09999999999999</v>
-      </c>
-      <c r="M57" s="17" t="n">
-        <v>-38.4</v>
-      </c>
-      <c r="N57" s="19" t="n">
-        <v>-0.154</v>
-      </c>
+      <c r="L57" s="17" t="n"/>
+      <c r="M57" s="17" t="n"/>
+      <c r="N57" s="19" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -3025,7 +3001,7 @@
       <c r="K59" s="21" t="n"/>
       <c r="L59" s="21" t="n"/>
       <c r="M59" s="22" t="n">
-        <v>3255.11</v>
+        <v>3293.51</v>
       </c>
       <c r="N59" s="23" t="n"/>
     </row>
@@ -4056,7 +4032,7 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-10   ·   4 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🟢  2026-08-10   ·   4 trade(s), 4 closed   ·   Gross PnL: ₹4,659.52   ·   Net PnL: ₹3,919.88</t>
         </is>
       </c>
       <c r="B86" s="3" t="n"/>
@@ -4146,148 +4122,212 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B88" s="25" t="inlineStr">
+      <c r="A88" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B88" s="15" t="inlineStr">
         <is>
           <t>GARUDA</t>
         </is>
       </c>
-      <c r="C88" s="25" t="inlineStr">
+      <c r="C88" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="D88" s="25" t="n"/>
-      <c r="E88" s="26" t="n">
+      <c r="D88" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="n">
         <v>128</v>
       </c>
-      <c r="F88" s="27" t="n">
+      <c r="F88" s="17" t="n">
         <v>194</v>
       </c>
-      <c r="G88" s="27" t="n">
+      <c r="G88" s="17" t="n">
         <v>24832</v>
       </c>
-      <c r="H88" s="27" t="n">
+      <c r="H88" s="17" t="n">
         <v>24832</v>
       </c>
-      <c r="I88" s="27" t="n"/>
-      <c r="J88" s="27" t="n"/>
-      <c r="K88" s="28" t="n"/>
-      <c r="L88" s="27" t="n"/>
-      <c r="M88" s="27" t="n"/>
-      <c r="N88" s="29" t="n"/>
+      <c r="I88" s="17" t="n">
+        <v>194.315</v>
+      </c>
+      <c r="J88" s="17" t="n">
+        <v>40.32</v>
+      </c>
+      <c r="K88" s="18" t="n">
+        <v>0.1624</v>
+      </c>
+      <c r="L88" s="17" t="n">
+        <v>70.90000000000001</v>
+      </c>
+      <c r="M88" s="17" t="n">
+        <v>-30.58</v>
+      </c>
+      <c r="N88" s="19" t="n">
+        <v>-0.1231</v>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B89" s="25" t="inlineStr">
+      <c r="A89" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B89" s="15" t="inlineStr">
         <is>
           <t>JGCHEM</t>
         </is>
       </c>
-      <c r="C89" s="25" t="inlineStr">
+      <c r="C89" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="D89" s="25" t="n"/>
-      <c r="E89" s="26" t="n">
+      <c r="D89" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="n">
         <v>80</v>
       </c>
-      <c r="F89" s="27" t="n">
+      <c r="F89" s="17" t="n">
         <v>619.3</v>
       </c>
-      <c r="G89" s="27" t="n">
+      <c r="G89" s="17" t="n">
         <v>49544</v>
       </c>
-      <c r="H89" s="27" t="n">
+      <c r="H89" s="17" t="n">
         <v>17957.4</v>
       </c>
-      <c r="I89" s="27" t="n"/>
-      <c r="J89" s="27" t="n"/>
-      <c r="K89" s="28" t="n"/>
-      <c r="L89" s="27" t="n"/>
-      <c r="M89" s="27" t="n"/>
-      <c r="N89" s="29" t="n"/>
+      <c r="I89" s="17" t="n">
+        <v>646.95</v>
+      </c>
+      <c r="J89" s="17" t="n">
+        <v>2212</v>
+      </c>
+      <c r="K89" s="18" t="n">
+        <v>4.4647</v>
+      </c>
+      <c r="L89" s="17" t="n">
+        <v>222.66</v>
+      </c>
+      <c r="M89" s="17" t="n">
+        <v>1989.34</v>
+      </c>
+      <c r="N89" s="19" t="n">
+        <v>4.0153</v>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B90" s="25" t="inlineStr">
+      <c r="A90" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B90" s="15" t="inlineStr">
         <is>
           <t>PIXTRANS</t>
         </is>
       </c>
-      <c r="C90" s="25" t="inlineStr">
+      <c r="C90" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="D90" s="25" t="n"/>
-      <c r="E90" s="26" t="n">
+      <c r="D90" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="F90" s="27" t="n">
+      <c r="F90" s="17" t="n">
         <v>1972</v>
       </c>
-      <c r="G90" s="27" t="n">
+      <c r="G90" s="17" t="n">
         <v>49300</v>
       </c>
-      <c r="H90" s="27" t="n">
+      <c r="H90" s="17" t="n">
         <v>16130.96</v>
       </c>
-      <c r="I90" s="27" t="n"/>
-      <c r="J90" s="27" t="n"/>
-      <c r="K90" s="28" t="n"/>
-      <c r="L90" s="27" t="n"/>
-      <c r="M90" s="27" t="n"/>
-      <c r="N90" s="29" t="n"/>
+      <c r="I90" s="17" t="n">
+        <v>2022.372</v>
+      </c>
+      <c r="J90" s="17" t="n">
+        <v>1259.3</v>
+      </c>
+      <c r="K90" s="18" t="n">
+        <v>2.5544</v>
+      </c>
+      <c r="L90" s="17" t="n">
+        <v>221.8</v>
+      </c>
+      <c r="M90" s="17" t="n">
+        <v>1037.5</v>
+      </c>
+      <c r="N90" s="19" t="n">
+        <v>2.1045</v>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B91" s="25" t="inlineStr">
+      <c r="A91" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B91" s="15" t="inlineStr">
         <is>
           <t>RAMCOIND</t>
         </is>
       </c>
-      <c r="C91" s="25" t="inlineStr">
+      <c r="C91" s="15" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="D91" s="25" t="n"/>
-      <c r="E91" s="26" t="n">
+      <c r="D91" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="n">
         <v>134</v>
       </c>
-      <c r="F91" s="27" t="n">
+      <c r="F91" s="17" t="n">
         <v>373.5836</v>
       </c>
-      <c r="G91" s="27" t="n">
+      <c r="G91" s="17" t="n">
         <v>50060.2</v>
       </c>
-      <c r="H91" s="27" t="n">
+      <c r="H91" s="17" t="n">
         <v>16871.52</v>
       </c>
-      <c r="I91" s="27" t="n"/>
-      <c r="J91" s="27" t="n"/>
-      <c r="K91" s="28" t="n"/>
-      <c r="L91" s="27" t="n"/>
-      <c r="M91" s="27" t="n"/>
-      <c r="N91" s="29" t="n"/>
+      <c r="I91" s="17" t="n">
+        <v>382.15</v>
+      </c>
+      <c r="J91" s="17" t="n">
+        <v>1147.9</v>
+      </c>
+      <c r="K91" s="18" t="n">
+        <v>2.293</v>
+      </c>
+      <c r="L91" s="17" t="n">
+        <v>224.28</v>
+      </c>
+      <c r="M91" s="17" t="n">
+        <v>923.62</v>
+      </c>
+      <c r="N91" s="19" t="n">
+        <v>1.845</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="20" t="inlineStr">
@@ -4304,17 +4344,242 @@
       <c r="H92" s="21" t="n"/>
       <c r="I92" s="21" t="n"/>
       <c r="J92" s="22" t="n">
-        <v>0</v>
+        <v>4659.52</v>
       </c>
       <c r="K92" s="21" t="n"/>
       <c r="L92" s="21" t="n"/>
       <c r="M92" s="22" t="n">
+        <v>3919.88</v>
+      </c>
+      <c r="N92" s="23" t="n"/>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-11   ·   3 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="3" t="n"/>
+      <c r="D94" s="3" t="n"/>
+      <c r="E94" s="3" t="n"/>
+      <c r="F94" s="3" t="n"/>
+      <c r="G94" s="3" t="n"/>
+      <c r="H94" s="3" t="n"/>
+      <c r="I94" s="3" t="n"/>
+      <c r="J94" s="3" t="n"/>
+      <c r="K94" s="3" t="n"/>
+      <c r="L94" s="3" t="n"/>
+      <c r="M94" s="3" t="n"/>
+      <c r="N94" s="4" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C95" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I95" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="J95" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="K95" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="L95" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="M95" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="N95" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B96" s="25" t="inlineStr">
+        <is>
+          <t>KOLTEPATIL</t>
+        </is>
+      </c>
+      <c r="C96" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="D96" s="25" t="n"/>
+      <c r="E96" s="26" t="n">
+        <v>145</v>
+      </c>
+      <c r="F96" s="27" t="n">
+        <v>516.6731</v>
+      </c>
+      <c r="G96" s="27" t="n">
+        <v>74917.60000000001</v>
+      </c>
+      <c r="H96" s="27" t="n">
+        <v>23770.29</v>
+      </c>
+      <c r="I96" s="27" t="n"/>
+      <c r="J96" s="27" t="n"/>
+      <c r="K96" s="28" t="n"/>
+      <c r="L96" s="27" t="n"/>
+      <c r="M96" s="27" t="n"/>
+      <c r="N96" s="29" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B97" s="25" t="inlineStr">
+        <is>
+          <t>ROLEXRINGS</t>
+        </is>
+      </c>
+      <c r="C97" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="D97" s="25" t="n"/>
+      <c r="E97" s="26" t="n">
+        <v>425</v>
+      </c>
+      <c r="F97" s="27" t="n">
+        <v>177.4387</v>
+      </c>
+      <c r="G97" s="27" t="n">
+        <v>75411.45</v>
+      </c>
+      <c r="H97" s="27" t="n">
+        <v>25411.73</v>
+      </c>
+      <c r="I97" s="27" t="n"/>
+      <c r="J97" s="27" t="n"/>
+      <c r="K97" s="28" t="n"/>
+      <c r="L97" s="27" t="n"/>
+      <c r="M97" s="27" t="n"/>
+      <c r="N97" s="29" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B98" s="25" t="inlineStr">
+        <is>
+          <t>WINDLAS</t>
+        </is>
+      </c>
+      <c r="C98" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="D98" s="25" t="n"/>
+      <c r="E98" s="26" t="n">
+        <v>79</v>
+      </c>
+      <c r="F98" s="27" t="n">
+        <v>941.6797</v>
+      </c>
+      <c r="G98" s="27" t="n">
+        <v>74392.7</v>
+      </c>
+      <c r="H98" s="27" t="n">
+        <v>24271.68</v>
+      </c>
+      <c r="I98" s="27" t="n"/>
+      <c r="J98" s="27" t="n"/>
+      <c r="K98" s="28" t="n"/>
+      <c r="L98" s="27" t="n"/>
+      <c r="M98" s="27" t="n"/>
+      <c r="N98" s="29" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B99" s="21" t="n"/>
+      <c r="C99" s="21" t="n"/>
+      <c r="D99" s="21" t="n"/>
+      <c r="E99" s="21" t="n"/>
+      <c r="F99" s="21" t="n"/>
+      <c r="G99" s="21" t="n"/>
+      <c r="H99" s="21" t="n"/>
+      <c r="I99" s="21" t="n"/>
+      <c r="J99" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="N92" s="23" t="n"/>
+      <c r="K99" s="21" t="n"/>
+      <c r="L99" s="21" t="n"/>
+      <c r="M99" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N99" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
+    <mergeCell ref="A94:N94"/>
     <mergeCell ref="A67:N67"/>
     <mergeCell ref="A3:N3"/>
     <mergeCell ref="A61:N61"/>
@@ -4526,6 +4791,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J96:J98">
+    <cfRule type="dataBar" priority="23">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M96:M98">
+    <cfRule type="dataBar" priority="24">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-12 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N99"/>
+  <dimension ref="A1:N111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4356,7 +4356,7 @@
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-11   ·   3 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🔴  2026-08-11   ·   3 trade(s), 3 closed   ·   Gross PnL: ₹-7,481.25   ·   Net PnL: ₹-8,327.08</t>
         </is>
       </c>
       <c r="B94" s="3" t="n"/>
@@ -4446,112 +4446,160 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B96" s="25" t="inlineStr">
+      <c r="A96" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B96" s="9" t="inlineStr">
         <is>
           <t>KOLTEPATIL</t>
         </is>
       </c>
-      <c r="C96" s="25" t="inlineStr">
+      <c r="C96" s="9" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="D96" s="25" t="n"/>
-      <c r="E96" s="26" t="n">
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E96" s="10" t="n">
         <v>145</v>
       </c>
-      <c r="F96" s="27" t="n">
+      <c r="F96" s="11" t="n">
         <v>516.6731</v>
       </c>
-      <c r="G96" s="27" t="n">
+      <c r="G96" s="11" t="n">
         <v>74917.60000000001</v>
       </c>
-      <c r="H96" s="27" t="n">
+      <c r="H96" s="11" t="n">
         <v>23770.29</v>
       </c>
-      <c r="I96" s="27" t="n"/>
-      <c r="J96" s="27" t="n"/>
-      <c r="K96" s="28" t="n"/>
-      <c r="L96" s="27" t="n"/>
-      <c r="M96" s="27" t="n"/>
-      <c r="N96" s="29" t="n"/>
+      <c r="I96" s="11" t="n">
+        <v>493.3248</v>
+      </c>
+      <c r="J96" s="11" t="n">
+        <v>-3385.5</v>
+      </c>
+      <c r="K96" s="12" t="n">
+        <v>-4.519</v>
+      </c>
+      <c r="L96" s="11" t="n">
+        <v>281.33</v>
+      </c>
+      <c r="M96" s="11" t="n">
+        <v>-3666.83</v>
+      </c>
+      <c r="N96" s="13" t="n">
+        <v>-4.8945</v>
+      </c>
     </row>
     <row r="97">
-      <c r="A97" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B97" s="25" t="inlineStr">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B97" s="9" t="inlineStr">
         <is>
           <t>ROLEXRINGS</t>
         </is>
       </c>
-      <c r="C97" s="25" t="inlineStr">
+      <c r="C97" s="9" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="D97" s="25" t="n"/>
-      <c r="E97" s="26" t="n">
+      <c r="D97" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E97" s="10" t="n">
         <v>425</v>
       </c>
-      <c r="F97" s="27" t="n">
+      <c r="F97" s="11" t="n">
         <v>177.4387</v>
       </c>
-      <c r="G97" s="27" t="n">
+      <c r="G97" s="11" t="n">
         <v>75411.45</v>
       </c>
-      <c r="H97" s="27" t="n">
+      <c r="H97" s="11" t="n">
         <v>25411.73</v>
       </c>
-      <c r="I97" s="27" t="n"/>
-      <c r="J97" s="27" t="n"/>
-      <c r="K97" s="28" t="n"/>
-      <c r="L97" s="27" t="n"/>
-      <c r="M97" s="27" t="n"/>
-      <c r="N97" s="29" t="n"/>
+      <c r="I97" s="11" t="n">
+        <v>173.87</v>
+      </c>
+      <c r="J97" s="11" t="n">
+        <v>-1516.7</v>
+      </c>
+      <c r="K97" s="12" t="n">
+        <v>-2.0112</v>
+      </c>
+      <c r="L97" s="11" t="n">
+        <v>283.83</v>
+      </c>
+      <c r="M97" s="11" t="n">
+        <v>-1800.53</v>
+      </c>
+      <c r="N97" s="13" t="n">
+        <v>-2.3876</v>
+      </c>
     </row>
     <row r="98">
-      <c r="A98" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B98" s="25" t="inlineStr">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="inlineStr">
         <is>
           <t>WINDLAS</t>
         </is>
       </c>
-      <c r="C98" s="25" t="inlineStr">
+      <c r="C98" s="9" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="D98" s="25" t="n"/>
-      <c r="E98" s="26" t="n">
+      <c r="D98" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="E98" s="10" t="n">
         <v>79</v>
       </c>
-      <c r="F98" s="27" t="n">
+      <c r="F98" s="11" t="n">
         <v>941.6797</v>
       </c>
-      <c r="G98" s="27" t="n">
+      <c r="G98" s="11" t="n">
         <v>74392.7</v>
       </c>
-      <c r="H98" s="27" t="n">
+      <c r="H98" s="11" t="n">
         <v>24271.68</v>
       </c>
-      <c r="I98" s="27" t="n"/>
-      <c r="J98" s="27" t="n"/>
-      <c r="K98" s="28" t="n"/>
-      <c r="L98" s="27" t="n"/>
-      <c r="M98" s="27" t="n"/>
-      <c r="N98" s="29" t="n"/>
+      <c r="I98" s="11" t="n">
+        <v>909.0335</v>
+      </c>
+      <c r="J98" s="11" t="n">
+        <v>-2579.05</v>
+      </c>
+      <c r="K98" s="12" t="n">
+        <v>-3.4668</v>
+      </c>
+      <c r="L98" s="11" t="n">
+        <v>280.67</v>
+      </c>
+      <c r="M98" s="11" t="n">
+        <v>-2859.72</v>
+      </c>
+      <c r="N98" s="13" t="n">
+        <v>-3.8441</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="20" t="inlineStr">
@@ -4568,17 +4616,421 @@
       <c r="H99" s="21" t="n"/>
       <c r="I99" s="21" t="n"/>
       <c r="J99" s="22" t="n">
-        <v>0</v>
+        <v>-7481.25</v>
       </c>
       <c r="K99" s="21" t="n"/>
       <c r="L99" s="21" t="n"/>
       <c r="M99" s="22" t="n">
+        <v>-8327.08</v>
+      </c>
+      <c r="N99" s="23" t="n"/>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⏳  2026-08-12   ·   8 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="n"/>
+      <c r="C101" s="3" t="n"/>
+      <c r="D101" s="3" t="n"/>
+      <c r="E101" s="3" t="n"/>
+      <c r="F101" s="3" t="n"/>
+      <c r="G101" s="3" t="n"/>
+      <c r="H101" s="3" t="n"/>
+      <c r="I101" s="3" t="n"/>
+      <c r="J101" s="3" t="n"/>
+      <c r="K101" s="3" t="n"/>
+      <c r="L101" s="3" t="n"/>
+      <c r="M101" s="3" t="n"/>
+      <c r="N101" s="4" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>Stock Name</t>
+        </is>
+      </c>
+      <c r="C102" s="6" t="inlineStr">
+        <is>
+          <t>Position entry date</t>
+        </is>
+      </c>
+      <c r="D102" s="6" t="inlineStr">
+        <is>
+          <t>Position Exit date</t>
+        </is>
+      </c>
+      <c r="E102" s="6" t="inlineStr">
+        <is>
+          <t>No of shares</t>
+        </is>
+      </c>
+      <c r="F102" s="6" t="inlineStr">
+        <is>
+          <t>Entry Price</t>
+        </is>
+      </c>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>Capital Deployed</t>
+        </is>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
+        <is>
+          <t>Margin Used</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>Exit Price</t>
+        </is>
+      </c>
+      <c r="J102" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL</t>
+        </is>
+      </c>
+      <c r="K102" s="6" t="inlineStr">
+        <is>
+          <t>Realised PnL Pct</t>
+        </is>
+      </c>
+      <c r="L102" s="6" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="M102" s="6" t="inlineStr">
+        <is>
+          <t>Net PnL</t>
+        </is>
+      </c>
+      <c r="N102" s="7" t="inlineStr">
+        <is>
+          <t>Net PnL Pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B103" s="25" t="inlineStr">
+        <is>
+          <t>DIVGIITTS</t>
+        </is>
+      </c>
+      <c r="C103" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D103" s="25" t="n"/>
+      <c r="E103" s="26" t="n">
+        <v>24</v>
+      </c>
+      <c r="F103" s="27" t="n">
+        <v>1228.55</v>
+      </c>
+      <c r="G103" s="27" t="n">
+        <v>29485.2</v>
+      </c>
+      <c r="H103" s="27" t="n">
+        <v>14763.6</v>
+      </c>
+      <c r="I103" s="27" t="n"/>
+      <c r="J103" s="27" t="n"/>
+      <c r="K103" s="28" t="n"/>
+      <c r="L103" s="27" t="n"/>
+      <c r="M103" s="27" t="n"/>
+      <c r="N103" s="29" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B104" s="25" t="inlineStr">
+        <is>
+          <t>DOLPHIN</t>
+        </is>
+      </c>
+      <c r="C104" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D104" s="25" t="n"/>
+      <c r="E104" s="26" t="n">
+        <v>30</v>
+      </c>
+      <c r="F104" s="27" t="n">
+        <v>499.3</v>
+      </c>
+      <c r="G104" s="27" t="n">
+        <v>14979</v>
+      </c>
+      <c r="H104" s="27" t="n">
+        <v>14979</v>
+      </c>
+      <c r="I104" s="27" t="n"/>
+      <c r="J104" s="27" t="n"/>
+      <c r="K104" s="28" t="n"/>
+      <c r="L104" s="27" t="n"/>
+      <c r="M104" s="27" t="n"/>
+      <c r="N104" s="29" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B105" s="25" t="inlineStr">
+        <is>
+          <t>GIPCL</t>
+        </is>
+      </c>
+      <c r="C105" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D105" s="25" t="n"/>
+      <c r="E105" s="26" t="n">
+        <v>172</v>
+      </c>
+      <c r="F105" s="27" t="n">
+        <v>174.17</v>
+      </c>
+      <c r="G105" s="27" t="n">
+        <v>29957.24</v>
+      </c>
+      <c r="H105" s="27" t="n">
+        <v>9760.639999999999</v>
+      </c>
+      <c r="I105" s="27" t="n"/>
+      <c r="J105" s="27" t="n"/>
+      <c r="K105" s="28" t="n"/>
+      <c r="L105" s="27" t="n"/>
+      <c r="M105" s="27" t="n"/>
+      <c r="N105" s="29" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B106" s="25" t="inlineStr">
+        <is>
+          <t>JINDALPOLY</t>
+        </is>
+      </c>
+      <c r="C106" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D106" s="25" t="n"/>
+      <c r="E106" s="26" t="n">
+        <v>44</v>
+      </c>
+      <c r="F106" s="27" t="n">
+        <v>669.6</v>
+      </c>
+      <c r="G106" s="27" t="n">
+        <v>29462.4</v>
+      </c>
+      <c r="H106" s="27" t="n">
+        <v>14692.7</v>
+      </c>
+      <c r="I106" s="27" t="n"/>
+      <c r="J106" s="27" t="n"/>
+      <c r="K106" s="28" t="n"/>
+      <c r="L106" s="27" t="n"/>
+      <c r="M106" s="27" t="n"/>
+      <c r="N106" s="29" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B107" s="25" t="inlineStr">
+        <is>
+          <t>MANINDS</t>
+        </is>
+      </c>
+      <c r="C107" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D107" s="25" t="n"/>
+      <c r="E107" s="26" t="n">
+        <v>50</v>
+      </c>
+      <c r="F107" s="27" t="n">
+        <v>599.1</v>
+      </c>
+      <c r="G107" s="27" t="n">
+        <v>29955</v>
+      </c>
+      <c r="H107" s="27" t="n">
+        <v>11947.05</v>
+      </c>
+      <c r="I107" s="27" t="n"/>
+      <c r="J107" s="27" t="n"/>
+      <c r="K107" s="28" t="n"/>
+      <c r="L107" s="27" t="n"/>
+      <c r="M107" s="27" t="n"/>
+      <c r="N107" s="29" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B108" s="25" t="inlineStr">
+        <is>
+          <t>ORISSAMINE</t>
+        </is>
+      </c>
+      <c r="C108" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D108" s="25" t="n"/>
+      <c r="E108" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="F108" s="27" t="n">
+        <v>4952</v>
+      </c>
+      <c r="G108" s="27" t="n">
+        <v>29712</v>
+      </c>
+      <c r="H108" s="27" t="n">
+        <v>10398.99</v>
+      </c>
+      <c r="I108" s="27" t="n"/>
+      <c r="J108" s="27" t="n"/>
+      <c r="K108" s="28" t="n"/>
+      <c r="L108" s="27" t="n"/>
+      <c r="M108" s="27" t="n"/>
+      <c r="N108" s="29" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B109" s="25" t="inlineStr">
+        <is>
+          <t>PITTIENG</t>
+        </is>
+      </c>
+      <c r="C109" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D109" s="25" t="n"/>
+      <c r="E109" s="26" t="n">
+        <v>28</v>
+      </c>
+      <c r="F109" s="27" t="n">
+        <v>1047.6</v>
+      </c>
+      <c r="G109" s="27" t="n">
+        <v>29332.8</v>
+      </c>
+      <c r="H109" s="27" t="n">
+        <v>9701.129999999999</v>
+      </c>
+      <c r="I109" s="27" t="n"/>
+      <c r="J109" s="27" t="n"/>
+      <c r="K109" s="28" t="n"/>
+      <c r="L109" s="27" t="n"/>
+      <c r="M109" s="27" t="n"/>
+      <c r="N109" s="29" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="24" t="inlineStr">
+        <is>
+          <t>⏳ OPEN</t>
+        </is>
+      </c>
+      <c r="B110" s="25" t="inlineStr">
+        <is>
+          <t>WSTCSTPAPR</t>
+        </is>
+      </c>
+      <c r="C110" s="25" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="D110" s="25" t="n"/>
+      <c r="E110" s="26" t="n">
+        <v>48</v>
+      </c>
+      <c r="F110" s="27" t="n">
+        <v>619.35</v>
+      </c>
+      <c r="G110" s="27" t="n">
+        <v>29728.8</v>
+      </c>
+      <c r="H110" s="27" t="n">
+        <v>9564.290000000001</v>
+      </c>
+      <c r="I110" s="27" t="n"/>
+      <c r="J110" s="27" t="n"/>
+      <c r="K110" s="28" t="n"/>
+      <c r="L110" s="27" t="n"/>
+      <c r="M110" s="27" t="n"/>
+      <c r="N110" s="29" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="20" t="inlineStr">
+        <is>
+          <t>Σ Day total</t>
+        </is>
+      </c>
+      <c r="B111" s="21" t="n"/>
+      <c r="C111" s="21" t="n"/>
+      <c r="D111" s="21" t="n"/>
+      <c r="E111" s="21" t="n"/>
+      <c r="F111" s="21" t="n"/>
+      <c r="G111" s="21" t="n"/>
+      <c r="H111" s="21" t="n"/>
+      <c r="I111" s="21" t="n"/>
+      <c r="J111" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="N99" s="23" t="n"/>
+      <c r="K111" s="21" t="n"/>
+      <c r="L111" s="21" t="n"/>
+      <c r="M111" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N111" s="23" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A94:N94"/>
     <mergeCell ref="A67:N67"/>
     <mergeCell ref="A3:N3"/>
@@ -4587,6 +5039,7 @@
     <mergeCell ref="A35:N35"/>
     <mergeCell ref="A78:N78"/>
     <mergeCell ref="A30:N30"/>
+    <mergeCell ref="A101:N101"/>
     <mergeCell ref="A86:N86"/>
     <mergeCell ref="A52:N52"/>
     <mergeCell ref="A43:N43"/>
@@ -4809,6 +5262,24 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J103:J110">
+    <cfRule type="dataBar" priority="25">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M103:M110">
+    <cfRule type="dataBar" priority="26">
+      <dataBar showValue="1">
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="0063C384"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Data update — 2026-08-13 candle + results refresh
</commit_message>
<xml_diff>
--- a/results/trade_book.xlsx
+++ b/results/trade_book.xlsx
@@ -20,7 +20,7 @@
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,12 +47,8 @@
     <font>
       <color rgb="00006100"/>
     </font>
-    <font>
-      <i val="1"/>
-      <color rgb="007F6000"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -77,11 +73,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -225,7 +216,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -260,12 +251,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4628,7 +4613,7 @@
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ⏳  2026-08-12   ·   8 trade(s), 0 closed   ·   Gross PnL: ₹0.00   ·   Net PnL: ₹0.00</t>
+          <t xml:space="preserve">  🔴  2026-08-12   ·   8 trade(s), 8 closed   ·   Gross PnL: ₹-607.69   ·   Net PnL: ₹-1,850.58</t>
         </is>
       </c>
       <c r="B101" s="3" t="n"/>
@@ -4718,292 +4703,420 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B103" s="25" t="inlineStr">
+      <c r="A103" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B103" s="9" t="inlineStr">
         <is>
           <t>DIVGIITTS</t>
         </is>
       </c>
-      <c r="C103" s="25" t="inlineStr">
+      <c r="C103" s="9" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D103" s="25" t="n"/>
-      <c r="E103" s="26" t="n">
+      <c r="D103" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E103" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="F103" s="27" t="n">
+      <c r="F103" s="11" t="n">
         <v>1228.55</v>
       </c>
-      <c r="G103" s="27" t="n">
+      <c r="G103" s="11" t="n">
         <v>29485.2</v>
       </c>
-      <c r="H103" s="27" t="n">
+      <c r="H103" s="11" t="n">
         <v>14763.6</v>
       </c>
-      <c r="I103" s="27" t="n"/>
-      <c r="J103" s="27" t="n"/>
-      <c r="K103" s="28" t="n"/>
-      <c r="L103" s="27" t="n"/>
-      <c r="M103" s="27" t="n"/>
-      <c r="N103" s="29" t="n"/>
+      <c r="I103" s="11" t="n">
+        <v>1192</v>
+      </c>
+      <c r="J103" s="11" t="n">
+        <v>-877.2</v>
+      </c>
+      <c r="K103" s="12" t="n">
+        <v>-2.9751</v>
+      </c>
+      <c r="L103" s="11" t="n">
+        <v>168.1</v>
+      </c>
+      <c r="M103" s="11" t="n">
+        <v>-1045.3</v>
+      </c>
+      <c r="N103" s="13" t="n">
+        <v>-3.5452</v>
+      </c>
     </row>
     <row r="104">
-      <c r="A104" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B104" s="25" t="inlineStr">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
         <is>
           <t>DOLPHIN</t>
         </is>
       </c>
-      <c r="C104" s="25" t="inlineStr">
+      <c r="C104" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D104" s="25" t="n"/>
-      <c r="E104" s="26" t="n">
+      <c r="D104" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="F104" s="27" t="n">
+      <c r="F104" s="17" t="n">
         <v>499.3</v>
       </c>
-      <c r="G104" s="27" t="n">
+      <c r="G104" s="17" t="n">
         <v>14979</v>
       </c>
-      <c r="H104" s="27" t="n">
+      <c r="H104" s="17" t="n">
         <v>14979</v>
       </c>
-      <c r="I104" s="27" t="n"/>
-      <c r="J104" s="27" t="n"/>
-      <c r="K104" s="28" t="n"/>
-      <c r="L104" s="27" t="n"/>
-      <c r="M104" s="27" t="n"/>
-      <c r="N104" s="29" t="n"/>
+      <c r="I104" s="17" t="n">
+        <v>510</v>
+      </c>
+      <c r="J104" s="17" t="n">
+        <v>321</v>
+      </c>
+      <c r="K104" s="18" t="n">
+        <v>2.143</v>
+      </c>
+      <c r="L104" s="17" t="n">
+        <v>48.75</v>
+      </c>
+      <c r="M104" s="17" t="n">
+        <v>272.25</v>
+      </c>
+      <c r="N104" s="19" t="n">
+        <v>1.8175</v>
+      </c>
     </row>
     <row r="105">
-      <c r="A105" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B105" s="25" t="inlineStr">
+      <c r="A105" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B105" s="9" t="inlineStr">
         <is>
           <t>GIPCL</t>
         </is>
       </c>
-      <c r="C105" s="25" t="inlineStr">
+      <c r="C105" s="9" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D105" s="25" t="n"/>
-      <c r="E105" s="26" t="n">
+      <c r="D105" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E105" s="10" t="n">
         <v>172</v>
       </c>
-      <c r="F105" s="27" t="n">
+      <c r="F105" s="11" t="n">
         <v>174.17</v>
       </c>
-      <c r="G105" s="27" t="n">
+      <c r="G105" s="11" t="n">
         <v>29957.24</v>
       </c>
-      <c r="H105" s="27" t="n">
+      <c r="H105" s="11" t="n">
         <v>9760.639999999999</v>
       </c>
-      <c r="I105" s="27" t="n"/>
-      <c r="J105" s="27" t="n"/>
-      <c r="K105" s="28" t="n"/>
-      <c r="L105" s="27" t="n"/>
-      <c r="M105" s="27" t="n"/>
-      <c r="N105" s="29" t="n"/>
+      <c r="I105" s="11" t="n">
+        <v>174.05</v>
+      </c>
+      <c r="J105" s="11" t="n">
+        <v>-20.64</v>
+      </c>
+      <c r="K105" s="12" t="n">
+        <v>-0.0689</v>
+      </c>
+      <c r="L105" s="11" t="n">
+        <v>172.15</v>
+      </c>
+      <c r="M105" s="11" t="n">
+        <v>-192.79</v>
+      </c>
+      <c r="N105" s="13" t="n">
+        <v>-0.6435999999999999</v>
+      </c>
     </row>
     <row r="106">
-      <c r="A106" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B106" s="25" t="inlineStr">
+      <c r="A106" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B106" s="9" t="inlineStr">
         <is>
           <t>JINDALPOLY</t>
         </is>
       </c>
-      <c r="C106" s="25" t="inlineStr">
+      <c r="C106" s="9" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D106" s="25" t="n"/>
-      <c r="E106" s="26" t="n">
+      <c r="D106" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E106" s="10" t="n">
         <v>44</v>
       </c>
-      <c r="F106" s="27" t="n">
+      <c r="F106" s="11" t="n">
         <v>669.6</v>
       </c>
-      <c r="G106" s="27" t="n">
+      <c r="G106" s="11" t="n">
         <v>29462.4</v>
       </c>
-      <c r="H106" s="27" t="n">
+      <c r="H106" s="11" t="n">
         <v>14692.7</v>
       </c>
-      <c r="I106" s="27" t="n"/>
-      <c r="J106" s="27" t="n"/>
-      <c r="K106" s="28" t="n"/>
-      <c r="L106" s="27" t="n"/>
-      <c r="M106" s="27" t="n"/>
-      <c r="N106" s="29" t="n"/>
+      <c r="I106" s="11" t="n">
+        <v>656.6909000000001</v>
+      </c>
+      <c r="J106" s="11" t="n">
+        <v>-568</v>
+      </c>
+      <c r="K106" s="12" t="n">
+        <v>-1.9279</v>
+      </c>
+      <c r="L106" s="11" t="n">
+        <v>168.39</v>
+      </c>
+      <c r="M106" s="11" t="n">
+        <v>-736.39</v>
+      </c>
+      <c r="N106" s="13" t="n">
+        <v>-2.4994</v>
+      </c>
     </row>
     <row r="107">
-      <c r="A107" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B107" s="25" t="inlineStr">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B107" s="9" t="inlineStr">
         <is>
           <t>MANINDS</t>
         </is>
       </c>
-      <c r="C107" s="25" t="inlineStr">
+      <c r="C107" s="9" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D107" s="25" t="n"/>
-      <c r="E107" s="26" t="n">
+      <c r="D107" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E107" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="F107" s="27" t="n">
+      <c r="F107" s="11" t="n">
         <v>599.1</v>
       </c>
-      <c r="G107" s="27" t="n">
+      <c r="G107" s="11" t="n">
         <v>29955</v>
       </c>
-      <c r="H107" s="27" t="n">
+      <c r="H107" s="11" t="n">
         <v>11947.05</v>
       </c>
-      <c r="I107" s="27" t="n"/>
-      <c r="J107" s="27" t="n"/>
-      <c r="K107" s="28" t="n"/>
-      <c r="L107" s="27" t="n"/>
-      <c r="M107" s="27" t="n"/>
-      <c r="N107" s="29" t="n"/>
+      <c r="I107" s="11" t="n">
+        <v>589.6</v>
+      </c>
+      <c r="J107" s="11" t="n">
+        <v>-475</v>
+      </c>
+      <c r="K107" s="12" t="n">
+        <v>-1.5857</v>
+      </c>
+      <c r="L107" s="11" t="n">
+        <v>170.8</v>
+      </c>
+      <c r="M107" s="11" t="n">
+        <v>-645.8</v>
+      </c>
+      <c r="N107" s="13" t="n">
+        <v>-2.1559</v>
+      </c>
     </row>
     <row r="108">
-      <c r="A108" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B108" s="25" t="inlineStr">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
         <is>
           <t>ORISSAMINE</t>
         </is>
       </c>
-      <c r="C108" s="25" t="inlineStr">
+      <c r="C108" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D108" s="25" t="n"/>
-      <c r="E108" s="26" t="n">
+      <c r="D108" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="F108" s="27" t="n">
+      <c r="F108" s="17" t="n">
         <v>4952</v>
       </c>
-      <c r="G108" s="27" t="n">
+      <c r="G108" s="17" t="n">
         <v>29712</v>
       </c>
-      <c r="H108" s="27" t="n">
+      <c r="H108" s="17" t="n">
         <v>10398.99</v>
       </c>
-      <c r="I108" s="27" t="n"/>
-      <c r="J108" s="27" t="n"/>
-      <c r="K108" s="28" t="n"/>
-      <c r="L108" s="27" t="n"/>
-      <c r="M108" s="27" t="n"/>
-      <c r="N108" s="29" t="n"/>
+      <c r="I108" s="17" t="n">
+        <v>5063.8167</v>
+      </c>
+      <c r="J108" s="17" t="n">
+        <v>670.9</v>
+      </c>
+      <c r="K108" s="18" t="n">
+        <v>2.258</v>
+      </c>
+      <c r="L108" s="17" t="n">
+        <v>172.01</v>
+      </c>
+      <c r="M108" s="17" t="n">
+        <v>498.89</v>
+      </c>
+      <c r="N108" s="19" t="n">
+        <v>1.6791</v>
+      </c>
     </row>
     <row r="109">
-      <c r="A109" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B109" s="25" t="inlineStr">
+      <c r="A109" s="14" t="inlineStr">
+        <is>
+          <t>🟢 WIN</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="inlineStr">
         <is>
           <t>PITTIENG</t>
         </is>
       </c>
-      <c r="C109" s="25" t="inlineStr">
+      <c r="C109" s="15" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D109" s="25" t="n"/>
-      <c r="E109" s="26" t="n">
+      <c r="D109" s="15" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E109" s="16" t="n">
         <v>28</v>
       </c>
-      <c r="F109" s="27" t="n">
+      <c r="F109" s="17" t="n">
         <v>1047.6</v>
       </c>
-      <c r="G109" s="27" t="n">
+      <c r="G109" s="17" t="n">
         <v>29332.8</v>
       </c>
-      <c r="H109" s="27" t="n">
+      <c r="H109" s="17" t="n">
         <v>9701.129999999999</v>
       </c>
-      <c r="I109" s="27" t="n"/>
-      <c r="J109" s="27" t="n"/>
-      <c r="K109" s="28" t="n"/>
-      <c r="L109" s="27" t="n"/>
-      <c r="M109" s="27" t="n"/>
-      <c r="N109" s="29" t="n"/>
+      <c r="I109" s="17" t="n">
+        <v>1066.2554</v>
+      </c>
+      <c r="J109" s="17" t="n">
+        <v>522.35</v>
+      </c>
+      <c r="K109" s="18" t="n">
+        <v>1.7808</v>
+      </c>
+      <c r="L109" s="17" t="n">
+        <v>171.19</v>
+      </c>
+      <c r="M109" s="17" t="n">
+        <v>351.16</v>
+      </c>
+      <c r="N109" s="19" t="n">
+        <v>1.1972</v>
+      </c>
     </row>
     <row r="110">
-      <c r="A110" s="24" t="inlineStr">
-        <is>
-          <t>⏳ OPEN</t>
-        </is>
-      </c>
-      <c r="B110" s="25" t="inlineStr">
+      <c r="A110" s="8" t="inlineStr">
+        <is>
+          <t>🔴 LOSS</t>
+        </is>
+      </c>
+      <c r="B110" s="9" t="inlineStr">
         <is>
           <t>WSTCSTPAPR</t>
         </is>
       </c>
-      <c r="C110" s="25" t="inlineStr">
+      <c r="C110" s="9" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="D110" s="25" t="n"/>
-      <c r="E110" s="26" t="n">
+      <c r="D110" s="9" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="E110" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="F110" s="27" t="n">
+      <c r="F110" s="11" t="n">
         <v>619.35</v>
       </c>
-      <c r="G110" s="27" t="n">
+      <c r="G110" s="11" t="n">
         <v>29728.8</v>
       </c>
-      <c r="H110" s="27" t="n">
+      <c r="H110" s="11" t="n">
         <v>9564.290000000001</v>
       </c>
-      <c r="I110" s="27" t="n"/>
-      <c r="J110" s="27" t="n"/>
-      <c r="K110" s="28" t="n"/>
-      <c r="L110" s="27" t="n"/>
-      <c r="M110" s="27" t="n"/>
-      <c r="N110" s="29" t="n"/>
+      <c r="I110" s="11" t="n">
+        <v>615.5771</v>
+      </c>
+      <c r="J110" s="11" t="n">
+        <v>-181.1</v>
+      </c>
+      <c r="K110" s="12" t="n">
+        <v>-0.6092</v>
+      </c>
+      <c r="L110" s="11" t="n">
+        <v>171.5</v>
+      </c>
+      <c r="M110" s="11" t="n">
+        <v>-352.6</v>
+      </c>
+      <c r="N110" s="13" t="n">
+        <v>-1.1861</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="20" t="inlineStr">
@@ -5020,12 +5133,12 @@
       <c r="H111" s="21" t="n"/>
       <c r="I111" s="21" t="n"/>
       <c r="J111" s="22" t="n">
-        <v>0</v>
+        <v>-607.6900000000001</v>
       </c>
       <c r="K111" s="21" t="n"/>
       <c r="L111" s="21" t="n"/>
       <c r="M111" s="22" t="n">
-        <v>0</v>
+        <v>-1850.58</v>
       </c>
       <c r="N111" s="23" t="n"/>
     </row>

</xml_diff>